<commit_message>
Add 변시3 OX (1216 items)
</commit_message>
<xml_diff>
--- a/assets/ox_civil_bar14.xlsx
+++ b/assets/ox_civil_bar14.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1144"/>
+  <dimension ref="A1:H1217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -46224,6 +46224,2926 @@
         </is>
       </c>
     </row>
+    <row r="1145">
+      <c r="A1145" t="n">
+        <v>301</v>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>매매계약이 합의해제된 경우 매도인의 원상회복청구권은 소유권에 기한 물권적 청구권이므로, 소멸시효의 대상이 되지 아니한다.</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>시효대상</t>
+        </is>
+      </c>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>판례는 합의해제 시 소유권이 매도인에게 복귀하므로 원상회복청구권이 물권적 청구권이어서 소멸시효에 걸리지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>대판 1982.7.27. 80다2968</t>
+        </is>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>제213조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="n">
+        <v>302</v>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>송전선이 토지 위를 통과하고 있다는 점을 알고서 토지를 취득한 경우, 그 취득자는 소유권 행사가 제한된 상태를 용인한 것이므로 송전선 철거 청구는 신의칙에 반한다.</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>신의칙</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>판례는 방해 사실을 알고 취득하였다는 점만으로 소유권 행사 제한을 용인한 것이 아니므로 철거 청구가 신의칙에 반하지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>대판 1995.8.25. 94다27069</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>제2조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="n">
+        <v>303</v>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>실효의 원칙을 적용함에 있어 종전 토지 소유자가 자신의 권리를 행사하지 않았다는 사정은, 그 토지의 소유권을 적법하게 취득한 새로운 권리자에게 실효의 원칙을 적용할 때 고려할 사정이 아니다.</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>실효</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>판례는 전 소유자의 권리 불행사 사정이 새 권리자에 대한 실효 원칙 적용에서 고려되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>대판 1995.8.25. 94다27069</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>제2조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="n">
+        <v>304</v>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>권리행사가 권리남용이 되려면 객관적으로 권리행사가 사회질서에 위반되고, 주관적으로 권리행사의 목적이 오직 상대방에게 고통을 주고 손해를 입히려는 데 있을 뿐 권리자에게 아무런 이익이 없어야 하며, 그 주관적 요건은 객관적 사정에 의하여 추인할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>남용요건</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>판례는 권리남용의 객관적·주관적 요건을 제시하고 주관적 요건의 객관적 추인을 인정한다.</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>대판 2003.2.14. 2002다62319</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>제2조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="n">
+        <v>305</v>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>통정허위표시에 기한 채무를 보증하고 그 보증채무를 이행한 보증인은, 민법 제108조 제2항의 보호되는 제3자에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>제3자범위</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>판례는 허위표시에 기초하여 구상권 취득의 이해관계를 가지게 된 보증인을 제3자로 본다.</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>대판 2000.7.6. 99다51258</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>제108조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="n">
+        <v>306</v>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>통정허위표시인 채권양도계약에서 양수인에게 아직 채무를 변제하지 않은 채무자는, 그 허위표시의 무효로 대항받지 않는 선의의 제3자에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>제3자범위</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>판례는 양도계약이 허위표시임이 밝혀진 이상 미변제 채무자는 선의의 제3자임을 내세워 진정한 채권자에게 지급을 거절할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>대판 1983.1.18. 82다594</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>제108조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="n">
+        <v>307</v>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>가장소비대차계약에 기해 발생한 가장채권을 양수한 한국자산관리공사는, 민법 제108조 제2항의 제3자에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>제3자범위</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>판례는 부실채권을 유상으로 인수하며 새로운 이해관계를 맺은 자산관리공사를 허위표시의 제3자로 본다.</t>
+        </is>
+      </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>대판 2004.1.15. 2002다31537</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>제108조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="n">
+        <v>308</v>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>법인 대표자의 업무에 관한 포괄적 위임과 그에 따른 수임인의 대행행위는 민법 제62조에 위반되어 법인에 대하여 효력이 없다.</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>복임제한</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>판례는 대표자가 특정행위만 대리하게 할 수 있을 뿐 업무를 포괄적으로 위임할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>민법 제62조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>제62조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="n">
+        <v>309</v>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>법인의 불법행위책임에 관한 민법 제35조의 '대표자'에는 명칭이나 등기 여부를 불문하고 당해 법인을 실질적으로 운영하면서 법인을 사실상 대표하여 사무를 집행하는 사람도 포함된다.</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>대표자범위</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>판례는 제35조의 대표자에 등기 여부와 무관하게 사실상 대표자도 포함되며 이는 비법인사단에도 적용된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>대판 2011.4.28. 2008다15438</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>제35조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="n">
+        <v>310</v>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>법인 대표자의 행위가 외형상 직무행위로 인정되는 것이라면, 그것이 대표자 개인의 사리를 도모하기 위한 것이거나 법령에 위배된 것이라도 제35조의 직무에 관한 행위에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>외형이론</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>판례는 직무관련성을 외형이론에 따라 판단한다.</t>
+        </is>
+      </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>대판 2004.2.27. 2003다15280</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>제35조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="n">
+        <v>311</v>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>법인 대표자의 행위가 직무에 관한 행위에 해당하지 아니함을 피해자 자신이 알았거나 중대한 과실로 알지 못한 경우에는, 법인에게 손해배상책임을 물을 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>악의중과실</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>판례는 외형이론에도 불구하고 피해자의 악의·중과실이 있으면 법인의 불법행위책임이 부정된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>대판 2004.3.26. 2003다34045</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>제35조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="n">
+        <v>312</v>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>법정대리인이 미성년자에게 어떠한 재산에 대한 처분을 허락하였더라도, 법정대리인의 그 재산에 대한 처분 대리권은 소멸하지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>대리권존속</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>판례·통설은 처분 허락으로 미성년자에게 행위능력이 생기는 것이 아니므로 법정대리인의 처분 대리권이 소멸하지 않고 병존한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>민법 제6조 · 통설</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>제6조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="n">
+        <v>313</v>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>미성년자가 법정대리인으로부터 허락을 얻은 특정한 영업에 관하여는 성년자와 동일한 행위능력이 있으므로, 그 영업에 관하여는 법정대리인의 동의권과 대리권이 모두 소멸한다.</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>영업허락</t>
+        </is>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>통설은 제8조 제1항의 영업허락 시 그 영업에 관한 법정대리인의 동의권·대리권이 소멸한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr">
+        <is>
+          <t>민법 제8조 · 통설</t>
+        </is>
+      </c>
+      <c r="H1157" t="inlineStr">
+        <is>
+          <t>제8조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="n">
+        <v>314</v>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>미성년후견인은 한 명으로 하여야 하지만, 성년후견인은 여러 명을 둘 수 있고 법인도 성년후견인이 될 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>수와자격</t>
+        </is>
+      </c>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>민법 제930조의 명문 규정이다.</t>
+        </is>
+      </c>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>민법 제930조</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>제930조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="n">
+        <v>315</v>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>후견인과 피후견인 사이에 이해상반행위가 있는 경우 특별대리인을 선임하여야 하지만, 후견감독인이 있는 경우에는 특별대리인을 선임할 필요가 없다.</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>이해상반</t>
+        </is>
+      </c>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>민법 제949조의3은 후견감독인이 있는 경우 그가 피후견인을 대리하므로 특별대리인 선임이 필요 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>민법 제949조의3</t>
+        </is>
+      </c>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>제949조의3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="n">
+        <v>316</v>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>피성년후견인의 법률행위는 성년후견인의 동의가 있었더라도 취소할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>취소가부</t>
+        </is>
+      </c>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>민법 제10조상 피성년후견인의 법률행위는 동의 유무와 관계없이 취소할 수 있다(일용품 구입 등 예외 제외).</t>
+        </is>
+      </c>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>민법 제10조</t>
+        </is>
+      </c>
+      <c r="H1160" t="inlineStr">
+        <is>
+          <t>제10조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="n">
+        <v>317</v>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>본인이 무권대리인에게 무권대리행위를 추인한 경우, 상대방이 그 추인 사실을 알지 못하는 동안에는 상대방은 여전히 철회를 할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>추인상대방</t>
+        </is>
+      </c>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>판례는 제132조상 무권대리인에 대한 추인은 상대방이 알지 못하는 동안에는 상대방에게 대항하지 못하므로 상대방이 철회할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>대판 1981.4.14. 80다2314</t>
+        </is>
+      </c>
+      <c r="H1161" t="inlineStr">
+        <is>
+          <t>제132조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="n">
+        <v>318</v>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>피보험자의 서면 동의를 결여한 타인의 생명보험계약은 강행규정 위반으로 확정적 무효이므로, 사후에 동의가 있더라도 추인에 의하여 유효로 될 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>강행규정</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>판례는 상법 제731조 위반의 타인 생명보험계약을 확정적 무효로 보아 추인을 부정한다.</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>대판 2006.9.22. 2004다56677</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>제139조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="n">
+        <v>319</v>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>무효인 소송행위를 추인하는 경우에는 추인의 소급효를 제한하는 민법 제133조 단서가 적용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>소송행위추인</t>
+        </is>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>판례는 소송행위 추인에는 제133조 단서(제3자 권리 보호)가 적용되지 않고 전체적으로 소급하여 유효하게 된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>대판 1997.3.14. 96다25227</t>
+        </is>
+      </c>
+      <c r="H1163" t="inlineStr">
+        <is>
+          <t>제133조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="n">
+        <v>320</v>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>재단법인 설립을 위하여 출연한 재산이 지명채권인 경우, 견해 대립 없이 법인이 성립한 때에 법인에게 귀속된다.</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>귀속시기</t>
+        </is>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>판례·통설은 지명채권은 별도의 공시방법이 필요 없어 제48조에 따라 법인 성립 시 귀속된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>민법 제48조</t>
+        </is>
+      </c>
+      <c r="H1164" t="inlineStr">
+        <is>
+          <t>제48조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="n">
+        <v>321</v>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>생전처분으로 재단법인을 설립하는 경우, 출연재산이 부동산인 때에는 출연자와 법인 사이의 관계에서는 법인 성립 외에 등기를 필요로 하지 않으나, 제3자에 대한 관계에서는 등기를 갖추어야 법인에게 귀속된다.</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>절충설</t>
+        </is>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>판례(절충설)는 출연자-법인 사이에서는 법인 성립 시 귀속하지만 제3자에 대한 관계에서는 등기를 갖추어야 한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>대판 1979.12.11. 78다481 전합 · 대판 1993.9.14. 93다8054</t>
+        </is>
+      </c>
+      <c r="H1165" t="inlineStr">
+        <is>
+          <t>제48조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="n">
+        <v>322</v>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>친양자를 입양하려는 사람은 원칙적으로 3년 이상 혼인 중인 부부로서 공동으로 입양하여야 하지만, 1년 이상 혼인 중인 부부의 한쪽이 그 배우자의 친생자를 친양자로 하는 경우에는 그러하지 아니하다.</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>입양요건</t>
+        </is>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>민법 제908조의2 제1항 제1호의 명문 규정이다.</t>
+        </is>
+      </c>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>민법 제908조의2</t>
+        </is>
+      </c>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>제908조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="n">
+        <v>323</v>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>친양자가 될 사람은 미성년자여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>입양요건</t>
+        </is>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>민법 제908조의2 제1항 제2호의 명문 규정이다.</t>
+        </is>
+      </c>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>민법 제908조의2</t>
+        </is>
+      </c>
+      <c r="H1167" t="inlineStr">
+        <is>
+          <t>제908조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="n">
+        <v>324</v>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>친양자 입양에서도 일반입양과 마찬가지로 일정한 사유가 있는 때에는 가정법원은 친생부모의 동의가 없어도 친양자 입양을 허가하는 심판을 할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>동의예외</t>
+        </is>
+      </c>
+      <c r="F1168" t="inlineStr">
+        <is>
+          <t>민법 제908조의2 제2항은 법정대리인의 부당한 동의·승낙 거부, 친생부모의 부양·면접교섭 불이행, 학대·유기 등의 경우 동의 없이도 인용할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>민법 제908조의2②</t>
+        </is>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>제908조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="n">
+        <v>325</v>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>친양자 입양의 취소는 소급효가 없다.</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>취소효과</t>
+        </is>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>민법 제908조의7은 친양자 입양 취소·파양의 효력이 소급하지 않고 장래에 향하여만 발생한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>민법 제908조의7</t>
+        </is>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>제908조의7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="n">
+        <v>326</v>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>혼인 중 부부 일방이 사망하여 상대방이 배우자로서 상속받은 후 그 혼인이 취소되었더라도, 혼인취소는 소급효가 없으므로 그 전에 이루어진 상속관계가 소급하여 무효가 되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>소급효</t>
+        </is>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>판례는 민법 제824조상 혼인취소의 소급효가 없으므로 상속이 유효하게 유지된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>대판 1996.12.23. 95다48308</t>
+        </is>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>제824조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="n">
+        <v>327</v>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>인지청구의 소에 의하여 상속인이 된 자가 상속회복청구를 하는 경우, 제척기간의 기산점이 되는 '상속권 침해를 안 날'은 인지심판 확정일이다.</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>기산점</t>
+        </is>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>판례는 사후 인지된 자의 상속회복청구권 제척기간 기산점을 인지심판 확정일로 본다.</t>
+        </is>
+      </c>
+      <c r="G1171" t="inlineStr">
+        <is>
+          <t>대판 2007.10.25. 2007다36223</t>
+        </is>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>제999조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="n">
+        <v>328</v>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>대습상속에서 피대습자는 피상속인의 직계비속 또는 형제자매에 한정되므로, 피상속인의 배우자는 피대습자가 될 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>피대습자</t>
+        </is>
+      </c>
+      <c r="F1172" t="inlineStr">
+        <is>
+          <t>민법 제1001조는 직계비속·형제자매를 피대습자로 정하므로 배우자는 피대습자가 될 수 없다(다만 배우자는 대습상속인은 될 수 있음).</t>
+        </is>
+      </c>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>민법 제1001조</t>
+        </is>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>제1001조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="n">
+        <v>329</v>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>상속포기는 대습상속의 원인이 된다.</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>대습원인</t>
+        </is>
+      </c>
+      <c r="F1173" t="inlineStr">
+        <is>
+          <t>민법 제1001조의 대습상속 원인은 상속인의 사망 또는 결격이고, 상속포기는 대습상속의 원인이 아니다.</t>
+        </is>
+      </c>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>민법 제1001조</t>
+        </is>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>제1001조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="n">
+        <v>330</v>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>근저당권 설정 후 경매로 인한 압류의 효력이 발생하기 전에 취득한 유치권으로는 경매절차의 매수인에게 대항할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>대항시점</t>
+        </is>
+      </c>
+      <c r="F1174" t="inlineStr">
+        <is>
+          <t>판례는 압류 전 취득한 유치권은 선행 근저당권이 있어도 매수인에게 대항할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>대판 2009.1.15. 2008다70763</t>
+        </is>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>제320조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="n">
+        <v>331</v>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>부동산 매도인이 매매대금을 다 지급받지 않은 상태에서 매수인에게 소유권이전등기를 마쳐주고 부동산을 계속 점유하는 경우, 매매대금채권을 피담보채권으로 하여 그 부동산의 소유권을 취득한 제3자에게 유치권을 주장할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>견련성</t>
+        </is>
+      </c>
+      <c r="F1175" t="inlineStr">
+        <is>
+          <t>판례는 매매대금채권은 매매목적물에 관하여 생긴 채권이 아니어서 견련성이 없으므로 유치권이 성립하지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>대판 2012.1.12. 2011마2380</t>
+        </is>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>제320조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="n">
+        <v>332</v>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>저당부동산의 제3취득자가 저당권의 피담보채무를 변제하고 저당권의 소멸을 청구하는 것은, 경매신청이 있은 후라도 그 매각이 종료되기 전까지는 허용된다.</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>변제시기</t>
+        </is>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>통설은 제3취득자의 변제가 경매신청 전후를 불문하고 매각 종료 전까지 허용된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1176" t="inlineStr">
+        <is>
+          <t>민법 제364조 · 통설</t>
+        </is>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>제364조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="n">
+        <v>333</v>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>후순위 저당권자는 민법 제364조의 제3취득자에 해당하여 저당권 소멸을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>제3취득자</t>
+        </is>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>판례는 후순위 저당권자는 제364조의 '소유권·지상권·전세권을 취득한 제3취득자'에 해당하지 않으므로 저당권 소멸청구를 할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>대판 2006.1.26. 2005다17341</t>
+        </is>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>제364조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="n">
+        <v>334</v>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>공동저당의 목적인 채무자 소유 부동산과 물상보증인 소유 부동산을 동시에 경매하여 배당하는 경우, 민법 제368조 제1항이 적용되어 각 부동산 경매대가에 비례하여 채권 분담을 정한다.</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>동시배당</t>
+        </is>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>판례는 이 경우 물상보증인의 변제자대위 보호를 위해 제368조 제1항이 적용되지 않고 채무자 소유 부동산에서 우선 배당한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>대판 2010.4.15. 2008다41475</t>
+        </is>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>제368조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="n">
+        <v>335</v>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>공동저당에서 '각 부동산의 경매대가'란 매각대금에서 당해 부동산이 부담할 경매비용과 선순위채권을 공제한 잔액을 의미한다.</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>경매대가</t>
+        </is>
+      </c>
+      <c r="F1179" t="inlineStr">
+        <is>
+          <t>판례는 제368조 제1항의 경매대가를 경매비용·선순위채권 공제 후의 잔액으로 본다.</t>
+        </is>
+      </c>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>대판 2003.9.5. 2001다66291</t>
+        </is>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>제368조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="n">
+        <v>336</v>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>가등기가 경료된 부동산에 점유취득시효가 완성된 후 그 가등기에 기한 본등기가 경료된 경우, 시효완성 후의 취득자인지 여부는 본등기 시를 기준으로 판단한다.</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>기준시점</t>
+        </is>
+      </c>
+      <c r="F1180" t="inlineStr">
+        <is>
+          <t>판례는 가등기는 순위보전 효력만 있고 본등기 시 물권변동 효력이 발생하므로 시효완성 후 취득자 판단을 본등기 시 기준으로 한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>대판 1992.9.25. 92다21258</t>
+        </is>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>제245조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="n">
+        <v>337</v>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>토지의 점유자가 소유자를 상대로 매매를 원인으로 한 소유권이전등기청구소송을 제기하였다가 패소하고 그 판결이 확정되었다는 사정만으로는, 그 점유가 자주점유에서 타주점유로 전환되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>점유전환</t>
+        </is>
+      </c>
+      <c r="F1181" t="inlineStr">
+        <is>
+          <t>판례는 이전등기청구 패소 확정만으로는 자주점유 추정이 번복되어 타주점유로 전환되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>대판 2009.12.10. 2006다19177</t>
+        </is>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>제197조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="n">
+        <v>338</v>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>취득시효가 완성된 후 소유권이전등기의무가 이행불능이 된 경우, 시효취득자는 부동산 소유자에 대하여 채무불이행을 원인으로 한 손해배상을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>손해배상</t>
+        </is>
+      </c>
+      <c r="F1182" t="inlineStr">
+        <is>
+          <t>판례는 부동산 소유자와 시효취득자 사이에 계약상 채권채무관계가 성립하는 것이 아니므로 채무불이행을 원인으로 한 손해배상을 청구할 수 없다고 한다(불법행위 책임은 별론).</t>
+        </is>
+      </c>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>대판 1995.7.11. 94다4509</t>
+        </is>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>제245조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="n">
+        <v>339</v>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>악의의 점유자는 수취한 과실을 반환하여야 하며, 소비하였거나 과실로 인하여 훼손 또는 수취하지 못한 경우에는 그 과실의 대가를 보상하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1183" t="inlineStr">
+        <is>
+          <t>과실반환</t>
+        </is>
+      </c>
+      <c r="F1183" t="inlineStr">
+        <is>
+          <t>민법 제201조 제2항의 명문 규정이다.</t>
+        </is>
+      </c>
+      <c r="G1183" t="inlineStr">
+        <is>
+          <t>민법 제201조②</t>
+        </is>
+      </c>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>제201조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="n">
+        <v>340</v>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>점유물이 점유자의 책임 있는 사유로 멸실·훼손된 경우, 소유의 의사가 없는 점유자는 선의인 경우에도 손해의 전부를 배상하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1184" t="inlineStr">
+        <is>
+          <t>배상범위</t>
+        </is>
+      </c>
+      <c r="F1184" t="inlineStr">
+        <is>
+          <t>민법 제202조의 명문 규정으로, 타주점유자는 선의라도 전부 배상한다.</t>
+        </is>
+      </c>
+      <c r="G1184" t="inlineStr">
+        <is>
+          <t>민법 제202조</t>
+        </is>
+      </c>
+      <c r="H1184" t="inlineStr">
+        <is>
+          <t>제202조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="n">
+        <v>341</v>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>점유자가 점유물을 보존하기 위하여 지출한 필요비의 상환을 청구할 수 있으나, 점유자가 과실을 취득한 경우에는 통상의 필요비는 청구하지 못한다.</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1185" t="inlineStr">
+        <is>
+          <t>상환제한</t>
+        </is>
+      </c>
+      <c r="F1185" t="inlineStr">
+        <is>
+          <t>민법 제203조 제1항 단서의 명문 규정이다.</t>
+        </is>
+      </c>
+      <c r="G1185" t="inlineStr">
+        <is>
+          <t>민법 제203조①</t>
+        </is>
+      </c>
+      <c r="H1185" t="inlineStr">
+        <is>
+          <t>제203조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="n">
+        <v>342</v>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>공유토지의 1/2 지분권자가 다른 공유자와 협의 없이 단독으로 토지 전부를 제3자에게 임대한 경우, 다른 소수지분권자는 공유물의 보존행위로서 임차인에 대하여 토지 전부의 인도를 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1186" t="inlineStr">
+        <is>
+          <t>보존행위</t>
+        </is>
+      </c>
+      <c r="F1186" t="inlineStr">
+        <is>
+          <t>판례(전합)는 소수지분권자가 보존행위로서 인도를 청구할 수 없고 자신의 지분권에 기초하여 방해 상태 제거나 방해행위 금지를 청구할 수 있을 뿐이라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>대판 2020.5.21. 2018다287522 전합</t>
+        </is>
+      </c>
+      <c r="H1186" t="inlineStr">
+        <is>
+          <t>제265조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="n">
+        <v>343</v>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>부동산 공유자 중 1인은 자신의 공유지분이 아닌 다른 공유자의 공유지분을 침해하는 제3자 명의의 원인무효 등기에 대하여, 공유물의 보존행위로서 그 부분 등기의 말소를 구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1187" t="inlineStr">
+        <is>
+          <t>보존행위</t>
+        </is>
+      </c>
+      <c r="F1187" t="inlineStr">
+        <is>
+          <t>판례는 다른 공유자의 지분을 침해하는 등기의 말소는 그 지분권자가 구할 수 있을 뿐 보존행위로 구할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>대판 1994.11.11. 94다35008</t>
+        </is>
+      </c>
+      <c r="H1187" t="inlineStr">
+        <is>
+          <t>제265조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="n">
+        <v>344</v>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>채무자가 횡령한 금전을 채권자에 대한 채무변제에 사용한 경우, 채권자가 그 금전이 횡령된 것임에 대하여 단순한 과실이 있는 경우에는 피해자가 채권자에게 부당이득반환을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1188" t="inlineStr">
+        <is>
+          <t>악의중과실</t>
+        </is>
+      </c>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>판례는 채권자에게 악의 또는 중대한 과실이 없는 한 그 변제 수령에 법률상 원인이 있어 부당이득이 되지 않으므로, 단순 과실만으로는 부당이득반환을 청구할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1188" t="inlineStr">
+        <is>
+          <t>대판 2008.3.13. 2006다53733</t>
+        </is>
+      </c>
+      <c r="H1188" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="n">
+        <v>345</v>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>취득시효 완성 후 등기명의인이 설정한 저당권의 피담보채무를 시효완성자가 변제한 경우, 시효완성자는 원소유자에게 대위변제를 이유로 구상권을 행사하거나 부당이득반환을 청구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1189" t="inlineStr">
+        <is>
+          <t>용인부담</t>
+        </is>
+      </c>
+      <c r="F1189" t="inlineStr">
+        <is>
+          <t>판례는 그 변제가 시효취득자가 용인해야 할 부담을 제거하여 완전한 소유권을 확보하기 위한 자기 이익을 위한 행위이므로 구상권·부당이득반환청구를 할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1189" t="inlineStr">
+        <is>
+          <t>대판 2006.5.12. 2005다75910</t>
+        </is>
+      </c>
+      <c r="H1189" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="n">
+        <v>346</v>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>토지에 대하여 가압류가 집행된 후 그 토지가 수용되어 가압류의 효력이 소멸한 경우, 토지소유자가 받은 보상금은 법률상 원인이 없는 부당이득에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1190" t="inlineStr">
+        <is>
+          <t>법률상원인</t>
+        </is>
+      </c>
+      <c r="F1190" t="inlineStr">
+        <is>
+          <t>판례는 토지소유자가 받은 수용보상금은 법률상 원인이 있으므로 부당이득이 아니라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1190" t="inlineStr">
+        <is>
+          <t>대판 2009.9.10. 2006다61536</t>
+        </is>
+      </c>
+      <c r="H1190" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="n">
+        <v>347</v>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>법인의 대표자가 법인에게 불법행위를 한 경우 그 손해배상청구권의 단기소멸시효는, 법인의 이익을 정당하게 보전할 권한을 가진 다른 임원·사원·직원 등이 손해배상청구권을 행사할 수 있을 정도로 이를 안 때부터 진행한다.</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1191" t="inlineStr">
+        <is>
+          <t>기산점</t>
+        </is>
+      </c>
+      <c r="F1191" t="inlineStr">
+        <is>
+          <t>판례는 대표자가 가해자인 경우 그 대표자의 인식이 아니라 법인의 이익을 보전할 다른 자의 인식을 기준으로 시효 기산점을 정한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1191" t="inlineStr">
+        <is>
+          <t>대판 2002.6.14. 2002다11441</t>
+        </is>
+      </c>
+      <c r="H1191" t="inlineStr">
+        <is>
+          <t>제766조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="n">
+        <v>348</v>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>파견근로자가 사용사업주의 구체적인 지시·감독을 받아 사용사업주의 업무를 행하던 중 불법행위를 한 경우, 파견사업주가 파견근로자의 선발 및 일반적 지휘·감독에 주의를 다하였다고 인정되면 파견사업주는 사용자책임을 면할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>파견근로</t>
+        </is>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>판례는 원칙적으로 파견사업주가 사용자책임을 지나, 사용사업주의 구체적 지시·감독 중의 불법행위에서 파견사업주가 선발·일반적 감독에 주의를 다하면 면책될 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>대판 2003.10.9. 2001다24655</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>제756조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="n">
+        <v>349</v>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>호의동승은 그 자체만으로 손해배상액의 감경사유가 된다.</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>호의동승</t>
+        </is>
+      </c>
+      <c r="F1193" t="inlineStr">
+        <is>
+          <t>판례는 단순한 호의동승 사실만으로는 배상액 감경사유가 되지 않고, 운행 목적·동승 경위 등에 비추어 신의칙·형평상 부당한 경우에 한하여 감경할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>대판 1992.5.12. 91다40993</t>
+        </is>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>제763조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="n">
+        <v>350</v>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>수급인이 자기의 노력과 재료로 건물을 신축한 경우 원칙적으로 수급인이 원시취득하지만, 도급인 명의로 건축허가·보존등기를 하기로 하는 등 완성된 건물의 소유권을 도급인에게 귀속시키기로 합의한 경우에는 도급인에게 원시적으로 귀속된다.</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>소유귀속</t>
+        </is>
+      </c>
+      <c r="F1194" t="inlineStr">
+        <is>
+          <t>판례는 신축건물의 원시취득자를 원칙적으로 수급인으로 보되 귀속 합의가 있으면 도급인이 원시취득한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>대판 2005.11.25. 2004다36352</t>
+        </is>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>제664조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="n">
+        <v>351</v>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>수급인의 하자담보책임은 법이 특별히 인정한 무과실책임이므로 민법 제396조의 과실상계 규정이 준용되지 않지만, 공평의 원칙상 하자 발생 및 확대에 가공한 도급인의 잘못을 참작할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>과실참작</t>
+        </is>
+      </c>
+      <c r="F1195" t="inlineStr">
+        <is>
+          <t>판례는 무과실책임인 하자담보책임에 과실상계가 준용되지 않으나 손해배상 범위 산정에서 도급인의 잘못을 참작할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>대판 2004.8.20. 2001다70337</t>
+        </is>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>제667조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="n">
+        <v>352</v>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>제3자를 위한 도급계약에서 수익의 의사표시를 한 수익자는, 요약자가 낙약자의 채무불이행을 이유로 계약을 해제한 경우 낙약자에게 자기가 입은 손해의 배상을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>수익자손해배상</t>
+        </is>
+      </c>
+      <c r="F1196" t="inlineStr">
+        <is>
+          <t>판례는 수익의 의사표시를 한 제3자가 낙약자의 채무불이행으로 입은 손해의 배상을 낙약자에게 청구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>대판 1994.8.12. 92다41559</t>
+        </is>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>제539조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="n">
+        <v>353</v>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>임차인의 채무불이행으로 임대차계약이 해지된 경우, 임차인은 부속물매수청구권을 행사할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1197" t="inlineStr">
+        <is>
+          <t>채무불이행</t>
+        </is>
+      </c>
+      <c r="F1197" t="inlineStr">
+        <is>
+          <t>판례는 임차인의 채무불이행으로 인한 해지의 경우 부속물매수청구권이 인정되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1197" t="inlineStr">
+        <is>
+          <t>대판 1990.1.23. 88다카7245</t>
+        </is>
+      </c>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>제646조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="n">
+        <v>354</v>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>권리금이 일정 기간 이상 임차권을 보장하는 약정 하에 지급된 경우, 그 보장기간 동안의 이용이 유효하게 이루어졌다면 임대인은 권리금의 반환의무를 지지 않지만, 임대인의 사정으로 중도 해지되면 임대인은 권리금의 반환의무를 진다.</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1198" t="inlineStr">
+        <is>
+          <t>권리금</t>
+        </is>
+      </c>
+      <c r="F1198" t="inlineStr">
+        <is>
+          <t>판례는 임차권 보장 약정 하의 권리금에서 보장기간 이용이 이루어지면 반환의무가 없으나, 임대인의 사정으로 중도 해지되면 잔여기간에 상응하는 반환의무를 진다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1198" t="inlineStr">
+        <is>
+          <t>대판 2002.7.26. 2002다25013</t>
+        </is>
+      </c>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>제618조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="n">
+        <v>355</v>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>지상물매수청구권의 대상이 되는 건물은 반드시 임대차계약 당시의 기존 건물이거나 임대인의 동의를 얻어 신축한 것에 한정되며, 무허가건물은 그 대상이 되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1199" t="inlineStr">
+        <is>
+          <t>매수청구</t>
+        </is>
+      </c>
+      <c r="F1199" t="inlineStr">
+        <is>
+          <t>판례는 지상물매수청구권의 공익적 목적상 임대차 당시의 기존 건물이나 임대인 동의를 얻은 신축 건물에 한정되지 않고 무허가건물도 그 대상이 된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1199" t="inlineStr">
+        <is>
+          <t>대판 1993.11.12. 93다34589 등</t>
+        </is>
+      </c>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>제643조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="n">
+        <v>356</v>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>매도인이 매수인에 대하여 매매계약의 이행을 최고하고 매매잔대금의 지급을 구하는 소송을 제기한 것만으로는, 민법 제565조의 이행에 착수하였다고 볼 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1200" t="inlineStr">
+        <is>
+          <t>이행착수</t>
+        </is>
+      </c>
+      <c r="F1200" t="inlineStr">
+        <is>
+          <t>판례는 이행청구·대금 지급 소송 제기만으로는 이행의 착수가 아니므로 해약금 해제가 여전히 가능하다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1200" t="inlineStr">
+        <is>
+          <t>대판 2008.10.23. 2007다72274</t>
+        </is>
+      </c>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>제565조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="n">
+        <v>357</v>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>부동산 매매계약 체결 후 매수인 앞으로 이전등기를 마치기 전에 제3자가 그 부동산을 다시 매수하여 처분금지가처분등기를 한 상태에서 매매계약이 해제된 경우, 가처분등기의 말소와 매도인의 대금반환의무는 동시이행관계에 있지 않다.</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1201" t="inlineStr">
+        <is>
+          <t>동시이행</t>
+        </is>
+      </c>
+      <c r="F1201" t="inlineStr">
+        <is>
+          <t>판례는 가처분등기 말소의무와 매도인의 대금반환의무 사이에 견련관계가 없어 동시이행관계가 아니라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1201" t="inlineStr">
+        <is>
+          <t>대판 2009.7.9. 2009다18526</t>
+        </is>
+      </c>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>제536조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="n">
+        <v>358</v>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>민법 제450조 제2항의 채권양도의 제3자에 대한 대항요건은 양도된 채권이 존속하는 동안 양수인의 지위와 양립할 수 없는 법률상 지위를 취득한 제3자가 있는 경우에 적용되므로, 양도된 채권이 이미 변제로 소멸한 경우에는 문제되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1202" t="inlineStr">
+        <is>
+          <t>대항요건</t>
+        </is>
+      </c>
+      <c r="F1202" t="inlineStr">
+        <is>
+          <t>판례는 채권이 변제로 소멸한 경우 대항요건의 우열 문제가 발생하지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1202" t="inlineStr">
+        <is>
+          <t>대판 2003.10.24. 2003다37426</t>
+        </is>
+      </c>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>제450조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="n">
+        <v>359</v>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>연대채무자 1인에 대한 이행청구는 다른 연대채무자에게도 효력이 있으므로, 그 이행청구로 인한 이행지체의 효과도 다른 연대채무자에게 미친다.</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1203" t="inlineStr">
+        <is>
+          <t>절대효</t>
+        </is>
+      </c>
+      <c r="F1203" t="inlineStr">
+        <is>
+          <t>판례는 제416조에 따라 연대채무자 1인에 대한 이행청구가 절대효를 가지므로 그로 인한 이행지체도 다른 연대채무자에게 효력이 미친다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1203" t="inlineStr">
+        <is>
+          <t>민법 제416조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>제416조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="n">
+        <v>360</v>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>채권자대위권 행사의 통지를 받은 후 또는 채무자가 대위권 행사 사실을 안 후에도, 채무자가 자신의 명의로 소유권이전등기를 경료하는 것은 처분행위가 아니므로 채권자에게 대항할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1204" t="inlineStr">
+        <is>
+          <t>처분해당성</t>
+        </is>
+      </c>
+      <c r="F1204" t="inlineStr">
+        <is>
+          <t>판례는 채무자의 변제수령이나 소유권이전등기 경료는 처분행위가 아니어서 대위권 행사 통지 후에도 가능하다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1204" t="inlineStr">
+        <is>
+          <t>대판 1991.4.12. 90다9407</t>
+        </is>
+      </c>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>제405조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="n">
+        <v>361</v>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>보증한도액을 정한 근보증에서 보증채무는 특별한 사정이 없는 한 보증한도 범위 안에서 확정된 주채무 및 그 이자, 위약금, 손해배상 기타 주채무에 종속한 채무를 모두 포함한다.</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1205" t="inlineStr">
+        <is>
+          <t>보증범위</t>
+        </is>
+      </c>
+      <c r="F1205" t="inlineStr">
+        <is>
+          <t>판례는 근보증의 보증한도액에 주채무의 이자·위약금·손해배상 등 종속채무가 모두 포함된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1205" t="inlineStr">
+        <is>
+          <t>대판 2000.4.11. 99다12123</t>
+        </is>
+      </c>
+      <c r="H1205" t="inlineStr">
+        <is>
+          <t>제429조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="n">
+        <v>362</v>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>주채무자가 채무를 승인하여 소멸시효가 중단된 경우, 그 시효중단의 효력은 보증인에게도 미친다.</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1206" t="inlineStr">
+        <is>
+          <t>중단효력</t>
+        </is>
+      </c>
+      <c r="F1206" t="inlineStr">
+        <is>
+          <t>민법 제440조는 주채무자에 대한 시효중단이 보증인에게도 효력이 있다고 정한다.</t>
+        </is>
+      </c>
+      <c r="G1206" t="inlineStr">
+        <is>
+          <t>민법 제440조</t>
+        </is>
+      </c>
+      <c r="H1206" t="inlineStr">
+        <is>
+          <t>제440조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="n">
+        <v>363</v>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>채권자취소소송에서 피보전채권의 존재는 본안판단 사항이므로 피보전채권이 인정되지 않으면 청구를 기각하지만, 채권자대위소송에서 피보전채권은 당사자적격의 문제이므로 인정되지 않으면 소를 각하한다.</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>소송요건</t>
+        </is>
+      </c>
+      <c r="F1207" t="inlineStr">
+        <is>
+          <t>판례는 채권자취소소송의 피보전채권을 본안사항(기각), 채권자대위소송의 피보전채권을 소송요건(각하)으로 구별한다.</t>
+        </is>
+      </c>
+      <c r="G1207" t="inlineStr">
+        <is>
+          <t>대판 2008.2.15. 2006다26243 등</t>
+        </is>
+      </c>
+      <c r="H1207" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="n">
+        <v>364</v>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>저당권이 설정된 부동산에 관하여 사해행위가 이루어진 후 변제 등으로 저당권설정등기가 말소된 경우, 채권자는 부동산 자체의 회복이 아니라 부동산 가액에서 피담보채무액을 공제한 잔액의 한도에서 사해행위를 취소하고 가액배상을 구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>가액배상</t>
+        </is>
+      </c>
+      <c r="F1208" t="inlineStr">
+        <is>
+          <t>판례는 사해행위 후 저당권이 말소된 경우 원물반환은 공평에 반하므로 가액배상에 의하도록 한다.</t>
+        </is>
+      </c>
+      <c r="G1208" t="inlineStr">
+        <is>
+          <t>대판 1998.2.13. 97다6711</t>
+        </is>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="n">
+        <v>365</v>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>채권자취소권은 취소원인을 안 날로부터 1년, 법률행위가 있은 날로부터 5년 내에 행사하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>제척기간</t>
+        </is>
+      </c>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>민법 제406조 제2항의 명문 규정이다.</t>
+        </is>
+      </c>
+      <c r="G1209" t="inlineStr">
+        <is>
+          <t>민법 제406조②</t>
+        </is>
+      </c>
+      <c r="H1209" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="n">
+        <v>366</v>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>채권자가 수익자를 상대로 사해행위 취소를 구하여 승소판결이 확정된 경우, 그 판결의 효력은 소송 당사자가 아닌 전득자에게도 미친다.</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>상대효</t>
+        </is>
+      </c>
+      <c r="F1210" t="inlineStr">
+        <is>
+          <t>판례는 취소판결의 효력이 소송 당사자가 아닌 전득자에게 미치지 않으므로, 전득자에 대해서는 별도로 제406조 제2항의 기간 내에 채무자·수익자 간 사해행위 취소의 소를 제기해야 한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1210" t="inlineStr">
+        <is>
+          <t>대판 2004.8.30. 2004다21923</t>
+        </is>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="n">
+        <v>367</v>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>변제할 정당한 이익이 있는 자가 근저당권의 피담보채무 일부를 대위변제한 경우, 대위변제자는 근저당권 일부이전의 부기등기 경료 여부와 관계없이 변제한 가액 범위에서 채권 및 담보에 관한 권리를 법률상 당연히 취득하며, 이때에도 채권자는 일부 대위변제자에 대하여 우선변제권을 가진다.</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>일부대위</t>
+        </is>
+      </c>
+      <c r="F1211" t="inlineStr">
+        <is>
+          <t>판례는 일부 대위변제 시 부기등기 여부와 무관하게 권리를 당연 취득하나 채권자가 잔존 채권에 관하여 우선변제권을 가진다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1211" t="inlineStr">
+        <is>
+          <t>대판 2002.7.26. 2001다53929</t>
+        </is>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>제483조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="n">
+        <v>368</v>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>저당물의 후순위 근저당권자는 민법 제482조 제2항 제2호의 '제3취득자'에 포함되지 않으므로, 후순위 근저당권자는 보증인에 대하여 채권자를 대위할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>대위관계</t>
+        </is>
+      </c>
+      <c r="F1212" t="inlineStr">
+        <is>
+          <t>판례는 후순위 근저당권자가 제482조 제2항 제2호의 제3취득자에 포함되지 않으므로, 오히려 저당물의 후순위 근저당권자가 보증인에 대하여 채권자를 대위할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1212" t="inlineStr">
+        <is>
+          <t>대판 2013.2.15. 2012다48855</t>
+        </is>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>제482조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="n">
+        <v>369</v>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>보증인은 미리 저당권의 등기에 그 대위를 부기하지 않고서도, 저당물에 후순위 근저당권을 취득한 제3자에 대하여 채권자를 대위할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>대위관계</t>
+        </is>
+      </c>
+      <c r="F1213" t="inlineStr">
+        <is>
+          <t>판례는 후순위 근저당권자가 제482조 제2항 제1호의 '제3자'에 포함되지 않으므로 보증인이 부기등기 없이도 그에 대하여 채권자를 대위할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>대판 2013.2.15. 2012다48855</t>
+        </is>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>제482조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="n">
+        <v>370</v>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>제3자의 변제에서 이해관계 있는 제3자란 변제하지 않으면 채권자로부터 집행을 받거나 채무자에 대한 자기의 권리를 잃게 되는 지위에 있어 변제할 정당한 이익이 있는 자를 말하며, 물상보증인·담보물의 제3취득자 등이 이에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>이해관계인</t>
+        </is>
+      </c>
+      <c r="F1214" t="inlineStr">
+        <is>
+          <t>판례는 이해관계 있는 제3자를 변제할 정당한 이익이 있는 자로 보고 물상보증인·제3취득자 등을 포함한다.</t>
+        </is>
+      </c>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>민법 제469조·제481조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>제469조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="n">
+        <v>371</v>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>매매계약상 금전채무자가 채권자의 지시에 따라 채권자의 채권자에게 직접 금전을 지급한 단축급부에서 매매계약이 무효·해제된 경우, 금전채무자는 매매계약의 상대방인 채권자에게 부당이득반환을 구할 수 있을 뿐 그 채권자의 채권자에게는 구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>삼각관계</t>
+        </is>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>판례는 단축급부 시 급부가 계약당사자 간에 이루어진 것이므로 제3자가 아닌 계약 상대방에게 부당이득반환을 구해야 한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1215" t="inlineStr">
+        <is>
+          <t>대판 2003.12.26. 2001다46730</t>
+        </is>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="n">
+        <v>372</v>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>인지 전에 공동상속인들에 의하여 이미 분할되거나 처분된 상속재산은, 분할받은 공동상속인이나 그로부터 양수한 자에게 소유권이 확정적으로 귀속되고, 사후 인지된 자는 가액의 지급을 청구할 수 있을 뿐이다.</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>인지후분할</t>
+        </is>
+      </c>
+      <c r="F1216" t="inlineStr">
+        <is>
+          <t>판례는 제1014조에 따라 인지 전 분할·처분의 효력을 인정하고 사후 인지자에게는 가액지급청구권만 인정한다.</t>
+        </is>
+      </c>
+      <c r="G1216" t="inlineStr">
+        <is>
+          <t>민법 제1014조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>제1014조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="n">
+        <v>373</v>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>변시3</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>친권자가 수인의 미성년 자녀의 법정대리인으로서 상속재산 분할협의를 한 경우, 그 분할협의는 피대리자 전원에 의한 추인이 없는 한 무효이다.</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1217" t="inlineStr">
+        <is>
+          <t>이해상반</t>
+        </is>
+      </c>
+      <c r="F1217" t="inlineStr">
+        <is>
+          <t>판례는 공동상속인인 친권자와 여러 미성년 자녀 사이의 분할협의가 이해상반행위이므로 각자 특별대리인을 선임해야 하고 위반 시 전원 추인 없으면 무효라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>대판 1994.9.9. 94다6680</t>
+        </is>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>제921조</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 변시2 OX (1282 items)
</commit_message>
<xml_diff>
--- a/assets/ox_civil_bar14.xlsx
+++ b/assets/ox_civil_bar14.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1217"/>
+  <dimension ref="A1:H1283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -49144,6 +49144,2646 @@
         </is>
       </c>
     </row>
+    <row r="1218">
+      <c r="A1218" t="n">
+        <v>201</v>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>재단법인의 기존 기본재산을 처분하는 행위뿐만 아니라 새로이 기본재산으로 편입하는 행위도 정관변경을 초래하므로 주무관청의 허가가 있어야 유효하다.</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1218" t="inlineStr">
+        <is>
+          <t>기본재산</t>
+        </is>
+      </c>
+      <c r="F1218" t="inlineStr">
+        <is>
+          <t>판례는 기본재산의 편입·처분 모두 정관변경사항이어서 주무관청 허가를 받아야 효력이 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1218" t="inlineStr">
+        <is>
+          <t>대판 1982.9.28. 82다카499</t>
+        </is>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>제42조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="n">
+        <v>202</v>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>비법인사단의 총유재산 보존을 위한 소송은 그 대표자가 개인 자격으로 당사자가 되어 제기하면 충분하고, 사원총회의 결의나 구성원 전원의 참여는 필요하지 않다.</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1219" t="inlineStr">
+        <is>
+          <t>총유보존</t>
+        </is>
+      </c>
+      <c r="F1219" t="inlineStr">
+        <is>
+          <t>총유재산에 관한 소송은 사원총회 결의를 거쳐 사단 명의로 하거나 구성원 전원이 필수적 공동소송 형태로 제기해야 하고, 대표자 개인은 당사자가 될 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1219" t="inlineStr">
+        <is>
+          <t>대판(전) 2005.9.15. 2004다44971</t>
+        </is>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>제276조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="n">
+        <v>203</v>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>통정허위표시에 의하여 외형상 형성된 법률관계를 토대로 새로 그 채권을 가압류한 자도 민법 제108조 제2항의 보호받는 선의의 제3자에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>허위표시제3자</t>
+        </is>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>판례는 허위표시에 기한 채권을 가압류한 자도 새로운 이해관계를 맺은 선의의 제3자로 보호된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>대판 2004.5.28. 2003다70041</t>
+        </is>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>제108조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="n">
+        <v>204</v>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>제3자의 사기로 의사표시를 한 자는 그 계약을 취소하지 않고서도 제3자에 대하여 불법행위를 원인으로 한 손해배상을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>제3자사기</t>
+        </is>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>판례는 계약을 취소하지 않더라도 제3자의 기망으로 인한 손해에 관하여 불법행위 손해배상을 청구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1221" t="inlineStr">
+        <is>
+          <t>대판 1998.3.10. 97다55829</t>
+        </is>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>제110조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="n">
+        <v>205</v>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>통정허위표시에서 파산관재인이 민법 제108조 제2항의 제3자에 해당하는 경우, 그 선의·악의는 파산관재인 개인을 기준으로 판단하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>파산관재인</t>
+        </is>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>파산관재인은 총파산채권자를 대표하므로 선의 여부는 파산관재인 개인이 아니라 총파산채권자를 기준으로 판단한다.</t>
+        </is>
+      </c>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>대판(전) 2006.11.23. 2004다3925</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>제108조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="n">
+        <v>206</v>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>매매계약 체결에 관한 포괄적 대리권을 수여받은 대리인은 그 매매대금 지급기일을 연기하여 줄 권한도 가진다.</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>대리권범위</t>
+        </is>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>판례는 매매계약 체결의 포괄적 대리권에는 대금지급기일 연기 권한도 포함된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t>대판 1992.4.14. 91다43107</t>
+        </is>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>제118조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="n">
+        <v>207</v>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>대리인이 상대방에게 기망행위를 한 경우, 대리인은 민법 제110조 제2항의 '제3자'에 해당하므로 본인이 그 사실을 몰랐다면 상대방은 의사표시를 취소할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1224" t="inlineStr">
+        <is>
+          <t>대리인사기</t>
+        </is>
+      </c>
+      <c r="F1224" t="inlineStr">
+        <is>
+          <t>대리인은 제110조 제2항의 제3자에 해당하지 않으므로, 대리인의 기망이 있으면 본인의 선의 여부와 무관하게 상대방은 의사표시를 취소할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1224" t="inlineStr">
+        <is>
+          <t>대판 1998.1.23. 96다41496</t>
+        </is>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>제110조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="n">
+        <v>208</v>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>선의의 점유자라도 본권에 관한 소에서 패소한 때에는 그 소가 제기된 때부터 악의의 점유자로 본다.</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1225" t="inlineStr">
+        <is>
+          <t>악의의제</t>
+        </is>
+      </c>
+      <c r="F1225" t="inlineStr">
+        <is>
+          <t>민법 제197조 제2항에 따라 선의 점유자도 본권의 소에서 패소하면 소 제기 시부터 악의 점유자로 간주된다.</t>
+        </is>
+      </c>
+      <c r="G1225" t="inlineStr">
+        <is>
+          <t>민법 제197조 제2항</t>
+        </is>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>제197조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="n">
+        <v>209</v>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>점유취득시효가 완성된 점유자는 아직 소유권이전등기를 마치기 전이라도 소유자를 상대로 소유권확인의 소를 제기하여 승소할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1226" t="inlineStr">
+        <is>
+          <t>시효완성확인</t>
+        </is>
+      </c>
+      <c r="F1226" t="inlineStr">
+        <is>
+          <t>점유취득시효가 완성되어도 등기 전에는 소유권을 취득하지 못하므로 소유권확인소송에서 승소할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1226" t="inlineStr">
+        <is>
+          <t>민법 제245조 제1항 · 판례</t>
+        </is>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>제245조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="n">
+        <v>210</v>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>점유취득시효기간이 만료된 후에 그 토지의 소유권을 취득한 제3자에 대하여, 시효완성자는 등기 없이도 시효취득을 주장할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1227" t="inlineStr">
+        <is>
+          <t>시효후취득자</t>
+        </is>
+      </c>
+      <c r="F1227" t="inlineStr">
+        <is>
+          <t>시효완성 후 등기 전에 소유권을 취득한 제3자에게는 시효취득을 주장할 수 없다(이중매매 법리와 유사).</t>
+        </is>
+      </c>
+      <c r="G1227" t="inlineStr">
+        <is>
+          <t>대판 1998.7.10. 97다45402</t>
+        </is>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>제245조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="n">
+        <v>211</v>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>매매 등 쌍무계약이 불공정한 법률행위에 해당하여 무효인 경우, 그 계약에 관하여 별도로 체결한 부제소합의도 무효이다.</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1228" t="inlineStr">
+        <is>
+          <t>불공정합의</t>
+        </is>
+      </c>
+      <c r="F1228" t="inlineStr">
+        <is>
+          <t>판례는 불공정한 법률행위로 무효인 계약에 부수된 부제소합의 역시 무효라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>대판 2010.7.15. 2009다50308</t>
+        </is>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>제104조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="n">
+        <v>212</v>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>무효인 가등기를 유효한 등기로 전용하기로 하는 약정은 무효행위의 추인에 해당하나, 그 추인에는 소급효가 인정되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1229" t="inlineStr">
+        <is>
+          <t>무효행위추인</t>
+        </is>
+      </c>
+      <c r="F1229" t="inlineStr">
+        <is>
+          <t>무효행위의 추인은 새로운 행위로 보므로 소급효가 없고 추인한 때부터 유효하다.</t>
+        </is>
+      </c>
+      <c r="G1229" t="inlineStr">
+        <is>
+          <t>민법 제139조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>제139조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="n">
+        <v>213</v>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>수급인이 자기의 노력과 재료를 들여 건물을 신축한 경우, 도급인에게 소유권을 귀속시키기로 하는 특약이 없으면 그 건물의 소유권은 수급인이 원시취득한다.</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1230" t="inlineStr">
+        <is>
+          <t>신축건물귀속</t>
+        </is>
+      </c>
+      <c r="F1230" t="inlineStr">
+        <is>
+          <t>판례는 특약이 없는 한 자기 재료로 건물을 신축한 수급인이 소유권을 원시취득한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1230" t="inlineStr">
+        <is>
+          <t>대판 2005.11.25. 2004다36352</t>
+        </is>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>제664조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="n">
+        <v>214</v>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>유치권자는 유치물을 경매에 부쳐 환가할 수는 있으나, 그 매각대금으로부터 다른 채권자에 우선하여 변제받을 우선변제권은 인정되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1231" t="inlineStr">
+        <is>
+          <t>유치권환가</t>
+        </is>
+      </c>
+      <c r="F1231" t="inlineStr">
+        <is>
+          <t>유치권자는 형식적 경매로 환가할 수 있지만 우선변제권은 없고 일반채권자로 배당받는다.</t>
+        </is>
+      </c>
+      <c r="G1231" t="inlineStr">
+        <is>
+          <t>민법 제322조 · 제320조</t>
+        </is>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>제322조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="n">
+        <v>215</v>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>유치권의 행사, 즉 점유의 계속은 피담보채권의 소멸시효 진행을 중단시키는 효력이 있다.</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1232" t="inlineStr">
+        <is>
+          <t>유치권시효</t>
+        </is>
+      </c>
+      <c r="F1232" t="inlineStr">
+        <is>
+          <t>민법 제326조에 따라 유치권의 행사는 피담보채권의 소멸시효 진행에 영향을 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1232" t="inlineStr">
+        <is>
+          <t>민법 제326조</t>
+        </is>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>제326조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="n">
+        <v>216</v>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>근저당권자가 피담보채무의 불이행을 이유로 경매를 신청한 경우 그 경매신청 시에 피담보채권액이 확정되며, 이후 경매신청을 취하하더라도 확정의 효과는 번복되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1233" t="inlineStr">
+        <is>
+          <t>근저당확정</t>
+        </is>
+      </c>
+      <c r="F1233" t="inlineStr">
+        <is>
+          <t>판례는 근저당권자의 경매신청 시 채권이 확정되고 이후 취하해도 확정효과가 유지된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1233" t="inlineStr">
+        <is>
+          <t>대판 2002.11.26. 2001다73022</t>
+        </is>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>제357조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="n">
+        <v>217</v>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>후순위 근저당권자가 경매를 신청한 경우, 선순위 근저당권의 피담보채권은 후순위권자의 경매신청 시가 아니라 경락인이 경락대금을 완납한 때에 확정된다.</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1234" t="inlineStr">
+        <is>
+          <t>후순위확정</t>
+        </is>
+      </c>
+      <c r="F1234" t="inlineStr">
+        <is>
+          <t>판례는 후순위권자 경매신청 시 선순위 근저당 채권은 경락대금 완납 시에 확정된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1234" t="inlineStr">
+        <is>
+          <t>대판 1999.9.21. 99다26085</t>
+        </is>
+      </c>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>제357조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="n">
+        <v>218</v>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>미등기건물을 그 대지와 함께 매도하였으나 대지에 관하여만 매수인 앞으로 소유권이전등기가 경료된 경우, 매도인과 매수인 누구에게도 관습상의 법정지상권이 성립하지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1235" t="inlineStr">
+        <is>
+          <t>관습법정지상권</t>
+        </is>
+      </c>
+      <c r="F1235" t="inlineStr">
+        <is>
+          <t>판례는 대지·건물을 함께 매도한 사안에서는 관습상 법정지상권을 인정할 필요가 없어 성립하지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1235" t="inlineStr">
+        <is>
+          <t>대판 2002.6.20. 2002다9660</t>
+        </is>
+      </c>
+      <c r="H1235" t="inlineStr">
+        <is>
+          <t>제366조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="n">
+        <v>219</v>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>동산의 선의취득은 양도인이 무권리자라는 점을 제외하고는 거래행위 자체에 아무런 흠이 없어야 성립하므로, 기망을 이유로 취소된 거래로 점유를 승계한 자는 선의취득을 할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1236" t="inlineStr">
+        <is>
+          <t>선의취득요건</t>
+        </is>
+      </c>
+      <c r="F1236" t="inlineStr">
+        <is>
+          <t>판례는 유효한 거래행위를 전제로 선의취득이 성립하므로 취소된 거래의 점유 승계자는 선의취득할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1236" t="inlineStr">
+        <is>
+          <t>대판 1995.6.29. 94다22071</t>
+        </is>
+      </c>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>제249조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="n">
+        <v>220</v>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>손해배상 예정액은 부당히 과다한 경우 법원이 직권으로 감액할 수 있으나, 이미 예정된 손해배상액에 대하여 과실상계를 하는 것은 허용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1237" t="inlineStr">
+        <is>
+          <t>예정액감액</t>
+        </is>
+      </c>
+      <c r="F1237" t="inlineStr">
+        <is>
+          <t>판례는 손해배상 예정액은 직권 감액의 대상이나 과실상계는 따로 할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1237" t="inlineStr">
+        <is>
+          <t>대판 2002.1.25. 99다57126</t>
+        </is>
+      </c>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>제398조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="n">
+        <v>221</v>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>위약금 약정이 위약벌의 성질을 가지는 경우에도 법원은 민법 제398조 제2항을 유추적용하여 그 금액을 직권으로 감액할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1238" t="inlineStr">
+        <is>
+          <t>위약벌감액</t>
+        </is>
+      </c>
+      <c r="F1238" t="inlineStr">
+        <is>
+          <t>위약벌은 손해배상액의 예정과 달라 제398조 제2항이 적용되지 않으므로 직권 감액의 대상이 아니다(공서양속 위반 시 일부 무효만 가능).</t>
+        </is>
+      </c>
+      <c r="G1238" t="inlineStr">
+        <is>
+          <t>대판 2016.1.28. 2015다239324</t>
+        </is>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>제398조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="n">
+        <v>222</v>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>부동산실명법상 명의신탁약정과 그 약정에 따른 등기에 의한 물권변동은 모두 무효이다.</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1239" t="inlineStr">
+        <is>
+          <t>명의신탁무효</t>
+        </is>
+      </c>
+      <c r="F1239" t="inlineStr">
+        <is>
+          <t>부동산실명법 제4조 제1항·제2항에 따라 명의신탁약정과 그에 따른 물권변동은 무효이다.</t>
+        </is>
+      </c>
+      <c r="G1239" t="inlineStr">
+        <is>
+          <t>부동산실명법 제4조</t>
+        </is>
+      </c>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>제103조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="n">
+        <v>223</v>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>부동산실명법 제4조 제3항의 보호되는 '제3자'에는 소유권이나 저당권을 취득한 자만 포함되고, 압류 또는 가압류채권자는 포함되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1240" t="inlineStr">
+        <is>
+          <t>명의신탁제3자</t>
+        </is>
+      </c>
+      <c r="F1240" t="inlineStr">
+        <is>
+          <t>판례는 수탁자가 물권자임을 기초로 새로운 이해관계를 맺은 자에는 압류·가압류채권자도 포함되며 선의·악의를 묻지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1240" t="inlineStr">
+        <is>
+          <t>대판 2000.3.28. 99다56529</t>
+        </is>
+      </c>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>제103조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="n">
+        <v>224</v>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>계약상 급부가 그 계약 상대방이 아닌 제3자의 이익으로 귀결된 경우에도, 급부를 한 계약당사자는 계약 상대방에게 반대급부를 청구할 수 있을 뿐 그 제3자에게 직접 부당이득반환을 청구할 수는 없다.</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1241" t="inlineStr">
+        <is>
+          <t>전용물소권</t>
+        </is>
+      </c>
+      <c r="F1241" t="inlineStr">
+        <is>
+          <t>판례는 이른바 전용물소권을 부정하여 급부자는 계약 상대방에게만 청구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1241" t="inlineStr">
+        <is>
+          <t>대판 2002.8.23. 99다66564</t>
+        </is>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="n">
+        <v>225</v>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>공유물의 관리에 관한 사항은 공유자 지분의 과반수로 결정하며, 토지의 구체적인 이용방법도 과반수 지분으로 정할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1242" t="inlineStr">
+        <is>
+          <t>공유관리</t>
+        </is>
+      </c>
+      <c r="F1242" t="inlineStr">
+        <is>
+          <t>민법 제265조에 따라 공유물의 관리는 지분 과반수로 결정한다.</t>
+        </is>
+      </c>
+      <c r="G1242" t="inlineStr">
+        <is>
+          <t>민법 제265조</t>
+        </is>
+      </c>
+      <c r="H1242" t="inlineStr">
+        <is>
+          <t>제265조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="n">
+        <v>226</v>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>공유물을 협의 없이 자신의 지분을 초과하여 배타적으로 점유하는 소수지분권자에 대하여, 다른 소수지분권자는 보존행위로서 공유물 전부의 인도를 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1243" t="inlineStr">
+        <is>
+          <t>소수지분인도</t>
+        </is>
+      </c>
+      <c r="F1243" t="inlineStr">
+        <is>
+          <t>판례(전합)는 소수지분권자는 다른 소수지분권자의 배타적 점유에 대해 보존행위로서 공유물 인도를 청구할 수 없고 방해배제만 구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1243" t="inlineStr">
+        <is>
+          <t>대판(전) 2020.5.21. 2018다287522</t>
+        </is>
+      </c>
+      <c r="H1243" t="inlineStr">
+        <is>
+          <t>제265조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="n">
+        <v>227</v>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>변제충당에서 당사자 사이의 합의에 의한 충당이 최우선하며, 비용·이자·원본의 순서도 약정에 의하여 배제할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1244" t="inlineStr">
+        <is>
+          <t>합의충당</t>
+        </is>
+      </c>
+      <c r="F1244" t="inlineStr">
+        <is>
+          <t>판례는 합의충당이 지정·법정충당에 우선하고 제479조의 순서도 약정으로 배제할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1244" t="inlineStr">
+        <is>
+          <t>민법 제476조·제479조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1244" t="inlineStr">
+        <is>
+          <t>제476조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="n">
+        <v>228</v>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>강제경매나 담보권 실행을 위한 경매절차에서 배당금을 충당하는 경우에는 지정변제충당이 허용되지 않고 법정변제충당의 방법에 의하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1245" t="inlineStr">
+        <is>
+          <t>경매충당</t>
+        </is>
+      </c>
+      <c r="F1245" t="inlineStr">
+        <is>
+          <t>판례는 경매절차의 배당충당에는 당사자의 지정충당이 허용되지 않고 법정충당만 인정된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1245" t="inlineStr">
+        <is>
+          <t>대판 1996.5.10. 95다55504</t>
+        </is>
+      </c>
+      <c r="H1245" t="inlineStr">
+        <is>
+          <t>제477조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="n">
+        <v>229</v>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>저당권설정등기는 효력발생요건일 뿐 효력존속요건은 아니므로, 위조서류에 의하여 저당권설정등기가 원인 없이 말소되더라도 그 저당권은 소멸하지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1246" t="inlineStr">
+        <is>
+          <t>불법말소</t>
+        </is>
+      </c>
+      <c r="F1246" t="inlineStr">
+        <is>
+          <t>판례는 등기는 효력존속요건이 아니므로 부적법하게 말소되어도 물권이 소멸하지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1246" t="inlineStr">
+        <is>
+          <t>대판 2001.1.16. 98다20110</t>
+        </is>
+      </c>
+      <c r="H1246" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="n">
+        <v>230</v>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>불법 말소된 근저당권설정등기의 목적 부동산이 경매절차에서 경락되어 근저당권이 소멸한 경우, 근저당권자는 실제로 배당받은 자에 대하여 부당이득반환을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1247" t="inlineStr">
+        <is>
+          <t>말소후경락</t>
+        </is>
+      </c>
+      <c r="F1247" t="inlineStr">
+        <is>
+          <t>판례는 불법말소 후 경락으로 근저당권이 소멸하면 배당받은 자에게 부당이득반환을 구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1247" t="inlineStr">
+        <is>
+          <t>대판 1998.10.2. 98다27197</t>
+        </is>
+      </c>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="n">
+        <v>231</v>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>채무자 소유 부동산과 물상보증인 소유 부동산이 함께 경매되어 그 대가를 동시에 배당하는 경우, 공동저당권자는 먼저 채무자 소유 부동산의 경매대가에서 우선 배당받고 부족분에 한하여 물상보증인 소유 부동산에서 배당받는다.</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1248" t="inlineStr">
+        <is>
+          <t>공동저당동시배당</t>
+        </is>
+      </c>
+      <c r="F1248" t="inlineStr">
+        <is>
+          <t>판례는 물상보증인 보호를 위해 채무자 소유 부동산에서 우선 배당하고 부족분만 물상보증인 부동산에서 배당한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1248" t="inlineStr">
+        <is>
+          <t>대판 2010.4.15. 2008다41475</t>
+        </is>
+      </c>
+      <c r="H1248" t="inlineStr">
+        <is>
+          <t>제368조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="n">
+        <v>232</v>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>대상청구권은 채무자의 귀책사유 없이 후발적 이행불능이 발생한 경우에도 행사할 수 있으며, 이때 채권자는 대상청구권과 부당이득반환청구권 중 하나를 선택하여 행사할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1249" t="inlineStr">
+        <is>
+          <t>대상청구권</t>
+        </is>
+      </c>
+      <c r="F1249" t="inlineStr">
+        <is>
+          <t>판례는 쌍방 책임 없는 사유로 후발적 불능이 된 경우에도 대상청구권을 인정하고 부당이득반환청구권과 선택적으로 행사할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1249" t="inlineStr">
+        <is>
+          <t>대판 1992.5.12. 92다4581 · 판례</t>
+        </is>
+      </c>
+      <c r="H1249" t="inlineStr">
+        <is>
+          <t>제390조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="n">
+        <v>233</v>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>채무자가 미리 이행하지 아니할 의사를 명백히 표시한 경우, 채권자는 이행기 전이라도 이행의 최고 없이 계약을 해제하거나 손해배상을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1250" t="inlineStr">
+        <is>
+          <t>이행거절</t>
+        </is>
+      </c>
+      <c r="F1250" t="inlineStr">
+        <is>
+          <t>판례는 채무자의 명백한 이행거절 시 이행기 전이라도 최고 없이 해제·손해배상청구가 가능하다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1250" t="inlineStr">
+        <is>
+          <t>대판 1993.6.25. 93다11821</t>
+        </is>
+      </c>
+      <c r="H1250" t="inlineStr">
+        <is>
+          <t>제544조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="n">
+        <v>234</v>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>매매계약에서 잔대금 지급의무와 소유권이전등기의무처럼 쌍방의 채무가 동시이행관계에 있는 경우, 자동해제(실권)약정이 있더라도 이행지체만으로 곧바로 계약이 자동해제되지는 않는다.</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1251" t="inlineStr">
+        <is>
+          <t>자동해제</t>
+        </is>
+      </c>
+      <c r="F1251" t="inlineStr">
+        <is>
+          <t>판례는 동시이행관계인 채무에서는 자동해제약정이 있어도 상대방의 이행제공 없이는 자동해제되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1251" t="inlineStr">
+        <is>
+          <t>대판 1998.6.12. 98다505</t>
+        </is>
+      </c>
+      <c r="H1251" t="inlineStr">
+        <is>
+          <t>제544조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="n">
+        <v>235</v>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>면책적 채무인수가 있으면 종전 채무에 대한 보증이나 제3자가 제공한 담보는 원칙적으로 소멸하나, 보증인이나 제3자가 채무인수에 동의한 경우에는 존속한다.</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1252" t="inlineStr">
+        <is>
+          <t>면책적인수</t>
+        </is>
+      </c>
+      <c r="F1252" t="inlineStr">
+        <is>
+          <t>민법 제459조에 따라 면책적 채무인수 시 담보는 원칙 소멸하되 동의가 있으면 존속한다.</t>
+        </is>
+      </c>
+      <c r="G1252" t="inlineStr">
+        <is>
+          <t>민법 제459조</t>
+        </is>
+      </c>
+      <c r="H1252" t="inlineStr">
+        <is>
+          <t>제459조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="n">
+        <v>236</v>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>임대차가 종료된 후 임차인이 목적물을 계속 점유·사용한 경우, 임차인은 인도 완료일까지 차임 상당의 부당이득을 임대인에게 반환할 의무가 있다.</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1253" t="inlineStr">
+        <is>
+          <t>종료후점유</t>
+        </is>
+      </c>
+      <c r="F1253" t="inlineStr">
+        <is>
+          <t>판례는 임대차 종료 후에도 점유·사용한 경우 차임 상당의 부당이득반환의무가 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1253" t="inlineStr">
+        <is>
+          <t>대판 1992.4.14. 91다45202</t>
+        </is>
+      </c>
+      <c r="H1253" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="n">
+        <v>237</v>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>주택임대차보호법상 임대인의 임대차보증금 반환의무와 임차인의 임차권등기 말소의무는 동시이행관계에 있다.</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1254" t="inlineStr">
+        <is>
+          <t>보증금말소</t>
+        </is>
+      </c>
+      <c r="F1254" t="inlineStr">
+        <is>
+          <t>판례는 임차권등기는 임대차보증금 반환을 담보하기 위한 것이므로 임대인의 보증금 반환의무가 임차권등기 말소의무보다 선이행의무라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1254" t="inlineStr">
+        <is>
+          <t>대판 2005.6.9. 2005다4529</t>
+        </is>
+      </c>
+      <c r="H1254" t="inlineStr">
+        <is>
+          <t>제536조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="n">
+        <v>238</v>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>과실상계는 채무불이행이나 불법행위로 인한 손해배상책임에 적용되지만, 고의의 불법행위를 저지른 가해자는 피해자의 과실을 들어 과실상계를 주장할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1255" t="inlineStr">
+        <is>
+          <t>고의과실상계</t>
+        </is>
+      </c>
+      <c r="F1255" t="inlineStr">
+        <is>
+          <t>판례는 고의의 불법행위자가 피해자의 부주의를 이용한 경우 과실상계 주장은 신의칙상 허용되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1255" t="inlineStr">
+        <is>
+          <t>대판 2007.10.25. 2006다16758</t>
+        </is>
+      </c>
+      <c r="H1255" t="inlineStr">
+        <is>
+          <t>제396조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="n">
+        <v>239</v>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>예금계약은 예금자가 금융기관에 돈을 제공하고 금융기관이 이를 받아 확인하면 성립하는 요물계약이며, 그 직원이 받은 돈을 실제로 입금하였는지 여부는 예금계약의 성립에 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1256" t="inlineStr">
+        <is>
+          <t>예금성립</t>
+        </is>
+      </c>
+      <c r="F1256" t="inlineStr">
+        <is>
+          <t>판례는 예금계약을 요물계약으로 보고 직원의 실제 입금 여부는 성립에 영향이 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1256" t="inlineStr">
+        <is>
+          <t>대판 1996.1.26. 95다26919</t>
+        </is>
+      </c>
+      <c r="H1256" t="inlineStr">
+        <is>
+          <t>제702조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="n">
+        <v>240</v>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>착오로 송금·이체가 이루어진 경우에도, 그 원인인 법률관계의 존부와 관계없이 수취인은 수취은행에 대하여 이체금액 상당의 예금채권을 취득한다.</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1257" t="inlineStr">
+        <is>
+          <t>착오송금</t>
+        </is>
+      </c>
+      <c r="F1257" t="inlineStr">
+        <is>
+          <t>판례는 착오송금이라도 원인관계 유무와 무관하게 수취인이 예금채권을 취득한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1257" t="inlineStr">
+        <is>
+          <t>대판 2007.11.29. 2007다51239</t>
+        </is>
+      </c>
+      <c r="H1257" t="inlineStr">
+        <is>
+          <t>제702조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="n">
+        <v>241</v>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>부진정연대채무자 중 1인에 대하여 채권자가 한 채무면제는 상대적 효력만 있을 뿐 다른 채무자에게는 영향을 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1258" t="inlineStr">
+        <is>
+          <t>부진정면제</t>
+        </is>
+      </c>
+      <c r="F1258" t="inlineStr">
+        <is>
+          <t>판례는 부진정연대채무에서 면제는 상대적 효력만 가진다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1258" t="inlineStr">
+        <is>
+          <t>대판 2006.1.27. 2005다19378</t>
+        </is>
+      </c>
+      <c r="H1258" t="inlineStr">
+        <is>
+          <t>제419조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="n">
+        <v>242</v>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>연대채무에서 소멸시효의 완성에 절대적 효력을 인정하는 규정은 공동불법행위자 상호간의 부진정연대채무에도 그대로 적용된다.</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1259" t="inlineStr">
+        <is>
+          <t>부진정시효</t>
+        </is>
+      </c>
+      <c r="F1259" t="inlineStr">
+        <is>
+          <t>부진정연대채무에는 연대채무의 소멸시효 절대효 규정이 적용되지 않으므로, 1인에 대한 시효완성은 다른 채무자에게 영향을 주지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1259" t="inlineStr">
+        <is>
+          <t>대판 1997.12.23. 97다42830</t>
+        </is>
+      </c>
+      <c r="H1259" t="inlineStr">
+        <is>
+          <t>제421조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="n">
+        <v>243</v>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>피상속인의 형제자매가 상속인이 되는 경우, 그 형제자매에는 아버지가 같고 어머니가 다른 동성이복형제뿐만 아니라 어머니가 같고 아버지가 다른 이성동복형제도 포함된다.</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1260" t="inlineStr">
+        <is>
+          <t>형제자매범위</t>
+        </is>
+      </c>
+      <c r="F1260" t="inlineStr">
+        <is>
+          <t>판례는 제3순위 상속인인 형제자매에 부계·모계를 불문하고 반혈족 형제자매가 모두 포함된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1260" t="inlineStr">
+        <is>
+          <t>대판 1997.11.28. 96다5421</t>
+        </is>
+      </c>
+      <c r="H1260" t="inlineStr">
+        <is>
+          <t>제1000조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="n">
+        <v>244</v>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>상속인이 될 직계비속이나 형제자매가 상속을 포기한 경우, 그 직계비속이 포기자를 대습하여 상속한다.</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1261" t="inlineStr">
+        <is>
+          <t>대습원인</t>
+        </is>
+      </c>
+      <c r="F1261" t="inlineStr">
+        <is>
+          <t>대습상속의 원인은 상속개시 전 사망 또는 상속결격에 한하고 상속포기는 대습원인이 아니므로, 포기자의 직계비속은 대습상속하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1261" t="inlineStr">
+        <is>
+          <t>민법 제1001조</t>
+        </is>
+      </c>
+      <c r="H1261" t="inlineStr">
+        <is>
+          <t>제1001조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="n">
+        <v>245</v>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>쌍무계약에서 채무자의 책임 있는 사유로 채무의 일부가 이행불능이 되었고 나머지 부분만으로는 계약의 목적을 달성할 수 없는 경우, 채권자는 이행이 가능한 부분만의 급부를 청구할 수는 없다.</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1262" t="inlineStr">
+        <is>
+          <t>일부불능</t>
+        </is>
+      </c>
+      <c r="F1262" t="inlineStr">
+        <is>
+          <t>판례는 일부 이행불능으로 계약목적을 달성할 수 없으면 전부불능으로 보아 가능 부분만의 급부청구는 허용되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1262" t="inlineStr">
+        <is>
+          <t>대판 1995.7.25. 95다5929</t>
+        </is>
+      </c>
+      <c r="H1262" t="inlineStr">
+        <is>
+          <t>제390조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="n">
+        <v>246</v>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>사해행위취소소송에서 채무자의 악의가 입증되면 수익자나 전득자의 악의는 추정되므로, 수익자나 전득자가 자신의 선의를 증명하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1263" t="inlineStr">
+        <is>
+          <t>사해의사추정</t>
+        </is>
+      </c>
+      <c r="F1263" t="inlineStr">
+        <is>
+          <t>판례는 채무자의 사해의사가 인정되면 수익자·전득자의 악의가 추정되어 그들이 선의를 입증해야 한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1263" t="inlineStr">
+        <is>
+          <t>대판 2006.4.14. 2006다5710</t>
+        </is>
+      </c>
+      <c r="H1263" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="n">
+        <v>247</v>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>채권자취소권은 채권자가 취소원인을 안 날부터 1년, 법률행위가 있은 날부터 5년 내에 행사하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>취소제척기간</t>
+        </is>
+      </c>
+      <c r="F1264" t="inlineStr">
+        <is>
+          <t>민법 제406조 제2항에 따라 채권자취소권의 제척기간은 안 날 1년, 행위일 5년이다.</t>
+        </is>
+      </c>
+      <c r="G1264" t="inlineStr">
+        <is>
+          <t>민법 제406조 제2항</t>
+        </is>
+      </c>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="n">
+        <v>248</v>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>채무자가 유일한 부동산을 매도하여 사해행위를 한 후에 비로소 신용카드 사용으로 카드대금채권이 발생한 경우, 그 카드대금채권도 사해행위취소의 피보전채권이 될 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>피보전채권</t>
+        </is>
+      </c>
+      <c r="F1265" t="inlineStr">
+        <is>
+          <t>사해행위 이후에 발생한 채권은 원칙적으로 피보전채권이 될 수 없으므로, 처분 후 발생한 카드대금채권은 피보전채권이 되지 못한다.</t>
+        </is>
+      </c>
+      <c r="G1265" t="inlineStr">
+        <is>
+          <t>대판 2002.11.8. 2002다42957</t>
+        </is>
+      </c>
+      <c r="H1265" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="n">
+        <v>249</v>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>형성권적 기한이익 상실의 특약이 있는 경우, 일정한 사유가 발생하더라도 채권자가 기한이익 상실의 의사표시를 하여야 비로소 이행기가 도래하여 지체책임이 생긴다.</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>기한이익상실</t>
+        </is>
+      </c>
+      <c r="F1266" t="inlineStr">
+        <is>
+          <t>판례는 기한이익 상실특약은 원칙적으로 형성권적 특약으로 추정되어 채권자의 의사표시가 있어야 이행기가 도래한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1266" t="inlineStr">
+        <is>
+          <t>대판 2002.9.4. 2002다28340</t>
+        </is>
+      </c>
+      <c r="H1266" t="inlineStr">
+        <is>
+          <t>제388조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="n">
+        <v>250</v>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>토지거래허가구역 내 토지에 관하여 허가를 받지 않아 유동적 무효 상태인 매매계약에서는, 이행지체를 이유로 한 계약해제나 손해배상청구를 할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>유동적무효</t>
+        </is>
+      </c>
+      <c r="F1267" t="inlineStr">
+        <is>
+          <t>판례는 유동적 무효 상태에서는 이행청구나 그를 전제로 한 이행지체·해제·손해배상청구를 할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1267" t="inlineStr">
+        <is>
+          <t>대판(전) 1991.12.24. 90다12243</t>
+        </is>
+      </c>
+      <c r="H1267" t="inlineStr">
+        <is>
+          <t>제105조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="n">
+        <v>251</v>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>양육권이 없는 부모 일방이 임의로 자녀를 양육한 경우, 그 양육은 위법한 양육이므로 상대방에게 양육비를 청구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>임의양육</t>
+        </is>
+      </c>
+      <c r="F1268" t="inlineStr">
+        <is>
+          <t>판례는 양육권 없는 자가 임의로 한 양육은 위법하여 상대방에게 양육비를 청구할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1268" t="inlineStr">
+        <is>
+          <t>대판 2006.4.17. 2005스18</t>
+        </is>
+      </c>
+      <c r="H1268" t="inlineStr">
+        <is>
+          <t>제837조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="n">
+        <v>252</v>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>주채무자가 소멸시효의 이익을 포기하더라도 그 효과는 보증인에게 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>시효이익포기</t>
+        </is>
+      </c>
+      <c r="F1269" t="inlineStr">
+        <is>
+          <t>시효이익 포기의 효과는 상대적이어서 주채무자의 포기는 보증인에게 영향을 주지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1269" t="inlineStr">
+        <is>
+          <t>민법 제433조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1269" t="inlineStr">
+        <is>
+          <t>제433조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="n">
+        <v>253</v>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>부동산실명법에 위반되어 무효인 명의신탁약정에 기하여 명의수탁자 앞으로 경료된 등기는 불법원인급여에 해당하여 신탁자가 그 반환을 구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>명의신탁급여</t>
+        </is>
+      </c>
+      <c r="F1270" t="inlineStr">
+        <is>
+          <t>판례는 부동산실명법 위반 명의신탁등기는 불법원인급여에 해당하지 않으므로 신탁자가 그 반환(말소)을 구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1270" t="inlineStr">
+        <is>
+          <t>대판(전) 2019.6.20. 2013다218156</t>
+        </is>
+      </c>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>제746조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="n">
+        <v>254</v>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>도박자금 채무를 담보하기 위하여 근저당권설정등기를 경료한 경우, 이는 종국적인 급여가 아니므로 근저당권설정자는 그 말소를 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>도박담보</t>
+        </is>
+      </c>
+      <c r="F1271" t="inlineStr">
+        <is>
+          <t>판례는 담보 목적의 근저당권설정등기는 종국적 급여가 아니어서 불법원인급여로 보지 않아 말소청구가 가능하다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1271" t="inlineStr">
+        <is>
+          <t>대판 1995.8.11. 94다54108</t>
+        </is>
+      </c>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>제746조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="n">
+        <v>255</v>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>혼인 중 부부가 협력하여 이룩한 재산이 있는 경우, 혼인 파탄에 책임이 있는 유책배우자라도 재산분할을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>유책재산분할</t>
+        </is>
+      </c>
+      <c r="F1272" t="inlineStr">
+        <is>
+          <t>판례는 재산분할은 부양·청산의 성질을 가지므로 유책배우자도 청구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1272" t="inlineStr">
+        <is>
+          <t>대결 1993.5.11. 93스6</t>
+        </is>
+      </c>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>제839조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="n">
+        <v>256</v>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>이혼에 따른 재산분할청구권은 이혼한 날부터 2년이 지나면 행사할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>분할제척기간</t>
+        </is>
+      </c>
+      <c r="F1273" t="inlineStr">
+        <is>
+          <t>민법 제839조의2 제3항에 따라 재산분할청구권은 이혼한 날부터 2년의 제척기간에 걸린다.</t>
+        </is>
+      </c>
+      <c r="G1273" t="inlineStr">
+        <is>
+          <t>민법 제839조의2 제3항</t>
+        </is>
+      </c>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>제839조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="n">
+        <v>257</v>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>한정승인을 한 채무자가 채권자의 소송에서 사실심 변론종결 시까지 그 사실을 주장하지 않아 패소 확정된 경우에도, 채무자는 그 후 한정승인 사실을 들어 청구이의의 소를 제기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>한정승인이의</t>
+        </is>
+      </c>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>판례는 한정승인은 책임의 범위에 관한 것이어서 변론종결 후에도 청구이의의 소로 주장할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1274" t="inlineStr">
+        <is>
+          <t>대판(전) 2006.10.13. 2006다23138</t>
+        </is>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>제1028조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="n">
+        <v>258</v>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>상속포기를 한 채무자가 채권자의 소송에서 사실심 변론종결 시까지 이를 주장하지 않아 패소 확정된 경우, 그 후 상속포기 사실을 들어 청구이의의 소를 제기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>상속포기이의</t>
+        </is>
+      </c>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>상속포기는 채무의 존부 자체에 관한 것이어서 변론종결 전에 주장했어야 하므로, 확정판결 후 청구이의의 소로 다툴 수 없다(기판력에 의해 차단).</t>
+        </is>
+      </c>
+      <c r="G1275" t="inlineStr">
+        <is>
+          <t>대판 2009.5.28. 2008다79876</t>
+        </is>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>제1019조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="n">
+        <v>259</v>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>무효행위의 추인은 그 무효원인이 소멸한 후에 이루어지더라도 원칙적으로 법률행위를 한 때로 소급하여 효력이 생긴다.</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>추인소급효</t>
+        </is>
+      </c>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>무효행위의 추인은 새로운 법률행위로 보므로 소급효가 없고 추인한 때부터 장래를 향하여 효력이 생긴다.</t>
+        </is>
+      </c>
+      <c r="G1276" t="inlineStr">
+        <is>
+          <t>민법 제139조</t>
+        </is>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>제139조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="n">
+        <v>260</v>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>강제경매나 담보권 실행을 위한 경매의 배당금 충당에서도 당사자가 지정한 변제충당이 법정변제충당에 우선하여 적용된다.</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>경매지정충당</t>
+        </is>
+      </c>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>경매절차의 배당충당에는 당사자의 지정충당이 허용되지 않고 법정변제충당만 적용된다.</t>
+        </is>
+      </c>
+      <c r="G1277" t="inlineStr">
+        <is>
+          <t>대판 1996.5.10. 95다55504</t>
+        </is>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>제477조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="n">
+        <v>261</v>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>대상청구권은 채무자에게 이행불능에 관한 귀책사유가 있는 경우에 한하여 인정되고, 당사자 쌍방에게 책임 없는 사유로 불능이 된 때에는 인정되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>대상청구귀책</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>대상청구권은 채무자의 귀책사유를 불문하고 인정되며, 쌍방에 책임 없는 후발적 불능의 경우에도 행사할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1278" t="inlineStr">
+        <is>
+          <t>대판 1992.5.12. 92다4581</t>
+        </is>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>제390조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="n">
+        <v>262</v>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>무효등기의 유용에 관한 합의는 그 합의 이전에 이미 등기상 이해관계를 가지게 된 제3자에 대하여도 대항할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>무효등기유용</t>
+        </is>
+      </c>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>무효등기 유용의 합의는 그 전에 등기상 이해관계를 가진 제3자에게는 대항할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1279" t="inlineStr">
+        <is>
+          <t>대판 2009.2.26. 2006다72802</t>
+        </is>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="n">
+        <v>263</v>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>주택임대차보호법상 우선변제권을 가진 임차인으로부터 임차권과 분리하여 임차보증금 반환채권만을 양수한 자도 주택임대차보호법상의 우선변제권을 행사할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>보증금채권양수</t>
+        </is>
+      </c>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>판례는 임차권과 분리하여 보증금반환채권만을 양수한 자는 주임법상 우선변제권을 행사할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1280" t="inlineStr">
+        <is>
+          <t>대판 2010.5.27. 2010다10276</t>
+        </is>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>제3조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="n">
+        <v>264</v>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>혼인 중 부부의 일방 명의로 취득한 재산은 부부의 공유로 추정되므로, 상대방의 협력이 있었다는 사정만으로도 그 재산은 재산분할의 대상이 된다.</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>특유재산추정</t>
+        </is>
+      </c>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>혼인 중 일방 명의로 취득한 재산은 명의자의 특유재산으로 추정되며, 단순한 내조의 공만으로는 그 추정이 번복되지 않는다(다만 유지·증식에 기여하면 분할대상).</t>
+        </is>
+      </c>
+      <c r="G1281" t="inlineStr">
+        <is>
+          <t>대판 1998.4.10. 96므1434</t>
+        </is>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>제830조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="n">
+        <v>265</v>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>채권자가 주채무자에 대하여 변제기를 연장하여 준 경우, 그 효력은 연대보증채무에는 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>변제기연장</t>
+        </is>
+      </c>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>채권자가 주채무자에게 변제기를 연장해 주면 그 효력은 보증채무에도 미친다.</t>
+        </is>
+      </c>
+      <c r="G1282" t="inlineStr">
+        <is>
+          <t>민법 제430조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>제430조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="n">
+        <v>266</v>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>변시2</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>수탁보증인이 주채무자에게 사전통지를 하지 않고 변제 등 면책행위를 하였는데, 그에 앞서 주채무자가 이미 면책행위를 하고도 보증인에게 통지하지 않은 경우, 보증인은 자신의 면책행위가 유효함을 주장하여 주채무자에게 구상할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>이중면책</t>
+        </is>
+      </c>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>주채무자가 먼저 면책행위를 한 이상 채무소멸의 일반원칙에 따라 선행 변제가 유효하므로, 사전통지 없이 이중으로 면책행위를 한 보증인은 주채무자에게 구상할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1283" t="inlineStr">
+        <is>
+          <t>민법 제446조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>제446조</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 변시1 OX (1354 items, all years 1-14)
</commit_message>
<xml_diff>
--- a/assets/ox_civil_bar14.xlsx
+++ b/assets/ox_civil_bar14.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1283"/>
+  <dimension ref="A1:H1355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -51784,6 +51784,2886 @@
         </is>
       </c>
     </row>
+    <row r="1284">
+      <c r="A1284" t="n">
+        <v>101</v>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>고의의 불법행위로 인한 손해배상채권을 수동채권으로 하는 상계는 허용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>상계금지</t>
+        </is>
+      </c>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>민법 제496조에 따라 고의의 불법행위로 인한 손해배상채권을 수동채권으로 하는 상계는 금지된다.</t>
+        </is>
+      </c>
+      <c r="G1284" t="inlineStr">
+        <is>
+          <t>민법 제496조</t>
+        </is>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>제496조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="n">
+        <v>102</v>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>피용자의 고의의 불법행위로 사용자책임이 성립하는 경우, 그 사용자책임에 기한 손해배상채권을 수동채권으로 하는 상계도 허용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>사용자책임상계</t>
+        </is>
+      </c>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>판례는 사용자책임이 피용자의 고의 불법행위에 대한 대체적 책임이므로 이를 수동채권으로 하는 상계도 제496조 취지상 금지된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1285" t="inlineStr">
+        <is>
+          <t>대판 2006.10.26. 2004다63019</t>
+        </is>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>제496조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="n">
+        <v>103</v>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>상계의 수동채권은 상계자가 상대방에 대하여 부담하는 채무여야 하므로, 상대방이 제3자에 대하여 가지는 채권을 수동채권으로 하여 상계할 수는 없다.</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>수동채권요건</t>
+        </is>
+      </c>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>수동채권은 상계자가 상대방에게 부담하는 채무여야 하므로 상대방의 제3자에 대한 채권을 수동채권으로 삼을 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1286" t="inlineStr">
+        <is>
+          <t>민법 제492조</t>
+        </is>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>제492조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="n">
+        <v>104</v>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>혼인 외의 자를 혼인 중의 친생자로 출생신고한 경우, 그 신고는 인지신고로서의 효력이 인정된다.</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>무효행위전환</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>판례는 혼인외 자를 친생자로 출생신고한 경우 인지의 효력을 인정한다(무효행위의 전환).</t>
+        </is>
+      </c>
+      <c r="G1287" t="inlineStr">
+        <is>
+          <t>대판 1971.11.15. 71다1983</t>
+        </is>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>제855조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="n">
+        <v>105</v>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>비밀증서에 의한 유언이 그 방식에 흠결이 있더라도 자필증서에 의한 유언의 방식에 적합한 때에는 자필증서에 의한 유언으로서 효력이 있다.</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>유언전환</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>민법 제1071조에 따라 방식에 흠결 있는 비밀증서 유언이 자필증서 방식을 갖추면 자필증서 유언으로 전환된다.</t>
+        </is>
+      </c>
+      <c r="G1288" t="inlineStr">
+        <is>
+          <t>민법 제1071조</t>
+        </is>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>제1071조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="n">
+        <v>106</v>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>법적 절차에 따라 진행되는 경매에는 민법 제104조의 불공정한 법률행위에 관한 규정이 적용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>경매불공정</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>판례는 경매에는 제104조가 적용되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1289" t="inlineStr">
+        <is>
+          <t>대결 1980.3.21. 80마77</t>
+        </is>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>제104조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="n">
+        <v>107</v>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>불공정한 법률행위인지를 판단할 때 경솔·무경험은 대리인을 기준으로, 궁박 상태는 본인을 기준으로 판단한다.</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>불공정판단기준</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>판례는 대리행위의 경우 경솔·무경험은 대리인을, 궁박은 본인을 기준으로 판단한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1290" t="inlineStr">
+        <is>
+          <t>대판 2002.10.22. 2002다38927</t>
+        </is>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>제104조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="n">
+        <v>108</v>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>불공정한 법률행위로서 무효인 경우에도 당사자가 이를 추인하면 유효한 것으로 된다.</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>불공정추인</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>불공정한 법률행위는 절대적 무효여서 추인에 의하여 유효로 될 수 없다(다만 무효행위 전환은 가능).</t>
+        </is>
+      </c>
+      <c r="G1291" t="inlineStr">
+        <is>
+          <t>대판 1994.6.24. 94다10900</t>
+        </is>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>제104조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="n">
+        <v>109</v>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>강제집행을 면탈할 목적으로 통정하여 체결한 가장매매라도 그것만으로 민법 제103조 위반이나 불법원인급여에 해당하는 것은 아니어서, 급부한 자는 부당이득반환을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>강제집행면탈</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>판례는 강제집행 면탈 목적의 가장매매가 제103조 위반이나 불법원인급여에 해당하지 않아 반환청구가 가능하다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1292" t="inlineStr">
+        <is>
+          <t>대판 2004.5.28. 2003다70041</t>
+        </is>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>제746조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="n">
+        <v>110</v>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>통정허위표시로서 무효인 법률행위도 채권자취소권의 대상이 될 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>허위표시취소</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>판례는 통정허위표시로 무효인 행위라도 사해행위가 되면 채권자취소권의 대상이 된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>대판 1998.2.27. 97다50985</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="n">
+        <v>111</v>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>계약이 해제된 경우, 그 해제로 소멸하는 채권 자체를 양수하거나 그 채권을 압류·전부한 자는 민법 제548조 제1항 단서에서 보호되는 제3자에 해당하지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>해제제3자</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>판례는 해제로 소멸하는 채권의 양수인이나 압류·전부채권자는 제548조 제1항 단서의 제3자가 아니라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1294" t="inlineStr">
+        <is>
+          <t>대판 2003.1.24. 2000다22850</t>
+        </is>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>제548조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="n">
+        <v>112</v>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>계약 해제로 소멸하는 채권을 그 해제 전에 압류·전부한 자도 민법 제548조 제1항 단서의 보호되는 제3자에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>해제제3자</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>해제로 소멸하는 채권 자체를 압류·전부한 자는 제548조 제1항 단서의 제3자에 해당하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1295" t="inlineStr">
+        <is>
+          <t>대판 2000.4.11. 99다51685</t>
+        </is>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>제548조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="n">
+        <v>113</v>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>특정물 매매에서 매수인의 대금지급채무가 이행지체에 빠졌더라도, 그 목적물이 매수인에게 인도될 때까지는 매수인은 매매대금의 이자를 지급할 필요가 없다.</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>대금이자</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>민법 제587조에 따라 목적물 인도 전에는 매수인이 대금 이자를 지급할 의무가 없다.</t>
+        </is>
+      </c>
+      <c r="G1296" t="inlineStr">
+        <is>
+          <t>민법 제587조</t>
+        </is>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>제587조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="n">
+        <v>114</v>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>매매계약 후 아직 인도하지 아니한 목적물로부터 생긴 과실은 원칙적으로 매도인에게 귀속한다.</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>과실귀속</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>민법 제587조 제1문에 따라 인도 전 과실은 원칙적으로 매도인에게 귀속한다.</t>
+        </is>
+      </c>
+      <c r="G1297" t="inlineStr">
+        <is>
+          <t>민법 제587조</t>
+        </is>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>제587조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="n">
+        <v>115</v>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>부동산 이중매매가 반사회적 법률행위에 해당하여 무효인 경우, 제1매수인은 매도인을 대위하여 제2매수인 명의 등기의 말소를 구할 수 있을 뿐 직접 말소를 청구할 수는 없다.</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>이중매매</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>판례는 반사회적 이중매매에서 제1매수인이 매도인을 대위하여 말소를 구할 수 있을 뿐 직접 청구권은 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1298" t="inlineStr">
+        <is>
+          <t>대판 1983.4.26. 83다카57</t>
+        </is>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>제103조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="n">
+        <v>116</v>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>부동산 이중매매가 반사회적 법률행위로서 무효인 경우, 제2매수인으로부터 다시 매수한 선의의 전득자는 유효하게 소유권을 취득한다.</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>절대적무효</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>반사회적 이중매매의 무효는 절대적 무효이므로 선의의 전득자도 보호되지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1299" t="inlineStr">
+        <is>
+          <t>대판 1996.10.25. 96다29151</t>
+        </is>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>제103조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="n">
+        <v>117</v>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>전세권이 소멸한 경우 전세권자의 목적물 인도 및 전세권설정등기 말소에 필요한 서류 교부의무와 전세권설정자의 전세금 반환의무는 동시이행관계에 있다.</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>전세동시이행</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>민법 제317조에 따라 전세권자의 인도·말소서류 교부의무와 전세금 반환의무는 동시이행관계이다.</t>
+        </is>
+      </c>
+      <c r="G1300" t="inlineStr">
+        <is>
+          <t>민법 제317조</t>
+        </is>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>제317조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="n">
+        <v>118</v>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>금전소비대차에서 채권자가 변제를 받기 전 또는 변제와 상환으로 담보된 근저당권설정등기를 말소할 의무는 채무자의 변제의무와 동시이행관계에 있다.</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>담보말소</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>담보권설정등기 말소의무는 피담보채무 변제 후에 이행하는 후이행의무이므로 변제의무와 동시이행관계에 있지 않다.</t>
+        </is>
+      </c>
+      <c r="G1301" t="inlineStr">
+        <is>
+          <t>대판 1969.9.30. 69다1173</t>
+        </is>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>제536조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="n">
+        <v>119</v>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>재판상 이혼청구권은 일신전속적 권리이므로, 이혼소송 계속 중 당사자 일방이 사망하면 그 이혼소송은 종료된다.</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>이혼소송종료</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>판례는 재판상 이혼청구권의 일신전속성을 이유로 일방 사망 시 이혼소송이 종료된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1302" t="inlineStr">
+        <is>
+          <t>대판 1994.10.28. 94므246</t>
+        </is>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>제840조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="n">
+        <v>120</v>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>사실혼관계는 당사자 일방의 의사로 해소할 수 있고, 이 경우 상대방은 재산분할을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>사실혼분할</t>
+        </is>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>판례는 사실혼이 일방의 의사로 해소될 수 있고 그 경우 재산분할청구가 가능하다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1303" t="inlineStr">
+        <is>
+          <t>대판 1995.3.28. 94므1584</t>
+        </is>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>제839조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="n">
+        <v>121</v>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>소유권이전등기가 경료되어 있으면 그 등기는 권리의 귀속과 내용뿐만 아니라 등기원인과 그 절차의 적법까지 추정된다.</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>등기추정력</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>판례는 등기의 추정력이 등기원인과 절차의 적법에까지 미친다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1304" t="inlineStr">
+        <is>
+          <t>대판 2002.2.5. 2001다72029</t>
+        </is>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="n">
+        <v>122</v>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>점유의 추정력은 현재의 점유자뿐만 아니라 전(前) 점유자에게도 원용할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>점유추정력</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>점유의 추정력은 현 점유자에게만 인정되고 전 점유자는 이를 원용할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1305" t="inlineStr">
+        <is>
+          <t>대판 1982.4.13. 81다780</t>
+        </is>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>제200조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="n">
+        <v>123</v>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>나대지에 저당권을 설정한 후 저당권설정자나 제3자가 건물 신축공사를 계속하여 저당부동산의 교환가치 하락으로 우선변제청구권 행사가 방해될 우려가 있는 경우, 저당권자는 방해배제청구권의 행사로 공사중지를 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>방해배제</t>
+        </is>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>판례는 저당목적물의 교환가치를 해치는 행위에 대하여 저당권에 기한 방해배제로 공사중지를 청구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1306" t="inlineStr">
+        <is>
+          <t>대결 2006.1.27. 2003마1755</t>
+        </is>
+      </c>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>제370조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="n">
+        <v>124</v>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>후순위 근저당권자는 민법 제364조의 제3취득자에 해당하므로, 선순위 근저당권의 피담보채무를 변제하고 그 근저당권의 소멸을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>제364조변제</t>
+        </is>
+      </c>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>후순위 근저당권자는 제364조의 제3취득자에 해당하지 않으므로 그에 기한 변제로 선순위 근저당권의 소멸을 청구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1307" t="inlineStr">
+        <is>
+          <t>대판 2006.1.26. 2005다17341</t>
+        </is>
+      </c>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>제364조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="n">
+        <v>125</v>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>청구권보전을 위한 가등기는 본등기 전에는 그 자체로 실체법상 효력이나 순위보전적 효력이 없고, 본등기를 마치면 본등기의 순위가 가등기의 순위로 소급한다.</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>가등기효력</t>
+        </is>
+      </c>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>판례는 가등기는 본등기 전에는 실체법상 효력이 없고 본등기 시 순위만 소급한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1308" t="inlineStr">
+        <is>
+          <t>대판 1981.5.26. 80다3117</t>
+        </is>
+      </c>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="n">
+        <v>126</v>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>가등기에 기하여 본등기를 마치면 순위뿐만 아니라 물권변동의 효력도 가등기를 한 때로 소급하여 발생한다.</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>본등기소급</t>
+        </is>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>본등기를 하면 순위만 가등기 시로 소급할 뿐 물권변동의 효력은 본등기를 한 때에 발생한다.</t>
+        </is>
+      </c>
+      <c r="G1309" t="inlineStr">
+        <is>
+          <t>대판 1982.6.22. 81다1298</t>
+        </is>
+      </c>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="n">
+        <v>127</v>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>가등기에 기한 본등기를 청구할 때 그 상대방은 가등기 당시의 소유자이고, 가등기 후 소유권을 취득한 현재의 등기명의인이 아니다.</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>본등기상대방</t>
+        </is>
+      </c>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>판례는 가등기에 기한 본등기청구의 상대방은 가등기 당시의 소유자라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1310" t="inlineStr">
+        <is>
+          <t>대판 1998.11.27. 97다41103</t>
+        </is>
+      </c>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="n">
+        <v>128</v>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>토지의 공유자 중 소수지분권자가 그 토지에 건물을 신축한 경우, 다른 소수지분권자는 공유물의 보존행위로서 그 건물의 철거와 토지의 인도를 청구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>공유보존행위</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>판례(전합)는 소수지분권자의 무단 점유·사용에 대하여 다른 소수지분권자가 보존행위로 인도·철거를 구할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1311" t="inlineStr">
+        <is>
+          <t>대판(전) 2020.5.21. 2018다287522</t>
+        </is>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>제265조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="n">
+        <v>129</v>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>계약명의신탁에서 매도인이 선의여서 물권변동이 유효한 경우, 명의수탁자가 소유권을 취득하고 명의신탁자는 제공한 매수자금 상당액을 수탁자에게 부당이득으로 반환청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>계약명의신탁</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>판례는 매도인 선의의 계약명의신탁에서 수탁자가 소유권을 취득하고 신탁자는 매수자금의 부당이득반환을 구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1312" t="inlineStr">
+        <is>
+          <t>대판(전) 2005.1.27. 2002다42605</t>
+        </is>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>제103조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="n">
+        <v>130</v>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>계약명의신탁에서 명의신탁자가 부동산을 인도받아 점유하고 있는 경우, 매수자금 상당의 부당이득반환채권을 피담보채권으로 하여 그 부동산에 유치권을 행사할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>명의신탁유치권</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>부당이득반환채권은 목적 부동산과 견련관계가 없으므로 이를 피담보채권으로 한 유치권은 성립하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1313" t="inlineStr">
+        <is>
+          <t>대판 2009.3.26. 2008다34828</t>
+        </is>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>제320조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="n">
+        <v>131</v>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>매매로 인한 소유권이전등기청구권을 양도하는 경우에는 통상의 채권양도와 달리 양도인의 상대방인 채무자의 동의나 승낙이 있어야 양수인이 대항할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>이전등기청구권양도</t>
+        </is>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>판례는 소유권이전등기청구권 양도에는 채무자의 동의나 승낙이 있어야 대항할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1314" t="inlineStr">
+        <is>
+          <t>대판 2001.10.9. 2000다51216</t>
+        </is>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>제449조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="n">
+        <v>132</v>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>중간생략등기의 합의가 있으면 중간매수인의 최초매도인에 대한 소유권이전등기청구권은 소멸한다.</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>중간생략등기</t>
+        </is>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>중간생략등기의 합의가 있더라도 중간매수인의 최초매도인에 대한 등기청구권이 소멸하는 것은 아니다.</t>
+        </is>
+      </c>
+      <c r="G1315" t="inlineStr">
+        <is>
+          <t>대판 1991.12.13. 91다18316</t>
+        </is>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="n">
+        <v>133</v>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>채권의 소멸시효가 완성되면 채무는 당연히 소멸하지만, 이는 변론에서 당사자가 시효의 이익을 주장(원용)하여야 법원이 이를 고려할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>시효원용</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>판례는 소멸시효 완성의 이익은 변론에서 당사자가 원용하여야 재판상 고려된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1316" t="inlineStr">
+        <is>
+          <t>대판 1979.2.13. 78다2157</t>
+        </is>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>제162조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="n">
+        <v>134</v>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>소멸시효의 기산점은 변론주의의 적용대상이지만, 소멸시효의 기간은 법률상의 주장에 불과하여 법원이 직권으로 판단할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>시효기산점</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>판례는 기산점은 주요사실로 변론주의 대상이나, 시효기간은 법률적 판단으로 법원이 직권 판단할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>대판 2008.3.27. 2006다70929</t>
+        </is>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>제166조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="n">
+        <v>135</v>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>채무불이행으로 인한 손해배상액이 예정된 경우, 채권자는 채무불이행 사실만 증명하면 되고 손해의 발생이나 그 손해액을 증명할 필요가 없다.</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>예정액증명</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>판례는 손해배상액 예정 시 채권자는 채무불이행만 증명하면 되고 손해발생·손해액 증명은 불요라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1318" t="inlineStr">
+        <is>
+          <t>대판 2000.12.8. 2000다50350</t>
+        </is>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>제398조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="n">
+        <v>136</v>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>위약금의 약정은 손해배상액의 예정으로 추정된다.</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>위약금추정</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>민법 제398조 제4항에 따라 위약금은 손해배상액의 예정으로 추정된다.</t>
+        </is>
+      </c>
+      <c r="G1319" t="inlineStr">
+        <is>
+          <t>민법 제398조 제4항</t>
+        </is>
+      </c>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>제398조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="n">
+        <v>137</v>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>손해배상액이 예정되어 있는 경우에도 법원은 채권자의 과실을 참작하여 따로 과실상계를 할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>예정과실상계</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>손해배상액이 예정된 경우에는 과실상계를 따로 할 수 없고, 예정액이 부당히 과다하면 직권 감액만 할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1320" t="inlineStr">
+        <is>
+          <t>대판 2002.1.25. 99다57126</t>
+        </is>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>제398조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="n">
+        <v>138</v>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>부진정연대채무자 중 1인이 채권자에 대하여 한 상계는 절대적 효력이 있어, 채무소멸의 효력이 다른 부진정연대채무자에게도 전액 미친다.</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>부진정상계</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>판례는 부진정연대채무에서 변제와 마찬가지로 상계도 절대적 효력이 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1321" t="inlineStr">
+        <is>
+          <t>대판(전) 2010.9.16. 2008다97218</t>
+        </is>
+      </c>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>제418조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="n">
+        <v>139</v>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>피용자와 제3자의 공동불법행위에 대하여 사용자책임이 인정되는 경우, 사용자가 피용자의 부담부분을 초과하여 피해자에게 배상하였다면 사용자는 제3자에게 그 부담부분의 한도에서 구상할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>사용자구상</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>판례는 사용자가 부담부분을 초과 배상하면 다른 공동불법행위자에게 그 부담부분 한도에서 구상할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1322" t="inlineStr">
+        <is>
+          <t>대판 1992.6.23. 91다33070</t>
+        </is>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>제760조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="n">
+        <v>140</v>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>공동불법행위자 중 1인이 피해자의 부주의를 이용하여 고의의 불법행위를 한 경우, 그 가해자도 피해자의 과실을 들어 과실상계를 주장할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>고의과실상계</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>피해자의 부주의를 이용하여 고의의 불법행위를 한 자는 과실상계를 주장할 수 없다(다만 다른 불법행위자는 주장 가능).</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr">
+        <is>
+          <t>대판 2007.6.14. 2005다32999</t>
+        </is>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>제396조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="n">
+        <v>141</v>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>저당권이 설정되어 있는 부동산이 양도된 경우, 피담보채권액이 그 부동산의 가액을 초과하는 때에는 그 양도는 사해행위에 해당하지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>사해행위판단</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>판례는 피담보채권액이 부동산 가액을 초과하면 일반채권자의 공동담보가 없으므로 사해행위가 아니라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1324" t="inlineStr">
+        <is>
+          <t>대판 2001.10.9. 2000다42618</t>
+        </is>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="n">
+        <v>142</v>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>사해행위취소소송에서 채무자의 사해의사는 채권자가 증명하여야 하나, 채무자가 유일한 재산을 처분한 경우에는 그 사해의사가 추정된다.</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>사해의사추정</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>판례는 채무자가 유일재산을 처분한 경우 사해의사가 추정된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1325" t="inlineStr">
+        <is>
+          <t>대판 2001.4.24. 2000다41875</t>
+        </is>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="n">
+        <v>143</v>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>토지임차인의 지상물매수청구권에 관한 민법 제643조는 편면적 강행규정이므로, 이를 미리 포기하는 특약은 원칙적으로 무효이다.</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>지상물매수</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>판례는 제643조가 편면적 강행규정이어서 임차인에게 불리한 포기 특약은 무효라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1326" t="inlineStr">
+        <is>
+          <t>민법 제652조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>제643조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="n">
+        <v>144</v>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>토지임대인이 제기한 건물철거 및 토지인도 청구소송에서 임차인이 패소하여 확정된 경우, 그 후 건물철거가 집행되지 않았더라도 임차인은 더 이상 지상물매수청구권을 행사할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>매수청구기판력</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>판례는 패소 확정 후라도 건물철거가 집행되지 않은 이상 임차인은 별소로 건물매수청구권을 행사하여 매매대금을 청구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>대판 1995.12.26. 95다42195</t>
+        </is>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>제643조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="n">
+        <v>145</v>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>채권자대위소송에서 제3채무자는 채무자에 대하여 가지는 항변으로 채권자에게 대항할 수 있으나, 피보전채권의 소멸시효 완성은 채무자가 채권자에게 가지는 항변이므로 제3채무자가 이를 원용할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>제3채무자항변</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>판례는 피보전채권의 소멸시효 완성은 채무자의 항변이어서 제3채무자가 원용할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>대판 1992.11.10. 92다35899</t>
+        </is>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>제404조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="n">
+        <v>146</v>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>자기 소유 주택을 매도하고 그 주택에 임차인으로 계속 거주하는 경우, 임차인으로서의 대항력은 매수인 명의의 소유권이전등기가 마쳐진 다음 날에 취득한다.</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>대항력시기</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>판례는 매도 후 임차인으로 남은 경우 매수인 명의 이전등기 익일에 대항력을 취득한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1329" t="inlineStr">
+        <is>
+          <t>대판 2000.2.11. 99다59306</t>
+        </is>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>제3조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="n">
+        <v>147</v>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>대항요건과 확정일자를 갖춘 임차인이라도 경매절차에서 우선변제를 받으려면 배당요구의 종기까지 배당요구를 하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>배당요구</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>판례는 우선변제권 있는 임차인도 배당요구를 하여야 배당받을 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1330" t="inlineStr">
+        <is>
+          <t>대판 1998.10.13. 98다12379</t>
+        </is>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>제3조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="n">
+        <v>148</v>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>임시이사의 선임에 관한 민법 제63조는 비법인사단에도 유추적용된다.</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>비법인사단</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>판례는 제63조의 임시이사 선임 규정이 비법인사단에 유추적용된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1331" t="inlineStr">
+        <is>
+          <t>대결(전) 2009.11.19. 2008마699</t>
+        </is>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>제63조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="n">
+        <v>149</v>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>지교회가 교단을 탈퇴하거나 변경하려면 의결권을 가진 교인 과반수의 찬성으로 충분하다.</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>교단탈퇴</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>판례는 지교회의 교단 탈퇴·변경에는 의결권을 가진 교인 3분의 2 이상의 찬성이 필요하다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1332" t="inlineStr">
+        <is>
+          <t>대판(전) 2006.4.20. 2004다37775</t>
+        </is>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>제42조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="n">
+        <v>150</v>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>가등기담보법상 가등기담보의 사적 실행은 귀속정산의 방법만 인정되고, 청산절차 없이 목적물을 처분하는 처분정산형의 담보권 실행은 허용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>가등기담보실행</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>가등기담보법은 사적 실행으로 귀속정산만 인정하고 처분정산형 실행을 허용하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1333" t="inlineStr">
+        <is>
+          <t>가등기담보법 제3조·제4조</t>
+        </is>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>제607조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="n">
+        <v>151</v>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>가등기담보법은 목적물의 예약 당시 가액이 차용액 및 이에 붙인 이자의 합산액을 초과하는 경우에만 적용된다.</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>가등기담보적용</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>판례는 예약 당시 목적물 가액이 차용원리금을 초과하는 경우에만 가등기담보법이 적용된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1334" t="inlineStr">
+        <is>
+          <t>대판 2006.8.24. 2005다61140</t>
+        </is>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>제608조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="n">
+        <v>152</v>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>타인 소유의 토지 위에 권한 없이 건물을 소유하는 자는 그 건물을 실제로 사용·수익하지 않더라도 토지의 차임 상당액을 부당이득으로 반환할 의무가 있다.</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>무단건물소유</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>판례는 권한 없이 건물을 소유하여 토지를 점유하는 자는 사용·수익 여부와 무관하게 차임 상당 부당이득반환의무가 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1335" t="inlineStr">
+        <is>
+          <t>대판 1998.5.8. 98다2389</t>
+        </is>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="n">
+        <v>153</v>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>점유취득시효가 완성되었으나 아직 소유권이전등기를 마치지 못한 점유자에 대하여, 대지소유자는 그 점유가 불법점유임을 이유로 차임 상당의 부당이득반환을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>시효완성점유</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>시효완성자의 점유는 권원 있는 점유로 보아야 하므로 소유자는 불법점유를 이유로 부당이득반환을 청구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1336" t="inlineStr">
+        <is>
+          <t>대판 1993.5.25. 92다51280</t>
+        </is>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="n">
+        <v>154</v>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>취득시효가 완성된 점유자가 그 후 점유를 상실하더라도 소유권이전등기청구권이 즉시 소멸하는 것은 아니나, 그때부터 소멸시효가 진행하여 10년이 지나면 소멸한다.</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>점유상실</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>판례는 시효완성 후 점유를 상실해도 등기청구권이 곧바로 소멸하지 않고 다만 소멸시효가 진행한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1337" t="inlineStr">
+        <is>
+          <t>대판(전) 1996.3.8. 95다34866</t>
+        </is>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>제245조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="n">
+        <v>155</v>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>점유취득시효가 완성된 사실을 알 수 없었던 부동산 소유자가 시효완성자가 시효를 주장하거나 이전등기를 청구하기 전에 그 부동산을 제3자에게 처분한 경우, 소유자는 시효완성자에 대하여 손해배상책임을 진다.</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>시효처분책임</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>시효완성 사실을 알 수 없는 소유자가 시효 주장 전에 처분한 경우에는 특별한 사정이 없는 한 손해배상책임을 지지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1338" t="inlineStr">
+        <is>
+          <t>대판 1995.7.11. 94다4509</t>
+        </is>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>제245조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="n">
+        <v>156</v>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>채권이 이중으로 양도된 경우 양수인 상호간의 우열은 확정일자 있는 양도통지가 채무자에게 도달한 일시의 선후로 결정되며, 확정일자 자체의 선후로 결정되는 것이 아니다.</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>채권이중양도</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>판례는 이중양도 시 우열을 확정일자 있는 통지의 도달 선후로 결정한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1339" t="inlineStr">
+        <is>
+          <t>대판(전) 1994.4.26. 93다24223</t>
+        </is>
+      </c>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>제450조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="n">
+        <v>157</v>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>확정일자 있는 채권양도통지와 압류명령 등이 제3채무자에게 동시에 도달하여 그들 상호간에 우열이 없는 경우, 제3채무자가 그중 한 사람에게 채무 전액을 변제하면 다른 채권자에 대한 관계에서도 유효하게 면책된다.</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>동시도달</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>판례는 동시도달로 우열이 없는 경우 채무자가 한 채권자에게 전액 변제하면 다른 채권자에 대하여도 면책된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1340" t="inlineStr">
+        <is>
+          <t>대판 1994.4.26. 93다24223</t>
+        </is>
+      </c>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>제450조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="n">
+        <v>158</v>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>특별손해는 채무자가 그 특별한 사정을 알았거나 알 수 있었을 때에만 배상책임이 인정된다.</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>특별손해</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>민법 제393조 제2항에 따라 특별손해는 채무자가 그 사정을 알았거나 알 수 있었을 때 배상책임이 있다.</t>
+        </is>
+      </c>
+      <c r="G1341" t="inlineStr">
+        <is>
+          <t>민법 제393조 제2항</t>
+        </is>
+      </c>
+      <c r="H1341" t="inlineStr">
+        <is>
+          <t>제393조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="n">
+        <v>159</v>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>채권자가 연대보증인 1인에 대하여 채권을 포기하더라도 그 효력은 주채무자나 다른 연대보증인에게 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>연대보증포기</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>판례는 연대보증인 1인에 대한 채권포기는 상대적 효력만 있어 주채무자·다른 보증인에게 미치지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>민법 제419조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1342" t="inlineStr">
+        <is>
+          <t>제419조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="n">
+        <v>160</v>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>주채무자에 대한 시효중단의 효력은 보증채무에는 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>보증시효중단</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>민법 제440조에 따라 주채무자에 대한 시효중단은 보증채무에도 효력이 미친다(반면 보증채무의 시효중단은 주채무에 영향 없음).</t>
+        </is>
+      </c>
+      <c r="G1343" t="inlineStr">
+        <is>
+          <t>민법 제440조</t>
+        </is>
+      </c>
+      <c r="H1343" t="inlineStr">
+        <is>
+          <t>제440조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="n">
+        <v>161</v>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>전세권의 존속기간이 만료되면 용익물권적 권능은 전세권설정등기의 말소 없이도 당연히 소멸하나, 담보물권적 권능은 전세금이 반환될 때까지 존속한다.</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>전세권존속</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>판례는 존속기간 만료로 용익권능은 소멸하고 담보물권적 권능만 전세금 반환 시까지 존속한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1344" t="inlineStr">
+        <is>
+          <t>대판 2005.3.25. 2003다35659</t>
+        </is>
+      </c>
+      <c r="H1344" t="inlineStr">
+        <is>
+          <t>제303조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="n">
+        <v>162</v>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>유증은 유언자의 사망 전에 수증자가 먼저 사망한 때에는 그 효력이 생기지 않으며, 이는 사인증여의 경우에도 같다.</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>유증실효</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>민법 제1089조에 따라 수증자가 유언자보다 먼저 사망하면 유증은 효력이 없고 사인증여도 같다.</t>
+        </is>
+      </c>
+      <c r="G1345" t="inlineStr">
+        <is>
+          <t>민법 제1089조</t>
+        </is>
+      </c>
+      <c r="H1345" t="inlineStr">
+        <is>
+          <t>제1089조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="n">
+        <v>163</v>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>증여와 유증이 함께 유류분을 침해하는 경우, 유류분 권리자는 유증(사인증여)을 먼저 반환받은 후 그것으로 부족할 때 증여를 반환받는다.</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>유류분반환순서</t>
+        </is>
+      </c>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>민법 제1116조에 따라 유류분 반환은 유증을 먼저, 그 다음 증여의 순서로 한다.</t>
+        </is>
+      </c>
+      <c r="G1346" t="inlineStr">
+        <is>
+          <t>민법 제1116조</t>
+        </is>
+      </c>
+      <c r="H1346" t="inlineStr">
+        <is>
+          <t>제1116조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="n">
+        <v>164</v>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>변제할 정당한 이익이 있는 제3자는 채무자의 의사에 반하여도 변제할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>이해관계변제</t>
+        </is>
+      </c>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>민법 제469조 제2항에 따라 이해관계 있는 제3자는 채무자의 의사에 반하여도 변제할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1347" t="inlineStr">
+        <is>
+          <t>민법 제469조</t>
+        </is>
+      </c>
+      <c r="H1347" t="inlineStr">
+        <is>
+          <t>제469조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="n">
+        <v>165</v>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>채권의 일부를 대위변제한 경우, 그 일부 대위변제자는 채권자와 함께 권리를 행사하며 채권자에 우선하여 변제받는다.</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>일부대위우선</t>
+        </is>
+      </c>
+      <c r="F1348" t="inlineStr">
+        <is>
+          <t>일부 대위변제 시 대위자는 채권자와 함께 권리를 행사하나, 채권자가 일부 대위변제자에 우선하여 변제받는다.</t>
+        </is>
+      </c>
+      <c r="G1348" t="inlineStr">
+        <is>
+          <t>대판 1988.9.27. 88다카1797</t>
+        </is>
+      </c>
+      <c r="H1348" t="inlineStr">
+        <is>
+          <t>제483조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="n">
+        <v>166</v>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>보증인과 물상보증인의 지위를 함께 가지는 자는 변제자대위의 비율을 산정할 때 1인으로 보아 인원수에 산입한다.</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>이중자격대위</t>
+        </is>
+      </c>
+      <c r="F1349" t="inlineStr">
+        <is>
+          <t>판례는 보증인과 물상보증인의 지위를 겸하는 자는 대위비율 산정 시 1인으로 보아야 한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1349" t="inlineStr">
+        <is>
+          <t>대판(전) 2010.6.17. 2007다61113</t>
+        </is>
+      </c>
+      <c r="H1349" t="inlineStr">
+        <is>
+          <t>제482조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="n">
+        <v>167</v>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>혼인 중 부부 일방이 사망하여 상대방이 배우자로서 망인의 재산을 상속받은 후 그 혼인이 취소된 경우, 취소의 소급효로 인하여 상속받은 재산은 부당이득으로 반환하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>혼인취소비소급</t>
+        </is>
+      </c>
+      <c r="F1350" t="inlineStr">
+        <is>
+          <t>혼인의 취소에는 소급효가 없으므로(제824조), 취소 전에 배우자로서 상속받은 재산을 부당이득으로 반환할 의무는 없다.</t>
+        </is>
+      </c>
+      <c r="G1350" t="inlineStr">
+        <is>
+          <t>민법 제824조</t>
+        </is>
+      </c>
+      <c r="H1350" t="inlineStr">
+        <is>
+          <t>제824조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="n">
+        <v>168</v>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>쌍무계약이 취소된 경우, 선의의 매도인은 그가 받은 매매대금의 운용이익 내지 법정이자를 상대방에게 반환하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>선의반환범위</t>
+        </is>
+      </c>
+      <c r="F1351" t="inlineStr">
+        <is>
+          <t>판례는 쌍무계약 취소 시 선의의 매도인은 받은 대금의 운용이익이나 법정이자까지 반환할 의무는 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1351" t="inlineStr">
+        <is>
+          <t>대판 1993.5.14. 92다45025</t>
+        </is>
+      </c>
+      <c r="H1351" t="inlineStr">
+        <is>
+          <t>제748조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="n">
+        <v>169</v>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>가등기담보법이 적용되는 담보가등기의 피담보채권에는 소비대차에 의한 차용물반환채권뿐만 아니라 매매대금채권이나 공사대금채권도 포함된다.</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>담보가등기피담보</t>
+        </is>
+      </c>
+      <c r="F1352" t="inlineStr">
+        <is>
+          <t>가등기담보법은 소비대차(준소비대차 포함)에 기한 차용물반환채권에만 적용되므로 매매대금·공사대금채권을 담보하는 가등기에는 적용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1352" t="inlineStr">
+        <is>
+          <t>가등기담보법 제1조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1352" t="inlineStr">
+        <is>
+          <t>제607조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="n">
+        <v>170</v>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>채권에 대한 가압류가 있으면 제3채무자와 채무자는 그 채권의 발생원인인 계약을 합의해제할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>가압류합의해제</t>
+        </is>
+      </c>
+      <c r="F1353" t="inlineStr">
+        <is>
+          <t>가압류는 채권 자체를 대상으로 할 뿐 그 발생원인인 법률관계를 구속하지 않으므로, 제3채무자와 채무자는 그 계약을 합의해제할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1353" t="inlineStr">
+        <is>
+          <t>대판 2001.6.1. 98다17930</t>
+        </is>
+      </c>
+      <c r="H1353" t="inlineStr">
+        <is>
+          <t>제449조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="n">
+        <v>171</v>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>사해행위취소권을 행사하려면 채무자의 무자력 상태가 사해행위 당시에 존재하면 충분하고, 사실심 변론종결 시까지 계속될 필요는 없다.</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>무자력계속</t>
+        </is>
+      </c>
+      <c r="F1354" t="inlineStr">
+        <is>
+          <t>판례는 채무자의 무자력이 사해행위 시부터 사실심 변론종결 시까지 계속되어야 사해행위취소가 인정된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1354" t="inlineStr">
+        <is>
+          <t>대판 2009.3.26. 2007다63102</t>
+        </is>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="n">
+        <v>172</v>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>변시1</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>매도인에게 소유권이 유보된 자재가 제3자와 매수인 사이의 도급계약 이행으로 제3자 소유 건물에 부합된 경우, 그 제3자가 소유권 유보에 대하여 선의·무과실이더라도 매도인은 제3자에게 부당이득반환을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>부합부당이득</t>
+        </is>
+      </c>
+      <c r="F1355" t="inlineStr">
+        <is>
+          <t>제3자가 소유권 유보에 대하여 선의·무과실이면 선의취득에 준하여 법률상 원인이 있으므로, 매도인은 그 제3자에게 부당이득반환을 청구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1355" t="inlineStr">
+        <is>
+          <t>대판 2009.9.24. 2009다15602</t>
+        </is>
+      </c>
+      <c r="H1355" t="inlineStr">
+        <is>
+          <t>제261조</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 변시15 OX self-solved (1429 items)
</commit_message>
<xml_diff>
--- a/assets/ox_civil_bar14.xlsx
+++ b/assets/ox_civil_bar14.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1355"/>
+  <dimension ref="A1:H1430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -54664,6 +54664,3006 @@
         </is>
       </c>
     </row>
+    <row r="1356">
+      <c r="A1356" t="n">
+        <v>1501</v>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>타인의 성명을 모용한 자가 명의자 본인인 것처럼 상대방을 기망하여 직접 법률행위를 한 경우, 모용자에게 명의자를 대리할 기본대리권이 있었고 상대방이 명의자 본인의 권한 행사로 믿은 데 정당한 사유가 있었다면 민법 제126조의 표현대리 법리가 유추적용된다.</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>문1·성명모용</t>
+        </is>
+      </c>
+      <c r="F1356" t="inlineStr">
+        <is>
+          <t>판례는 성명모용에 기본대리권과 정당한 사유가 있으면 제126조 표현대리를 유추적용한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1356" t="inlineStr">
+        <is>
+          <t>대판 1993.2.23. 92다52436</t>
+        </is>
+      </c>
+      <c r="H1356" t="inlineStr">
+        <is>
+          <t>제126조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="n">
+        <v>1502</v>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>비법인사단인 교회의 대표자가 총유물인 교회 재산 처분에 관하여 교인총회 결의를 거치지 않아 권한이 없는 경우에도, 상대방이 대표자에게 권한이 있다고 믿을 정당한 이유가 있으면 민법 제126조의 표현대리 법리가 유추적용된다.</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>문1·총유처분</t>
+        </is>
+      </c>
+      <c r="F1357" t="inlineStr">
+        <is>
+          <t>총유물 처분에 사원총회 결의가 없으면 대표권 자체가 없어 제126조 표현대리 법리가 유추적용되지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1357" t="inlineStr">
+        <is>
+          <t>대판(전) 2009.2.12. 2006다23312</t>
+        </is>
+      </c>
+      <c r="H1357" t="inlineStr">
+        <is>
+          <t>제276조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="n">
+        <v>1503</v>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>어떤 사람이 대리인의 외양을 갖추고 행위하는 것을 본인이 알면서도 이의하지 않고 방임하는 등 사실상의 태도에 의하여도 대리권 수여가 추단될 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>문1·묵시수권</t>
+        </is>
+      </c>
+      <c r="F1358" t="inlineStr">
+        <is>
+          <t>판례는 본인이 대리행위를 알면서 방임하는 태도로도 묵시적 대리권 수여가 추단될 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1358" t="inlineStr">
+        <is>
+          <t>대판 1962.4.18. 4294민상1236</t>
+        </is>
+      </c>
+      <c r="H1358" t="inlineStr">
+        <is>
+          <t>제125조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="n">
+        <v>1504</v>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>타인 소유 토지 위에 무단으로 신축된 미등기건물을 매수하여 대금을 완납하고 이를 배타적으로 점유·사용하는 자는, 그 부지인 토지의 점유·사용으로 인한 부당이득을 토지소유자에게 반환할 의무가 있다.</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>문2·미등기건물</t>
+        </is>
+      </c>
+      <c r="F1359" t="inlineStr">
+        <is>
+          <t>판례는 미등기건물의 매수인을 사실상 처분권자로서 부지의 점유자로 보아 부당이득반환의무를 인정한다.</t>
+        </is>
+      </c>
+      <c r="G1359" t="inlineStr">
+        <is>
+          <t>대판 2022.9.29. 2018다243133</t>
+        </is>
+      </c>
+      <c r="H1359" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="n">
+        <v>1505</v>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>무단으로 신축된 미등기건물을 매수하여 점유하는 자는 아직 소유권이전등기를 마치지 못한 이상 그 건물에 대하여 소유권은 물론 소유권에 준하는 관습상의 물권도 인정받을 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>문2·관습물권</t>
+        </is>
+      </c>
+      <c r="F1360" t="inlineStr">
+        <is>
+          <t>판례는 미등기건물 매수인에게 소유권이나 소유권에 준하는 관습상 물권을 인정하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1360" t="inlineStr">
+        <is>
+          <t>대판(전) 2006.10.27. 2006다49000</t>
+        </is>
+      </c>
+      <c r="H1360" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="n">
+        <v>1506</v>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>법인 대표자의 직무에 관한 불법행위로 법인의 손해배상책임이 인정되고 그 행위가 피해자에 대한 불법행위를 구성하는 경우, 이에 가담한 사원은 피해자에 대하여 대표자와 연대하여 손해배상책임을 진다.</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>문3·공동불법행위</t>
+        </is>
+      </c>
+      <c r="F1361" t="inlineStr">
+        <is>
+          <t>가담한 사원은 공동불법행위자로서 대표자와 연대하여 책임을 진다.</t>
+        </is>
+      </c>
+      <c r="G1361" t="inlineStr">
+        <is>
+          <t>민법 제760조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1361" t="inlineStr">
+        <is>
+          <t>제760조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="n">
+        <v>1507</v>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>피해자가 법인 대표자의 행위가 직무에 관한 것이 아님을 알았거나 중대한 과실로 알지 못한 경우에는 법인에 대하여 손해배상책임을 물을 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>문3·외형이론</t>
+        </is>
+      </c>
+      <c r="F1362" t="inlineStr">
+        <is>
+          <t>판례는 피해자가 직무 외 행위임을 알았거나 중과실로 몰랐으면 법인 책임을 부정한다.</t>
+        </is>
+      </c>
+      <c r="G1362" t="inlineStr">
+        <is>
+          <t>대판 2004.3.26. 2003다34045</t>
+        </is>
+      </c>
+      <c r="H1362" t="inlineStr">
+        <is>
+          <t>제35조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="n">
+        <v>1508</v>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>행위의 외형상 법인 대표자의 직무행위라고 인정될 수 있는 것이라면, 대표자 개인의 사리를 도모하기 위한 것이거나 법령에 위배된 것이더라도 민법 제35조 제1항의 직무에 관한 행위에 해당한다.</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>문3·직무관련성</t>
+        </is>
+      </c>
+      <c r="F1363" t="inlineStr">
+        <is>
+          <t>판례는 외형상 직무행위로 보이면 사리도모·법령위배라도 직무관련성을 인정한다.</t>
+        </is>
+      </c>
+      <c r="G1363" t="inlineStr">
+        <is>
+          <t>대판 2004.2.27. 2003다15280</t>
+        </is>
+      </c>
+      <c r="H1363" t="inlineStr">
+        <is>
+          <t>제35조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="n">
+        <v>1509</v>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>재개발조합 대표기관의 직무상 불법행위로 조합이 과다한 채무를 부담하여 조합원의 경제적 이익이 침해된 경우, 그 조합원의 간접적인 손해는 민법 제35조에서 말하는 손해의 개념에 포함되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>문3·간접손해</t>
+        </is>
+      </c>
+      <c r="F1364" t="inlineStr">
+        <is>
+          <t>판례는 조합원이 입은 간접손해는 제35조의 손해에 포함되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1364" t="inlineStr">
+        <is>
+          <t>대판 1999.7.27. 99다19384</t>
+        </is>
+      </c>
+      <c r="H1364" t="inlineStr">
+        <is>
+          <t>제35조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="n">
+        <v>1510</v>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>장래에 발생할 막연한 사정을 예측·기대하고 법률행위를 한 경우 그 예측과 다른 사정이 발생하였더라도, 그로 인한 위험은 원칙적으로 행위자가 스스로 감수하여야 하므로 착오를 이유로 취소할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>문4·장래예측착오</t>
+        </is>
+      </c>
+      <c r="F1365" t="inlineStr">
+        <is>
+          <t>판례는 장래의 불확실한 사정에 대한 예측 착오의 위험은 원칙적으로 행위자가 부담한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1365" t="inlineStr">
+        <is>
+          <t>대판 2010.5.27. 2009다94841</t>
+        </is>
+      </c>
+      <c r="H1365" t="inlineStr">
+        <is>
+          <t>제109조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="n">
+        <v>1511</v>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>표의자에게 중대한 과실이 있어 착오에 빠졌더라도 상대방이 표의자의 착오를 알면서 이를 이용한 경우에는, 표의자는 착오를 이유로 의사표시를 취소할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>문4·중과실예외</t>
+        </is>
+      </c>
+      <c r="F1366" t="inlineStr">
+        <is>
+          <t>판례는 상대방이 표의자의 착오를 알고 이용한 경우에는 표의자의 중과실에도 불구하고 취소를 인정한다.</t>
+        </is>
+      </c>
+      <c r="G1366" t="inlineStr">
+        <is>
+          <t>대판 2014.11.27. 2013다49794</t>
+        </is>
+      </c>
+      <c r="H1366" t="inlineStr">
+        <is>
+          <t>제109조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="n">
+        <v>1512</v>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>보험회사의 설명의무 위반으로 고객이 계약의 중요 사항을 이해하지 못한 채 착오에 빠져 계약을 체결한 경우, 그 착오가 동기의 착오라도 그것이 없었다면 계약을 체결하지 않았을 것이 명백하면 중요 부분의 착오로서 취소할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr">
+        <is>
+          <t>문4·동기착오</t>
+        </is>
+      </c>
+      <c r="F1367" t="inlineStr">
+        <is>
+          <t>판례는 설명의무 위반으로 유발된 동기 착오도 중요 부분에 해당하면 취소를 인정한다.</t>
+        </is>
+      </c>
+      <c r="G1367" t="inlineStr">
+        <is>
+          <t>대판 2018.4.12. 2017다229536</t>
+        </is>
+      </c>
+      <c r="H1367" t="inlineStr">
+        <is>
+          <t>제109조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="n">
+        <v>1513</v>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>통정허위표시로 매매하고 등기를 마쳐 준 후, 그 사실을 과실로 알지 못한 채 목적물을 다시 매수하여 등기를 마친 자에 대하여, 매도인은 통정허위표시임을 이유로 대항할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>문5·허위표시제3자</t>
+        </is>
+      </c>
+      <c r="F1368" t="inlineStr">
+        <is>
+          <t>민법 제108조 제2항의 선의의 제3자는 과실이 있어도 보호되므로, 과실로 모른 선의의 제3자에게는 통정허위표시의 무효로 대항할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1368" t="inlineStr">
+        <is>
+          <t>민법 제108조 제2항</t>
+        </is>
+      </c>
+      <c r="H1368" t="inlineStr">
+        <is>
+          <t>제108조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="n">
+        <v>1514</v>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>매매목적물의 하자가 계약 내용의 중요 부분에 해당하여 하자담보책임으로 계약을 해제하거나 손해배상을 청구할 수 있는 경우, 매수인은 착오를 이유로는 그 매매계약을 취소할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>문5·담보책임착오경합</t>
+        </is>
+      </c>
+      <c r="F1369" t="inlineStr">
+        <is>
+          <t>판례는 하자담보책임과 착오취소는 경합할 수 있으므로, 담보책임을 물을 수 있는 경우에도 착오를 이유로 취소할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1369" t="inlineStr">
+        <is>
+          <t>대판 2018.9.13. 2015다78703</t>
+        </is>
+      </c>
+      <c r="H1369" t="inlineStr">
+        <is>
+          <t>제109조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="n">
+        <v>1515</v>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>경제적·사실적으로 일체로 체결된 임차권양도계약과 권리금계약에서 당사자가 어느 한 계약 없이는 다른 계약을 의욕하지 않았을 것으로 보이는 경우, 권리금계약을 기망을 이유로 취소하면 임차권양도계약에도 취소의 효력이 미친다.</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>문5·일체계약취소</t>
+        </is>
+      </c>
+      <c r="F1370" t="inlineStr">
+        <is>
+          <t>판례는 불가분적으로 결합된 계약 중 하나의 취소가 전체에 미친다고 본다.</t>
+        </is>
+      </c>
+      <c r="G1370" t="inlineStr">
+        <is>
+          <t>대판 2013.5.9. 2012다115120</t>
+        </is>
+      </c>
+      <c r="H1370" t="inlineStr">
+        <is>
+          <t>제137조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="n">
+        <v>1516</v>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>사기로 매도하고 등기를 마쳐 준 후 그로부터 목적물을 매수하여 등기한 제3자에게 사기 취소의 효과를 주장하는 경우, 그 제3자의 악의에 대한 증명책임은 취소를 주장하는 자에게 있다.</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>문5·제3자악의입증</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>제110조 제3항의 제3자는 선의로 추정되므로 악의의 증명책임은 취소를 주장하는 자가 진다.</t>
+        </is>
+      </c>
+      <c r="G1371" t="inlineStr">
+        <is>
+          <t>민법 제110조 제3항 · 판례</t>
+        </is>
+      </c>
+      <c r="H1371" t="inlineStr">
+        <is>
+          <t>제110조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="n">
+        <v>1517</v>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>동일한 채권자와 채무자 사이에 시효가 완성되지 않은 다수의 금전채무가 있고 채무자가 충당할 채무를 지정하지 않은 채 전부를 변제하기에 부족한 금액을 변제한 경우, 특별한 사정이 없는 한 그 변제는 모든 채무에 대한 승인으로서 시효중단의 효력이 있다.</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>문6·일부변제승인</t>
+        </is>
+      </c>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>판례는 충당 지정 없는 일부 변제는 다수 채무 전부에 대한 승인으로 시효를 중단시킨다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1372" t="inlineStr">
+        <is>
+          <t>대판 2021.9.30. 2021다239745</t>
+        </is>
+      </c>
+      <c r="H1372" t="inlineStr">
+        <is>
+          <t>제168조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="n">
+        <v>1518</v>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>후순위 담보권자는 선순위 담보권의 피담보채권이 소멸하면 순위 상승과 배당액 증가의 이익을 얻으므로, 선순위 담보권의 피담보채권에 관한 소멸시효의 완성을 주장(원용)할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>문6·후순위시효원용</t>
+        </is>
+      </c>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>판례는 후순위 담보권자는 순위 상승의 이익이 반사적 이익에 불과하여 선순위 피담보채권의 소멸시효를 원용할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1373" t="inlineStr">
+        <is>
+          <t>대판 2021.2.25. 2016다232597</t>
+        </is>
+      </c>
+      <c r="H1373" t="inlineStr">
+        <is>
+          <t>제162조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="n">
+        <v>1519</v>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>매매계약의 무효를 원인으로 한 매매대금 상당의 부당이득반환청구권은 특별한 사정이 없는 한 매매대금을 지급한 때부터 소멸시효가 진행한다.</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>문6·부당이득시효</t>
+        </is>
+      </c>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>부당이득반환청구권은 성립과 동시에 행사할 수 있으므로 급부(대금 지급) 시부터 시효가 진행한다.</t>
+        </is>
+      </c>
+      <c r="G1374" t="inlineStr">
+        <is>
+          <t>대판 1993.9.14. 93다17324 · 판례</t>
+        </is>
+      </c>
+      <c r="H1374" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="n">
+        <v>1520</v>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>매도인이 선의인 계약명의신탁에서 신탁자가 수탁자에게 자금을 제공한 경우, 신탁자는 목적물의 소유권을 취득하지 못하고 수탁자에게 제공한 매수자금 상당액의 부당이득반환을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>문7·계약명의신탁</t>
+        </is>
+      </c>
+      <c r="F1375" t="inlineStr">
+        <is>
+          <t>판례는 매도인 선의의 계약명의신탁에서 수탁자가 소유권을 취득하고 신탁자는 매수자금의 부당이득반환을 구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1375" t="inlineStr">
+        <is>
+          <t>대판(전) 2005.1.27. 2002다42605</t>
+        </is>
+      </c>
+      <c r="H1375" t="inlineStr">
+        <is>
+          <t>제103조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="n">
+        <v>1521</v>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>매도인이 선의인 계약명의신탁에서, 매도인이 매매계약 당시 명의신탁약정을 알았다면(악의) 명의신탁자는 매도인에게 직접 소유권이전등기절차의 이행을 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>문7·매도인악의</t>
+        </is>
+      </c>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>매도인이 악의이면 수탁자 명의 물권변동이 무효여서 소유권은 매도인에게 남고, 매매계약 당사자가 아닌 신탁자는 매도인에게 이전등기를 청구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1376" t="inlineStr">
+        <is>
+          <t>부동산실명법 제4조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1376" t="inlineStr">
+        <is>
+          <t>제103조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="n">
+        <v>1522</v>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>매도인이 선의인 계약명의신탁에서 수탁자가 목적물을 제3자에게 매도하고 받은 대금 중 일부를 또 다른 제3자에게 지급한 경우, 그 금원을 받은 제3자는 명의신탁자에게 이를 부당이득으로 반환할 의무가 있다.</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>문7·제3자부당이득</t>
+        </is>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>수탁자로부터 금원을 받은 제3자는 신탁자와 사이에 아무런 법률관계가 없으므로 신탁자에게 부당이득반환의무를 지지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1377" t="inlineStr">
+        <is>
+          <t>민법 제741조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1377" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="n">
+        <v>1523</v>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>선순위 근저당권과 후순위 근저당권, 그 후 가압류등기들이 차례로 마쳐진 부동산을 후순위 근저당권자가 매수하여 소유권을 취득한 경우, 그 후순위 근저당권은 혼동으로 소멸한다.</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>문8·혼동근저당</t>
+        </is>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>후순위 근저당권자가 소유권을 취득해도 그 근저당권이 제3자(중간 가압류 등)의 권리의 목적이 되어 존속시킬 이익이 있으므로 혼동으로 소멸하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1378" t="inlineStr">
+        <is>
+          <t>민법 제191조 제1항 단서</t>
+        </is>
+      </c>
+      <c r="H1378" t="inlineStr">
+        <is>
+          <t>제191조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="n">
+        <v>1524</v>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>토지를 점유하던 자가 그 토지의 소유권을 취득한 경우, 그의 점유권은 혼동으로 소멸한다.</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>문8·점유권혼동</t>
+        </is>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>민법 제191조 제3항에 따라 점유권에는 혼동에 관한 규정이 적용되지 않으므로 점유권은 혼동으로 소멸하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1379" t="inlineStr">
+        <is>
+          <t>민법 제191조 제3항</t>
+        </is>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>제191조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="n">
+        <v>1525</v>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>주택임대차보호법상 대항력과 우선변제권을 갖춘 임차인이 그 후 설정된 저당권에 앞서는 지위에 있는 상태에서 임차주택의 소유권을 취득한 경우, 그 임차권은 혼동으로 소멸한다.</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>문8·임차권혼동</t>
+        </is>
+      </c>
+      <c r="F1380" t="inlineStr">
+        <is>
+          <t>대항력·우선변제권 있는 임차권을 존속시킬 법률상 이익이 있는 경우에는 소유권 취득에도 임차권이 혼동으로 소멸하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1380" t="inlineStr">
+        <is>
+          <t>대판 2001.5.15. 2000다12693</t>
+        </is>
+      </c>
+      <c r="H1380" t="inlineStr">
+        <is>
+          <t>제191조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="n">
+        <v>1526</v>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>부동산이 전전 양도된 경우 적법한 원인행위에 기하여 일단 최종 양수인 명의로 중간생략등기가 이루어졌다면, 중간생략등기에 관한 합의가 없었다는 이유만으로는 그 등기가 무효가 되지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>문9·중간생략등기</t>
+        </is>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>판례는 실체관계에 부합하는 중간생략등기는 합의가 없었다는 사유만으로 무효가 되지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1381" t="inlineStr">
+        <is>
+          <t>대판 2005.9.29. 2003다40651</t>
+        </is>
+      </c>
+      <c r="H1381" t="inlineStr">
+        <is>
+          <t>제186조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="n">
+        <v>1527</v>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>채무자 소유 부동산과 물상보증인 소유 부동산에 공동저당권이 설정되고 두 부동산이 동시에 경매되는 경우, 공동저당권자는 두 부동산의 경매대가에 비례하여 안분 배당받는다.</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>문10·공동저당동시배당</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>채무자 소유와 물상보증인 소유 부동산이 함께 경매되는 경우에는 민법 제368조 제1항이 적용되지 않고, 채무자 소유 부동산의 경매대가에서 우선 배당받는다.</t>
+        </is>
+      </c>
+      <c r="G1382" t="inlineStr">
+        <is>
+          <t>대판 2010.4.15. 2008다41475</t>
+        </is>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>제368조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="n">
+        <v>1528</v>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>물상보증인 소유 부동산이 먼저 경매되어 공동저당권자가 채권 전액을 배당받은 경우, 물상보증인 소유 부동산의 후순위 저당권자는 물상보증인을 대위하여 채무자 소유 부동산에 관한 저당권이전의 부기등기를 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>문10·후순위대위</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>판례는 물상보증인의 변제자대위로 채무자 소유 부동산에 이전되는 저당권에 대하여 물상보증인 소유 부동산의 후순위 저당권자가 물상대위할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1383" t="inlineStr">
+        <is>
+          <t>대판 1994.5.10. 93다25417</t>
+        </is>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>제368조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="n">
+        <v>1529</v>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>당사자는 합의로 대여금 채권의 소멸시효 기간을 20년으로 연장할 수 있고, 그 연장 합의로 연대보증채권의 소멸시효 기간도 20년으로 연장된다.</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>문11·시효연장합의</t>
+        </is>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>민법 제184조 제2항에 따라 소멸시효는 법률행위로 이를 배제·연장·가중할 수 없으므로 시효기간을 연장하는 합의는 효력이 없다.</t>
+        </is>
+      </c>
+      <c r="G1384" t="inlineStr">
+        <is>
+          <t>민법 제184조 제2항</t>
+        </is>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>제184조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="n">
+        <v>1530</v>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>채권자가 주채무자의 재산을 가압류하였으나 그 사실을 연대보증인에게 통지하지 않은 경우, 연대보증채권에 대해서는 시효중단의 효력이 발생하지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>문11·보증시효중단</t>
+        </is>
+      </c>
+      <c r="F1385" t="inlineStr">
+        <is>
+          <t>민법 제440조에 따라 주채무자에 대한 시효중단은 보증인에게도 효력이 미치며, 보증인에 대한 별도의 통지는 필요하지 않다.</t>
+        </is>
+      </c>
+      <c r="G1385" t="inlineStr">
+        <is>
+          <t>민법 제440조</t>
+        </is>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>제440조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="n">
+        <v>1531</v>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>채무자가 제기한 채무부존재확인의 소에서 채권자가 청구기각을 구하며 채권의 존재를 적극적으로 주장하는 답변서를 제출한 경우, 그 응소는 재판상 청구에 준하여 답변서 제출 시에 시효중단의 효력이 생긴다.</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>문11·응소시효중단</t>
+        </is>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>판례는 채권자의 응소로 인한 시효중단은 현실적으로 권리를 주장한 때(답변서 제출 등)에 발생한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1386" t="inlineStr">
+        <is>
+          <t>대판 2010.8.26. 2008다42416</t>
+        </is>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>제168조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="n">
+        <v>1532</v>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>부동산을 양수하여 소유권이전등기청구권을 가진 자가 양도인의 이중양도로 부동산 가액 상당의 손해배상채권을 취득한 경우, 그 손해배상채권은 이중양도행위에 대한 채권자취소권의 피보전채권이 된다.</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>문12·취소피보전채권</t>
+        </is>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>판례는 이중양도로 발생한 금전 손해배상채권이 사해행위인 이중양도에 대한 채권자취소권의 피보전채권이 될 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1387" t="inlineStr">
+        <is>
+          <t>대판 1999.4.27. 98다56690</t>
+        </is>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="n">
+        <v>1533</v>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>채무자가 신용카드 가입계약을 체결하였더라도 자신의 유일한 부동산을 매도한 후에 비로소 신용카드를 사용하여 카드대금을 연체한 경우, 그 카드대금채권은 사해행위 이후 발생한 채권이어서 채권자취소권의 피보전채권이 될 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>문12·사후발생채권</t>
+        </is>
+      </c>
+      <c r="F1388" t="inlineStr">
+        <is>
+          <t>판례는 사해행위 후에 비로소 발생한 카드대금채권은 피보전채권이 될 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1388" t="inlineStr">
+        <is>
+          <t>대판 2004.11.12. 2004다40955</t>
+        </is>
+      </c>
+      <c r="H1388" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="n">
+        <v>1534</v>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>채무초과 상태의 채무자가 소멸시효 완성 후에 한 소멸시효이익의 포기행위는 채권자취소권의 대상인 사해행위가 될 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>문12·시효이익포기사해</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>판례는 채무초과 상태에서의 소멸시효이익 포기가 일반채권자를 해하는 사해행위가 될 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1389" t="inlineStr">
+        <is>
+          <t>대판 2013.5.31. 2012다4633</t>
+        </is>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>제406조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="n">
+        <v>1535</v>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>토지와 그 지상 건물을 공유하던 자가 건물에 관한 자신의 공유지분만을 제3자에게 양도한 경우, 그 제3자는 토지 전부에 관하여 건물 소유를 위한 관습법상 법정지상권을 취득한다.</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>문13·공유지분법정지상권</t>
+        </is>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>토지·건물 공유에서 건물 지분만의 양도로는 토지 공유자 전원의 처분이 아니어서 관습법상 법정지상권이 성립하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1390" t="inlineStr">
+        <is>
+          <t>대판 2014.9.4. 2011다73038</t>
+        </is>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>제366조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="n">
+        <v>1536</v>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>토지와 미등기건물을 함께 매도하여 토지에 관하여만 매수인 명의로 소유권이전등기가 이루어진 경우, 매도인은 그 미등기건물의 소유를 위한 관습법상 법정지상권을 취득한다.</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>문13·미등기건물법정지상권</t>
+        </is>
+      </c>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>토지와 건물을 함께 매도한 경우에는 관습법상 법정지상권을 인정할 필요가 없어 매도인에게 성립하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1391" t="inlineStr">
+        <is>
+          <t>대판 2002.6.20. 2002다9660</t>
+        </is>
+      </c>
+      <c r="H1391" t="inlineStr">
+        <is>
+          <t>제366조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="n">
+        <v>1537</v>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>연대보증인은 채권자의 이행청구에 대하여 주채무자에게 변제자력이 있고 그 집행이 용이함을 증명하여 먼저 주채무자에게 집행할 것을 항변할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>문14·최고검색항변</t>
+        </is>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>연대보증인에게는 민법 제437조 단서에 따라 최고·검색의 항변권이 인정되지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1392" t="inlineStr">
+        <is>
+          <t>민법 제437조 단서</t>
+        </is>
+      </c>
+      <c r="H1392" t="inlineStr">
+        <is>
+          <t>제437조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="n">
+        <v>1538</v>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>부담부분 비율에 관한 특약이 없는 공동연대보증인 중 1인이 자신의 부담부분에 미치지 못하는 금액을 변제한 경우, 그는 다른 연대보증인에게 구상권을 행사할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>문14·보증인구상</t>
+        </is>
+      </c>
+      <c r="F1393" t="inlineStr">
+        <is>
+          <t>공동보증인 사이의 구상은 자기의 부담부분을 넘는 변제를 한 경우에 인정된다.</t>
+        </is>
+      </c>
+      <c r="G1393" t="inlineStr">
+        <is>
+          <t>민법 제448조</t>
+        </is>
+      </c>
+      <c r="H1393" t="inlineStr">
+        <is>
+          <t>제448조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="n">
+        <v>1539</v>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>면책적 채무인수에 관하여 채권자가 승낙을 거절하는 의사표시를 하였다가 이후 이를 번복하여 승낙한 경우, 면책적 채무인수의 효력은 채무인수계약이 성립한 때로 소급하여 발생한다.</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>문15·승낙거절후번복</t>
+        </is>
+      </c>
+      <c r="F1394" t="inlineStr">
+        <is>
+          <t>채권자가 일단 승낙을 거절하면 그로써 채무인수의 효력이 확정적으로 발생하지 않게 되므로, 이후 다시 승낙하여도 소급효가 생기지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1394" t="inlineStr">
+        <is>
+          <t>민법 제457조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1394" t="inlineStr">
+        <is>
+          <t>제457조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="n">
+        <v>1540</v>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>점유취득시효가 완성된 점유자가 그 권리를 행사하지 않는 동안 시효완성 사실을 모르는 소유자가 제3자에게 저당권을 설정해 준 후, 점유자가 시효완성을 원인으로 소유권이전등기를 마친 경우, 점유자는 저당권의 부담이 있는 채로 소유권을 취득한다.</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>문16·시효완성후저당</t>
+        </is>
+      </c>
+      <c r="F1395" t="inlineStr">
+        <is>
+          <t>판례는 시효완성자가 등기 전에 설정된 저당권의 부담을 안은 채로 소유권을 취득한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1395" t="inlineStr">
+        <is>
+          <t>대판 2006.5.12. 2005다75910</t>
+        </is>
+      </c>
+      <c r="H1395" t="inlineStr">
+        <is>
+          <t>제245조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="n">
+        <v>1541</v>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>점유취득시효 완성자로부터 점유를 승계한 자는 전 점유자의 취득시효 완성의 효과를 주장하여 직접 자기에게 소유권이전등기를 청구할 수는 없다.</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>문16·점유승계</t>
+        </is>
+      </c>
+      <c r="F1396" t="inlineStr">
+        <is>
+          <t>판례는 점유의 승계가 있어도 취득시효 완성으로 인한 소유권이전등기청구권 자체가 당연히 승계되는 것은 아니어서 직접 청구할 수 없다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1396" t="inlineStr">
+        <is>
+          <t>대판 1995.3.28. 93다47745</t>
+        </is>
+      </c>
+      <c r="H1396" t="inlineStr">
+        <is>
+          <t>제245조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="n">
+        <v>1542</v>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>채권자대위소송에서 제3채무자는 피대위채권에 대한 항변뿐만 아니라, 채권자의 채무자에 대한 피보전채권이 변제로 소멸하였다는 사정도 주장하여 다툴 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>문17·피보전채권다툼</t>
+        </is>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>제3채무자는 채권자와 채무자 사이의 피보전채권의 존부를 다툴 수 없고, 이는 채권자와 채무자 사이의 문제에 불과하다.</t>
+        </is>
+      </c>
+      <c r="G1397" t="inlineStr">
+        <is>
+          <t>대판 2009.5.28. 2009다4787</t>
+        </is>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>제404조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="n">
+        <v>1543</v>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>채무자의 부동산에 제3자 명의의 소유권이전등기청구권 보전 가등기가 있는 경우, 그 가등기가 담보가등기로서 강제집행을 통한 매각이 가능하다는 등의 특별한 사정이 없는 한, 채무자의 무자력 판단에서 그 부동산은 적극재산으로 산정할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>문17·무자력산정</t>
+        </is>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>판례는 순위보전 가등기가 있는 부동산은 책임재산으로 평가하기 어려워 적극재산에 산입하지 않는다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1398" t="inlineStr">
+        <is>
+          <t>대판 2009.2.26. 2008다76556</t>
+        </is>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>제404조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="n">
+        <v>1544</v>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>구분소유적 공유관계를 표상하는 공유지분에 저당권이 설정된 후 특정 부분별로 토지가 분할되어 구분소유적 공유관계가 해소된 경우, 그 저당권은 종전의 구분소유적 공유지분의 비율대로 분할된 토지들 전부 위에 그대로 존속한다.</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>문18·구분공유저당</t>
+        </is>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>판례는 구분소유적 공유지분에 설정된 저당권은 분할 후에도 종전 지분 비율대로 분할된 각 토지 전부에 존속한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1399" t="inlineStr">
+        <is>
+          <t>대판 1989.8.8. 88다카24868</t>
+        </is>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>제356조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="n">
+        <v>1545</v>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>공유물의 소수지분권자가 다른 공유자와 협의 없이 공유물의 전부 또는 일부를 독점적으로 점유하는 경우, 다른 소수지분권자는 보존행위로서 그 점유자를 상대로 공유물의 인도를 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1400" t="inlineStr">
+        <is>
+          <t>문18·소수지분인도</t>
+        </is>
+      </c>
+      <c r="F1400" t="inlineStr">
+        <is>
+          <t>판례(전합)는 소수지분권자는 다른 소수지분권자의 독점 점유에 대해 보존행위로 공유물 인도를 청구할 수 없고 방해배제만 구할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1400" t="inlineStr">
+        <is>
+          <t>대판(전) 2020.5.21. 2018다287522</t>
+        </is>
+      </c>
+      <c r="H1400" t="inlineStr">
+        <is>
+          <t>제265조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="n">
+        <v>1546</v>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>과반수 지분을 가진 공유자가 공유물을 제3자에게 임대하여 수익을 얻는 것은 적법한 관리행위이므로 다른 공유자에 대한 불법행위가 되지 않으나, 소수지분권자는 자신의 지분에 상응하는 차임 상당액을 부당이득으로 반환청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>문18·과반수임대</t>
+        </is>
+      </c>
+      <c r="F1401" t="inlineStr">
+        <is>
+          <t>과반수 지분권자의 임대는 적법한 관리행위로 불법행위가 아니며, 소수지분권자는 지분 비율의 부당이득반환을 구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1401" t="inlineStr">
+        <is>
+          <t>대판 1991.9.24. 88다카33855</t>
+        </is>
+      </c>
+      <c r="H1401" t="inlineStr">
+        <is>
+          <t>제265조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="n">
+        <v>1547</v>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>불법행위로 건물이 훼손되어 사용·수리가 불가능한 경우, 특별한 사정이 없는 한 건물의 시가 외에 건물의 철거 비용도 통상손해의 범위에 포함된다.</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>문19·철거비용</t>
+        </is>
+      </c>
+      <c r="F1402" t="inlineStr">
+        <is>
+          <t>판례는 건물의 멸실에 준하는 훼손의 경우 시가 외에 철거비용도 통상손해에 포함된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1402" t="inlineStr">
+        <is>
+          <t>대판 2022.6.30. 2022다214042 · 판례</t>
+        </is>
+      </c>
+      <c r="H1402" t="inlineStr">
+        <is>
+          <t>제393조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="n">
+        <v>1548</v>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>이행기의 정함이 없는 채권의 양수인이 대항요건을 갖추지 못한 채 채무자를 상대로 이행의 소를 제기하고 소송 계속 중 채권양도통지가 이루어진 경우, 특별한 사정이 없는 한 채무자는 그 통지가 도달한 다음 날부터 이행지체의 책임을 진다.</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>문23·이행지체기산</t>
+        </is>
+      </c>
+      <c r="F1403" t="inlineStr">
+        <is>
+          <t>판례는 이행기 없는 채권에서 대항요건(통지)이 갖추어져 이행청구의 효력이 생긴 다음 날부터 지체책임이 발생한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1403" t="inlineStr">
+        <is>
+          <t>대판 2014.4.10. 2012다29557</t>
+        </is>
+      </c>
+      <c r="H1403" t="inlineStr">
+        <is>
+          <t>제387조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="n">
+        <v>1549</v>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>채권이 가압류되면 제3채무자는 채무자에게 지급하는 것이 금지되므로, 그 채권의 이행기가 경과하더라도 제3채무자는 이행지체의 책임을 지지 않는다.</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1404" t="inlineStr">
+        <is>
+          <t>문23·가압류지체</t>
+        </is>
+      </c>
+      <c r="F1404" t="inlineStr">
+        <is>
+          <t>채권의 가압류는 변제를 금지할 뿐이므로 이행기가 도래하면 제3채무자는 여전히 지체책임을 면하지 못한다.</t>
+        </is>
+      </c>
+      <c r="G1404" t="inlineStr">
+        <is>
+          <t>대판 1994.12.13. 93다951</t>
+        </is>
+      </c>
+      <c r="H1404" t="inlineStr">
+        <is>
+          <t>제387조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="n">
+        <v>1550</v>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>매매목적 부동산에 이미 제3자의 처분금지가처분 등기가 기입되어 있다는 사정만으로는 소유권이전등기절차의 이행이 불가능하게 되어 곧바로 매매계약이 이행불능으로 되는 것은 아니다.</t>
+        </is>
+      </c>
+      <c r="D1405" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1405" t="inlineStr">
+        <is>
+          <t>문23·가처분이행불능</t>
+        </is>
+      </c>
+      <c r="F1405" t="inlineStr">
+        <is>
+          <t>판례는 처분금지가처분 등기가 있더라도 그 사정만으로 매매가 이행불능이 되는 것은 아니라고 한다.</t>
+        </is>
+      </c>
+      <c r="G1405" t="inlineStr">
+        <is>
+          <t>대판 1999.6.11. 99다11045</t>
+        </is>
+      </c>
+      <c r="H1405" t="inlineStr">
+        <is>
+          <t>제390조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="n">
+        <v>1551</v>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>저당권과 함께 피담보채권을 양수한 자가 저당권이전의 부기등기를 마치고 저당권 실행 요건을 갖춘 경우, 채권양도의 대항요건을 갖추지 않았더라도 경매를 신청할 수 있고 경매개시결정 시 대항요건을 증명할 필요가 없다.</t>
+        </is>
+      </c>
+      <c r="D1406" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1406" t="inlineStr">
+        <is>
+          <t>문24·저당권부채권경매</t>
+        </is>
+      </c>
+      <c r="F1406" t="inlineStr">
+        <is>
+          <t>판례는 저당권부 채권 양수인이 부기등기를 마치면 대항요건 없이도 경매를 신청할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1406" t="inlineStr">
+        <is>
+          <t>대판 2005.6.23. 2004다29279</t>
+        </is>
+      </c>
+      <c r="H1406" t="inlineStr">
+        <is>
+          <t>제361조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="n">
+        <v>1552</v>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>양도금지특약을 위반하여 양도된 채권을 선의이며 중과실 없는 양수인이 취득한 후 다시 전득한 자는, 그 전득자가 양도금지특약을 알았거나 중과실로 알지 못하였더라도 채권을 유효하게 취득한다.</t>
+        </is>
+      </c>
+      <c r="D1407" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1407" t="inlineStr">
+        <is>
+          <t>문24·전득자취득</t>
+        </is>
+      </c>
+      <c r="F1407" t="inlineStr">
+        <is>
+          <t>판례는 선의·무중과실의 양수인이 일단 유효하게 취득하면 그로부터의 전득자는 악의라도 채권을 유효하게 취득한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1407" t="inlineStr">
+        <is>
+          <t>대판 2015.4.9. 2012다118020</t>
+        </is>
+      </c>
+      <c r="H1407" t="inlineStr">
+        <is>
+          <t>제449조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="n">
+        <v>1553</v>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>양도금지특약이 있는 채권의 양수인이 양수금 지급을 청구하는 경우, 양수인이 그 특약을 알지 못하였고 알지 못한 데 중과실이 없다는 점을 스스로 주장·증명하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1408" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1408" t="inlineStr">
+        <is>
+          <t>문24·증명책임</t>
+        </is>
+      </c>
+      <c r="F1408" t="inlineStr">
+        <is>
+          <t>양도금지특약의 존재와 양수인의 악의·중과실은 이를 이유로 무효를 주장하는 채무자가 주장·증명하여야 한다.</t>
+        </is>
+      </c>
+      <c r="G1408" t="inlineStr">
+        <is>
+          <t>대판 2019.12.19. 2016다24284</t>
+        </is>
+      </c>
+      <c r="H1408" t="inlineStr">
+        <is>
+          <t>제449조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="n">
+        <v>1554</v>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>저당물의 제3취득자가 그 부동산에 지출한 필요비·유익비는 민법 제367조에 따라 경매대가에서 우선 상환받을 수 있으므로, 제3취득자는 그 비용상환청구권을 피담보채권으로 하여 경매의 매수인에게 유치권으로 대항할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1409" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1409" t="inlineStr">
+        <is>
+          <t>문25·제367조유치권</t>
+        </is>
+      </c>
+      <c r="F1409" t="inlineStr">
+        <is>
+          <t>제367조의 비용상환청구권은 경매대가에서 우선상환을 받을 수 있을 뿐이고, 이를 피담보채권으로 한 유치권으로 매수인에게 대항할 수는 없다.</t>
+        </is>
+      </c>
+      <c r="G1409" t="inlineStr">
+        <is>
+          <t>대판 2023.7.13. 2022다265093</t>
+        </is>
+      </c>
+      <c r="H1409" t="inlineStr">
+        <is>
+          <t>제367조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="n">
+        <v>1555</v>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>유치권자가 피담보채권에 대한 별도의 시효중단 조치 없이 유치권확인의 소만을 제기하였더라도, 그 소송에서 피담보채권의 존재에 관한 주장에 대하여 실질적인 심리가 이루어졌다면 재판상 청구에 준하는 소멸시효 중단의 효력이 인정된다.</t>
+        </is>
+      </c>
+      <c r="D1410" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1410" t="inlineStr">
+        <is>
+          <t>문25·유치권확인시효</t>
+        </is>
+      </c>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>판례는 유치권확인소송에서 피담보채권에 관한 실질적 심리가 이루어지면 재판상 청구에 준하여 시효중단 효력을 인정한다.</t>
+        </is>
+      </c>
+      <c r="G1410" t="inlineStr">
+        <is>
+          <t>대판 2019.3.14. 2018다255648</t>
+        </is>
+      </c>
+      <c r="H1410" t="inlineStr">
+        <is>
+          <t>제168조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="n">
+        <v>1556</v>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>착오송금을 이유로 부당이득반환을 청구하는 소송에서 송금에 착오가 있었는지에 대한 증명책임은 반환을 구하는 송금인에게 있다.</t>
+        </is>
+      </c>
+      <c r="D1411" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1411" t="inlineStr">
+        <is>
+          <t>문26·착오송금입증</t>
+        </is>
+      </c>
+      <c r="F1411" t="inlineStr">
+        <is>
+          <t>부당이득반환을 구하는 자가 법률상 원인 없음(착오)을 증명하여야 한다.</t>
+        </is>
+      </c>
+      <c r="G1411" t="inlineStr">
+        <is>
+          <t>민법 제741조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1411" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="n">
+        <v>1557</v>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>토지소유자가 불법점유자를 상대로 차임 상당 부당이득반환을 청구하는 소송에서 점유자가 '불법점유가 없었더라도 소유자에게 차임 상당 이익이 발생할 여지가 없었다'고 주장하는 경우, 그 특별한 사정에 대한 증명책임은 점유자가 진다.</t>
+        </is>
+      </c>
+      <c r="D1412" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1412" t="inlineStr">
+        <is>
+          <t>문26·손실부존재입증</t>
+        </is>
+      </c>
+      <c r="F1412" t="inlineStr">
+        <is>
+          <t>판례는 손실이 없었다는 특별한 사정은 이를 주장하는 점유자(이득자)가 증명하여야 한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1412" t="inlineStr">
+        <is>
+          <t>대판 2008.1.17. 2006다586</t>
+        </is>
+      </c>
+      <c r="H1412" t="inlineStr">
+        <is>
+          <t>제741조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="n">
+        <v>1558</v>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>기존 금전채무의 변제에 갈음하여 부동산 소유권을 이전하기로 하는 대물변제예약을 체결한 경우, 소유권이전등기를 완료하기 전에 기존 금전채무가 소멸하였더라도 당사자 사이에서는 예약된 대물변제 계약에 기하여 소유권이전등기를 청구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1413" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1413" t="inlineStr">
+        <is>
+          <t>문27·대물변제예약</t>
+        </is>
+      </c>
+      <c r="F1413" t="inlineStr">
+        <is>
+          <t>대물변제예약은 기존 채무의 변제를 위한 것이므로 기존 채무가 소멸하면 대물변제할 이유가 없어 소유권이전등기를 청구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1413" t="inlineStr">
+        <is>
+          <t>민법 제466조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1413" t="inlineStr">
+        <is>
+          <t>제466조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="n">
+        <v>1559</v>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>변제기 전 변제에 관한 약정이 없는 이자부 금전소비대차의 채무자가 변제기 전에 변제하는 경우, 변제기까지의 약정이자 등 채권자의 손해를 함께 제공하지 않으면 채권자는 그 수령을 거절할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1414" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1414" t="inlineStr">
+        <is>
+          <t>문27·기한전변제</t>
+        </is>
+      </c>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>판례는 이자부 소비대차에서 기한 전 변제 시 채권자의 기한이익(약정이자)을 배상하지 않으면 수령을 거절할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1414" t="inlineStr">
+        <is>
+          <t>민법 제468조 · 판례</t>
+        </is>
+      </c>
+      <c r="H1414" t="inlineStr">
+        <is>
+          <t>제468조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="n">
+        <v>1560</v>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>공작물책임에서 공작물이 본래 갖추어야 할 안전성은 그 용도에 한정된 안전성만이 아니라, 공작물이 현실적으로 설치되어 사용되고 있는 상황에서 요구되는 안전성을 의미한다.</t>
+        </is>
+      </c>
+      <c r="D1415" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1415" t="inlineStr">
+        <is>
+          <t>문28·공작물안전성</t>
+        </is>
+      </c>
+      <c r="F1415" t="inlineStr">
+        <is>
+          <t>판례는 공작물의 안전성을 현실적 설치·사용 상황에서 요구되는 정도로 본다.</t>
+        </is>
+      </c>
+      <c r="G1415" t="inlineStr">
+        <is>
+          <t>대판 2018.7.12. 2015다68348 · 판례</t>
+        </is>
+      </c>
+      <c r="H1415" t="inlineStr">
+        <is>
+          <t>제758조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="n">
+        <v>1561</v>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>공작물책임에서 공작물의 점유자는 자신의 과실 유무와 관계없이 책임을 지고, 소유자는 자신의 과실이 있는 경우에만 책임을 진다.</t>
+        </is>
+      </c>
+      <c r="D1416" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1416" t="inlineStr">
+        <is>
+          <t>문28·점유자소유자책임</t>
+        </is>
+      </c>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>점유자는 손해 방지에 필요한 주의를 다하였음을 증명하면 면책되는 중간책임을 지고, 소유자는 면책이 인정되지 않는 무과실책임을 진다.</t>
+        </is>
+      </c>
+      <c r="G1416" t="inlineStr">
+        <is>
+          <t>민법 제758조 제1항</t>
+        </is>
+      </c>
+      <c r="H1416" t="inlineStr">
+        <is>
+          <t>제758조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="n">
+        <v>1562</v>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>부동산 매매에서 매수인이 선이행하여야 할 중도금을 지급하지 않은 채 잔대금 지급일을 경과한 경우, 특별한 사정이 없는 한 매수인의 중도금 및 그에 대한 지연손해금과 잔대금 지급의무는 매도인의 소유권이전등기의무와 동시이행관계에 있다.</t>
+        </is>
+      </c>
+      <c r="D1417" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1417" t="inlineStr">
+        <is>
+          <t>문29·중도금동시이행</t>
+        </is>
+      </c>
+      <c r="F1417" t="inlineStr">
+        <is>
+          <t>판례는 중도금 미지급 후 잔대금일이 지나면 중도금·지연손해금·잔대금 지급의무와 이전등기의무가 동시이행관계에 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1417" t="inlineStr">
+        <is>
+          <t>대판 1991.3.27. 90다19930</t>
+        </is>
+      </c>
+      <c r="H1417" t="inlineStr">
+        <is>
+          <t>제536조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="n">
+        <v>1563</v>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>동시이행관계에 있는 쌍방 채무 중 어느 한 채무가 이행불능이 되어 손해배상채무로 변한 경우, 그 손해배상채무도 다른 채무와 여전히 동시이행관계에 있다.</t>
+        </is>
+      </c>
+      <c r="D1418" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1418" t="inlineStr">
+        <is>
+          <t>문29·손배동시이행</t>
+        </is>
+      </c>
+      <c r="F1418" t="inlineStr">
+        <is>
+          <t>판례는 동시이행관계의 채무가 손해배상채무로 변경되어도 동일성이 유지되어 동시이행관계가 존속한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1418" t="inlineStr">
+        <is>
+          <t>대판 2000.2.25. 97다30066</t>
+        </is>
+      </c>
+      <c r="H1418" t="inlineStr">
+        <is>
+          <t>제536조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="n">
+        <v>1564</v>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>매수인이 매매대금을 완납하였다면 목적물을 아직 인도받지 못하였더라도 그 이후 목적물에서 생기는 과실의 수취권은 매수인에게 귀속된다.</t>
+        </is>
+      </c>
+      <c r="D1419" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1419" t="inlineStr">
+        <is>
+          <t>문30·과실수취권</t>
+        </is>
+      </c>
+      <c r="F1419" t="inlineStr">
+        <is>
+          <t>민법 제587조에 따라 매수인이 대금을 완납하면 그 후의 과실수취권은 매수인에게 귀속된다.</t>
+        </is>
+      </c>
+      <c r="G1419" t="inlineStr">
+        <is>
+          <t>민법 제587조</t>
+        </is>
+      </c>
+      <c r="H1419" t="inlineStr">
+        <is>
+          <t>제587조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="n">
+        <v>1565</v>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>매매목적물을 인도받지 못하고 매수인 자신도 대금을 지급하지 않은 경우, 매수인은 매도인에게 인도의무의 지체로 인한 손해배상금의 지급을 구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1420" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1420" t="inlineStr">
+        <is>
+          <t>문30·동시이행지체</t>
+        </is>
+      </c>
+      <c r="F1420" t="inlineStr">
+        <is>
+          <t>매수인이 대금을 지급하지 않은 이상 매도인의 인도의무는 동시이행 항변으로 지체에 빠지지 않으므로 지체로 인한 손해배상을 구할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1420" t="inlineStr">
+        <is>
+          <t>민법 제536조 · 제587조</t>
+        </is>
+      </c>
+      <c r="H1420" t="inlineStr">
+        <is>
+          <t>제536조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="n">
+        <v>1566</v>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>상가건물 임대차에서 임차인이 임대차기간 중 3기의 차임액에 이르도록 차임을 연체한 사실이 있다면, 계약갱신 요구 당시 연체액이 3기에 이르지 않게 되었더라도 임대인은 그 갱신 요구를 거절할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1421" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1421" t="inlineStr">
+        <is>
+          <t>문31·3기연체갱신</t>
+        </is>
+      </c>
+      <c r="F1421" t="inlineStr">
+        <is>
+          <t>판례는 과거에 3기 연체 사실이 있으면 갱신 요구 당시 연체가 해소되었어도 갱신거절 사유가 된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1421" t="inlineStr">
+        <is>
+          <t>대판 2021.5.13. 2020다255429</t>
+        </is>
+      </c>
+      <c r="H1421" t="inlineStr">
+        <is>
+          <t>제640조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="n">
+        <v>1567</v>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr">
+        <is>
+          <t>임대차보증금이 수수된 임대차에서 차임채권에 압류 및 추심명령이 있었더라도, 임대차가 종료되어 목적물이 반환될 때까지 추심되지 않은 차임채권액은 임대차보증금에서 당연히 공제된다.</t>
+        </is>
+      </c>
+      <c r="D1422" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1422" t="inlineStr">
+        <is>
+          <t>문31·차임공제</t>
+        </is>
+      </c>
+      <c r="F1422" t="inlineStr">
+        <is>
+          <t>판례는 차임채권에 압류·추심명령이 있어도 종료 시까지 미추심 차임은 보증금에서 당연 공제된다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1422" t="inlineStr">
+        <is>
+          <t>대판 2004.12.23. 2004다56554</t>
+        </is>
+      </c>
+      <c r="H1422" t="inlineStr">
+        <is>
+          <t>제618조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="n">
+        <v>1568</v>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr">
+        <is>
+          <t>자필증서에 의한 유언에서 유언자가 주소를 자서하지 않았더라도 유언자의 특정에 지장이 없다면 그 유언은 유효하다.</t>
+        </is>
+      </c>
+      <c r="D1423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1423" t="inlineStr">
+        <is>
+          <t>문32·자필증서주소</t>
+        </is>
+      </c>
+      <c r="F1423" t="inlineStr">
+        <is>
+          <t>민법 제1066조는 자필증서 유언의 요건으로 주소의 자서를 요구하므로, 주소를 자서하지 않은 자필증서 유언은 무효이다.</t>
+        </is>
+      </c>
+      <c r="G1423" t="inlineStr">
+        <is>
+          <t>민법 제1066조</t>
+        </is>
+      </c>
+      <c r="H1423" t="inlineStr">
+        <is>
+          <t>제1066조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="n">
+        <v>1569</v>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr">
+        <is>
+          <t>유언증서가 성립한 후에 멸실되거나 분실되었더라도 유언자가 유언을 철회한 것으로 볼 수 없는 이상 그 사유만으로 유언이 실효되는 것은 아니고, 이해관계인은 유언증서의 내용을 증명하여 유언의 효력을 주장할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1424" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1424" t="inlineStr">
+        <is>
+          <t>문32·유언증서멸실</t>
+        </is>
+      </c>
+      <c r="F1424" t="inlineStr">
+        <is>
+          <t>판례는 유언증서의 멸실·분실만으로 유언이 실효되지 않고 내용을 증명하여 효력을 주장할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1424" t="inlineStr">
+        <is>
+          <t>대판 1996.9.20. 96다21119</t>
+        </is>
+      </c>
+      <c r="H1424" t="inlineStr">
+        <is>
+          <t>제1060조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="n">
+        <v>1570</v>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr">
+        <is>
+          <t>가정법원은 부 또는 모가 친권을 남용하여 자녀의 복리를 현저히 해치거나 해칠 우려가 있는 경우, 일정한 기간을 정하여 그 친권을 상실시킬 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1425" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1425" t="inlineStr">
+        <is>
+          <t>문33·친권상실기간</t>
+        </is>
+      </c>
+      <c r="F1425" t="inlineStr">
+        <is>
+          <t>친권상실 선고에는 기간을 정하지 않으며, 기간을 정하여 제한하는 것은 친권의 일시 정지에 해당한다.</t>
+        </is>
+      </c>
+      <c r="G1425" t="inlineStr">
+        <is>
+          <t>민법 제924조</t>
+        </is>
+      </c>
+      <c r="H1425" t="inlineStr">
+        <is>
+          <t>제924조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="n">
+        <v>1571</v>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr">
+        <is>
+          <t>상속재산분할에 관하여 공동상속인 사이에 협의가 성립되지 않거나 협의할 수 없는 경우, 각 공동상속인은 상속재산에 속하는 개별 재산에 관하여 공유물분할청구의 소를 제기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1426" t="inlineStr">
+        <is>
+          <t>문34·상속공유물분할</t>
+        </is>
+      </c>
+      <c r="F1426" t="inlineStr">
+        <is>
+          <t>상속재산분할은 가사비송인 상속재산분할심판에 의하여야 하고, 개별 재산에 관한 공유물분할청구의 소로 할 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1426" t="inlineStr">
+        <is>
+          <t>대판 2015.8.13. 2015다18367</t>
+        </is>
+      </c>
+      <c r="H1426" t="inlineStr">
+        <is>
+          <t>제1013조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="n">
+        <v>1572</v>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr">
+        <is>
+          <t>협의분할로 공동상속인 중 일부가 자기 고유의 상속분을 초과하여 상속재산을 취득한 경우, 이는 상속개시 당시에 소급하여 피상속인으로부터 승계받은 것으로 보아야 하고 다른 공동상속인으로부터 증여받은 것으로 볼 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1427" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1427" t="inlineStr">
+        <is>
+          <t>문34·협의분할소급</t>
+        </is>
+      </c>
+      <c r="F1427" t="inlineStr">
+        <is>
+          <t>민법 제1015조에 따라 상속재산분할은 상속개시 시로 소급하여 효력이 있으므로 증여로 보지 않는다.</t>
+        </is>
+      </c>
+      <c r="G1427" t="inlineStr">
+        <is>
+          <t>민법 제1015조</t>
+        </is>
+      </c>
+      <c r="H1427" t="inlineStr">
+        <is>
+          <t>제1015조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="n">
+        <v>1573</v>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr">
+        <is>
+          <t>이혼에 따른 재산분할에서 일방이 제3자와 합유하는 재산은 임의로 처분할 수 없어 직접 분할을 명할 수는 없으나, 그 지분의 가액을 산정하여 분할 대상으로 삼거나 다른 재산의 분할에 참작하는 방법으로 분할 대상에 포함하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1428" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1428" t="inlineStr">
+        <is>
+          <t>문35·합유재산분할</t>
+        </is>
+      </c>
+      <c r="F1428" t="inlineStr">
+        <is>
+          <t>판례는 합유재산은 직접 분할을 명할 수 없으나 지분 가액을 산정하여 재산분할에 참작하여야 한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1428" t="inlineStr">
+        <is>
+          <t>대판 2009.11.12. 2009므2840</t>
+        </is>
+      </c>
+      <c r="H1428" t="inlineStr">
+        <is>
+          <t>제839조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="n">
+        <v>1574</v>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr">
+        <is>
+          <t>이혼에 따른 재산분할 사건에서 법원은 당사자가 특정한 분할 방법에 구애받지 않고 재산분할의 대상과 가액을 직권으로 조사·판단할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1429" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1429" t="inlineStr">
+        <is>
+          <t>문35·직권조사</t>
+        </is>
+      </c>
+      <c r="F1429" t="inlineStr">
+        <is>
+          <t>재산분할은 가사비송사건으로 법원이 후견적 입장에서 직권으로 대상과 가액을 조사·판단한다.</t>
+        </is>
+      </c>
+      <c r="G1429" t="inlineStr">
+        <is>
+          <t>대판 2022.1.27. 2018므11273 · 판례</t>
+        </is>
+      </c>
+      <c r="H1429" t="inlineStr">
+        <is>
+          <t>제839조의2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="n">
+        <v>1575</v>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr">
+        <is>
+          <t>재산분할청구권은 이혼이 성립한 때 법적 효과로서 발생하므로, 협의나 심판에 의하여 그 구체적 내용이 형성되기 전이라도 이혼 성립 후에는 곧바로 채권양도의 대상이 된다.</t>
+        </is>
+      </c>
+      <c r="D1430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E1430" t="inlineStr">
+        <is>
+          <t>문35·분할청구권양도</t>
+        </is>
+      </c>
+      <c r="F1430" t="inlineStr">
+        <is>
+          <t>협의나 심판으로 구체적 내용이 형성되기 전의 재산분할청구권은 범위와 내용이 불명확하여 양도의 대상이 될 수 없다.</t>
+        </is>
+      </c>
+      <c r="G1430" t="inlineStr">
+        <is>
+          <t>대판 1999.4.9. 98다58016</t>
+        </is>
+      </c>
+      <c r="H1430" t="inlineStr">
+        <is>
+          <t>제839조의2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix 변시15 OX via 공기출 cross-check (1434 items)
</commit_message>
<xml_diff>
--- a/assets/ox_civil_bar14.xlsx
+++ b/assets/ox_civil_bar14.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1430"/>
+  <dimension ref="A1:H1435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -55920,17 +55920,17 @@
       </c>
       <c r="D1387" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1387" t="inlineStr">
         <is>
-          <t>문12·취소피보전채권</t>
+          <t>문12·이중양도피보전채권</t>
         </is>
       </c>
       <c r="F1387" t="inlineStr">
         <is>
-          <t>판례는 이중양도로 발생한 금전 손해배상채권이 사해행위인 이중양도에 대한 채권자취소권의 피보전채권이 될 수 있다고 한다.</t>
+          <t>판례는 이중양도로 취득하는 부동산 가액 상당의 손해배상채권은 사해행위(이중양도) 이후에 발생한 것이어서 그 이중양도행위에 대한 채권자취소권의 피보전채권이 될 수 없다고 한다.</t>
         </is>
       </c>
       <c r="G1387" t="inlineStr">
@@ -56315,27 +56315,27 @@
       </c>
       <c r="C1397" t="inlineStr">
         <is>
-          <t>채권자대위소송에서 제3채무자는 피대위채권에 대한 항변뿐만 아니라, 채권자의 채무자에 대한 피보전채권이 변제로 소멸하였다는 사정도 주장하여 다툴 수 있다.</t>
+          <t>채권자대위소송에서 제3채무자는 채권자의 채무자에 대한 피보전채권이 발생원인인 법률행위의 무효나 변제로 소멸하였다는 사정을 주장하여 다툴 수 있고, 이 경우 법원은 피보전채권의 존부를 직권으로 심리·판단하여야 한다.</t>
         </is>
       </c>
       <c r="D1397" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E1397" t="inlineStr">
         <is>
-          <t>문17·피보전채권다툼</t>
+          <t>문17·피보전채권소송요건</t>
         </is>
       </c>
       <c r="F1397" t="inlineStr">
         <is>
-          <t>제3채무자는 채권자와 채무자 사이의 피보전채권의 존부를 다툴 수 없고, 이는 채권자와 채무자 사이의 문제에 불과하다.</t>
+          <t>피보전채권의 존재는 채권자대위소송의 당사자적격에 관한 소송요건으로 법원의 직권조사사항이므로, 제3채무자도 그 부존재(무효·변제소멸)를 주장하여 다툴 수 있다.</t>
         </is>
       </c>
       <c r="G1397" t="inlineStr">
         <is>
-          <t>대판 2009.5.28. 2009다4787</t>
+          <t>대판 2009.4.23. 2009다3234</t>
         </is>
       </c>
       <c r="H1397" t="inlineStr">
@@ -56506,7 +56506,7 @@
     </row>
     <row r="1402">
       <c r="A1402" t="n">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="B1402" t="inlineStr">
         <is>
@@ -56515,7 +56515,7 @@
       </c>
       <c r="C1402" t="inlineStr">
         <is>
-          <t>불법행위로 건물이 훼손되어 사용·수리가 불가능한 경우, 특별한 사정이 없는 한 건물의 시가 외에 건물의 철거 비용도 통상손해의 범위에 포함된다.</t>
+          <t>이행기의 정함이 없는 채권의 양수인이 대항요건을 갖추지 못한 채 채무자를 상대로 이행의 소를 제기하고 소송 계속 중 채권양도통지가 이루어진 경우, 특별한 사정이 없는 한 채무자는 그 통지가 도달한 다음 날부터 이행지체의 책임을 진다.</t>
         </is>
       </c>
       <c r="D1402" t="inlineStr">
@@ -56525,28 +56525,28 @@
       </c>
       <c r="E1402" t="inlineStr">
         <is>
-          <t>문19·철거비용</t>
+          <t>문23·이행지체기산</t>
         </is>
       </c>
       <c r="F1402" t="inlineStr">
         <is>
-          <t>판례는 건물의 멸실에 준하는 훼손의 경우 시가 외에 철거비용도 통상손해에 포함된다고 한다.</t>
+          <t>판례는 이행기 없는 채권에서 대항요건(통지)이 갖추어져 이행청구의 효력이 생긴 다음 날부터 지체책임이 발생한다고 한다.</t>
         </is>
       </c>
       <c r="G1402" t="inlineStr">
         <is>
-          <t>대판 2022.6.30. 2022다214042 · 판례</t>
+          <t>대판 2014.4.10. 2012다29557</t>
         </is>
       </c>
       <c r="H1402" t="inlineStr">
         <is>
-          <t>제393조</t>
+          <t>제387조</t>
         </is>
       </c>
     </row>
     <row r="1403">
       <c r="A1403" t="n">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="B1403" t="inlineStr">
         <is>
@@ -56555,27 +56555,27 @@
       </c>
       <c r="C1403" t="inlineStr">
         <is>
-          <t>이행기의 정함이 없는 채권의 양수인이 대항요건을 갖추지 못한 채 채무자를 상대로 이행의 소를 제기하고 소송 계속 중 채권양도통지가 이루어진 경우, 특별한 사정이 없는 한 채무자는 그 통지가 도달한 다음 날부터 이행지체의 책임을 진다.</t>
+          <t>채권이 가압류되면 제3채무자는 채무자에게 지급하는 것이 금지되므로, 그 채권의 이행기가 경과하더라도 제3채무자는 이행지체의 책임을 지지 않는다.</t>
         </is>
       </c>
       <c r="D1403" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1403" t="inlineStr">
         <is>
-          <t>문23·이행지체기산</t>
+          <t>문23·가압류지체</t>
         </is>
       </c>
       <c r="F1403" t="inlineStr">
         <is>
-          <t>판례는 이행기 없는 채권에서 대항요건(통지)이 갖추어져 이행청구의 효력이 생긴 다음 날부터 지체책임이 발생한다고 한다.</t>
+          <t>채권의 가압류는 변제를 금지할 뿐이므로 이행기가 도래하면 제3채무자는 여전히 지체책임을 면하지 못한다.</t>
         </is>
       </c>
       <c r="G1403" t="inlineStr">
         <is>
-          <t>대판 2014.4.10. 2012다29557</t>
+          <t>대판 1994.12.13. 93다951</t>
         </is>
       </c>
       <c r="H1403" t="inlineStr">
@@ -56586,7 +56586,7 @@
     </row>
     <row r="1404">
       <c r="A1404" t="n">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="B1404" t="inlineStr">
         <is>
@@ -56595,38 +56595,38 @@
       </c>
       <c r="C1404" t="inlineStr">
         <is>
-          <t>채권이 가압류되면 제3채무자는 채무자에게 지급하는 것이 금지되므로, 그 채권의 이행기가 경과하더라도 제3채무자는 이행지체의 책임을 지지 않는다.</t>
+          <t>매매목적 부동산에 이미 제3자의 처분금지가처분 등기가 기입되어 있다는 사정만으로는 소유권이전등기절차의 이행이 불가능하게 되어 곧바로 매매계약이 이행불능으로 되는 것은 아니다.</t>
         </is>
       </c>
       <c r="D1404" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E1404" t="inlineStr">
         <is>
-          <t>문23·가압류지체</t>
+          <t>문23·가처분이행불능</t>
         </is>
       </c>
       <c r="F1404" t="inlineStr">
         <is>
-          <t>채권의 가압류는 변제를 금지할 뿐이므로 이행기가 도래하면 제3채무자는 여전히 지체책임을 면하지 못한다.</t>
+          <t>판례는 처분금지가처분 등기가 있더라도 그 사정만으로 매매가 이행불능이 되는 것은 아니라고 한다.</t>
         </is>
       </c>
       <c r="G1404" t="inlineStr">
         <is>
-          <t>대판 1994.12.13. 93다951</t>
+          <t>대판 1999.6.11. 99다11045</t>
         </is>
       </c>
       <c r="H1404" t="inlineStr">
         <is>
-          <t>제387조</t>
+          <t>제390조</t>
         </is>
       </c>
     </row>
     <row r="1405">
       <c r="A1405" t="n">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="B1405" t="inlineStr">
         <is>
@@ -56635,7 +56635,7 @@
       </c>
       <c r="C1405" t="inlineStr">
         <is>
-          <t>매매목적 부동산에 이미 제3자의 처분금지가처분 등기가 기입되어 있다는 사정만으로는 소유권이전등기절차의 이행이 불가능하게 되어 곧바로 매매계약이 이행불능으로 되는 것은 아니다.</t>
+          <t>저당권과 함께 피담보채권을 양수한 자가 저당권이전의 부기등기를 마치고 저당권 실행 요건을 갖춘 경우, 채권양도의 대항요건을 갖추지 않았더라도 경매를 신청할 수 있고 경매개시결정 시 대항요건을 증명할 필요가 없다.</t>
         </is>
       </c>
       <c r="D1405" t="inlineStr">
@@ -56645,28 +56645,28 @@
       </c>
       <c r="E1405" t="inlineStr">
         <is>
-          <t>문23·가처분이행불능</t>
+          <t>문24·저당권부채권경매</t>
         </is>
       </c>
       <c r="F1405" t="inlineStr">
         <is>
-          <t>판례는 처분금지가처분 등기가 있더라도 그 사정만으로 매매가 이행불능이 되는 것은 아니라고 한다.</t>
+          <t>판례는 저당권부 채권 양수인이 부기등기를 마치면 대항요건 없이도 경매를 신청할 수 있다고 한다.</t>
         </is>
       </c>
       <c r="G1405" t="inlineStr">
         <is>
-          <t>대판 1999.6.11. 99다11045</t>
+          <t>대판 2005.6.23. 2004다29279</t>
         </is>
       </c>
       <c r="H1405" t="inlineStr">
         <is>
-          <t>제390조</t>
+          <t>제361조</t>
         </is>
       </c>
     </row>
     <row r="1406">
       <c r="A1406" t="n">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="B1406" t="inlineStr">
         <is>
@@ -56675,7 +56675,7 @@
       </c>
       <c r="C1406" t="inlineStr">
         <is>
-          <t>저당권과 함께 피담보채권을 양수한 자가 저당권이전의 부기등기를 마치고 저당권 실행 요건을 갖춘 경우, 채권양도의 대항요건을 갖추지 않았더라도 경매를 신청할 수 있고 경매개시결정 시 대항요건을 증명할 필요가 없다.</t>
+          <t>양도금지특약을 위반하여 양도된 채권을 선의이며 중과실 없는 양수인이 취득한 후 다시 전득한 자는, 그 전득자가 양도금지특약을 알았거나 중과실로 알지 못하였더라도 채권을 유효하게 취득한다.</t>
         </is>
       </c>
       <c r="D1406" t="inlineStr">
@@ -56685,28 +56685,28 @@
       </c>
       <c r="E1406" t="inlineStr">
         <is>
-          <t>문24·저당권부채권경매</t>
+          <t>문24·전득자취득</t>
         </is>
       </c>
       <c r="F1406" t="inlineStr">
         <is>
-          <t>판례는 저당권부 채권 양수인이 부기등기를 마치면 대항요건 없이도 경매를 신청할 수 있다고 한다.</t>
+          <t>판례는 선의·무중과실의 양수인이 일단 유효하게 취득하면 그로부터의 전득자는 악의라도 채권을 유효하게 취득한다고 한다.</t>
         </is>
       </c>
       <c r="G1406" t="inlineStr">
         <is>
-          <t>대판 2005.6.23. 2004다29279</t>
+          <t>대판 2015.4.9. 2012다118020</t>
         </is>
       </c>
       <c r="H1406" t="inlineStr">
         <is>
-          <t>제361조</t>
+          <t>제449조</t>
         </is>
       </c>
     </row>
     <row r="1407">
       <c r="A1407" t="n">
-        <v>1552</v>
+        <v>1553</v>
       </c>
       <c r="B1407" t="inlineStr">
         <is>
@@ -56715,27 +56715,27 @@
       </c>
       <c r="C1407" t="inlineStr">
         <is>
-          <t>양도금지특약을 위반하여 양도된 채권을 선의이며 중과실 없는 양수인이 취득한 후 다시 전득한 자는, 그 전득자가 양도금지특약을 알았거나 중과실로 알지 못하였더라도 채권을 유효하게 취득한다.</t>
+          <t>양도금지특약이 있는 채권의 양수인이 양수금 지급을 청구하는 경우, 양수인이 그 특약을 알지 못하였고 알지 못한 데 중과실이 없다는 점을 스스로 주장·증명하여야 한다.</t>
         </is>
       </c>
       <c r="D1407" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1407" t="inlineStr">
         <is>
-          <t>문24·전득자취득</t>
+          <t>문24·증명책임</t>
         </is>
       </c>
       <c r="F1407" t="inlineStr">
         <is>
-          <t>판례는 선의·무중과실의 양수인이 일단 유효하게 취득하면 그로부터의 전득자는 악의라도 채권을 유효하게 취득한다고 한다.</t>
+          <t>양도금지특약의 존재와 양수인의 악의·중과실은 이를 이유로 무효를 주장하는 채무자가 주장·증명하여야 한다.</t>
         </is>
       </c>
       <c r="G1407" t="inlineStr">
         <is>
-          <t>대판 2015.4.9. 2012다118020</t>
+          <t>대판 2019.12.19. 2016다24284</t>
         </is>
       </c>
       <c r="H1407" t="inlineStr">
@@ -56746,7 +56746,7 @@
     </row>
     <row r="1408">
       <c r="A1408" t="n">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="B1408" t="inlineStr">
         <is>
@@ -56755,7 +56755,7 @@
       </c>
       <c r="C1408" t="inlineStr">
         <is>
-          <t>양도금지특약이 있는 채권의 양수인이 양수금 지급을 청구하는 경우, 양수인이 그 특약을 알지 못하였고 알지 못한 데 중과실이 없다는 점을 스스로 주장·증명하여야 한다.</t>
+          <t>저당물의 제3취득자가 그 부동산에 지출한 필요비·유익비는 민법 제367조에 따라 경매대가에서 우선 상환받을 수 있으므로, 제3취득자는 그 비용상환청구권을 피담보채권으로 하여 경매의 매수인에게 유치권으로 대항할 수 있다.</t>
         </is>
       </c>
       <c r="D1408" t="inlineStr">
@@ -56765,28 +56765,28 @@
       </c>
       <c r="E1408" t="inlineStr">
         <is>
-          <t>문24·증명책임</t>
+          <t>문25·제367조유치권</t>
         </is>
       </c>
       <c r="F1408" t="inlineStr">
         <is>
-          <t>양도금지특약의 존재와 양수인의 악의·중과실은 이를 이유로 무효를 주장하는 채무자가 주장·증명하여야 한다.</t>
+          <t>제367조의 비용상환청구권은 경매대가에서 우선상환을 받을 수 있을 뿐이고, 이를 피담보채권으로 한 유치권으로 매수인에게 대항할 수는 없다.</t>
         </is>
       </c>
       <c r="G1408" t="inlineStr">
         <is>
-          <t>대판 2019.12.19. 2016다24284</t>
+          <t>대판 2023.7.13. 2022다265093</t>
         </is>
       </c>
       <c r="H1408" t="inlineStr">
         <is>
-          <t>제449조</t>
+          <t>제367조</t>
         </is>
       </c>
     </row>
     <row r="1409">
       <c r="A1409" t="n">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="B1409" t="inlineStr">
         <is>
@@ -56795,38 +56795,38 @@
       </c>
       <c r="C1409" t="inlineStr">
         <is>
-          <t>저당물의 제3취득자가 그 부동산에 지출한 필요비·유익비는 민법 제367조에 따라 경매대가에서 우선 상환받을 수 있으므로, 제3취득자는 그 비용상환청구권을 피담보채권으로 하여 경매의 매수인에게 유치권으로 대항할 수 있다.</t>
+          <t>유치권자가 피담보채권에 대한 별도의 시효중단 조치 없이 유치권확인의 소만을 제기하였더라도, 그 소송에서 피담보채권의 존재에 관한 주장에 대하여 실질적인 심리가 이루어졌다면 재판상 청구에 준하는 소멸시효 중단의 효력이 인정된다.</t>
         </is>
       </c>
       <c r="D1409" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E1409" t="inlineStr">
         <is>
-          <t>문25·제367조유치권</t>
+          <t>문25·유치권확인시효</t>
         </is>
       </c>
       <c r="F1409" t="inlineStr">
         <is>
-          <t>제367조의 비용상환청구권은 경매대가에서 우선상환을 받을 수 있을 뿐이고, 이를 피담보채권으로 한 유치권으로 매수인에게 대항할 수는 없다.</t>
+          <t>판례는 유치권 존재확인의 소에서 피담보채권에 관한 권리 실행의 의사가 표명되고 실질적으로 심리되면 재판상 청구에 준하여 그 피담보채권의 소멸시효 중단의 효력이 인정된다고 한다.</t>
         </is>
       </c>
       <c r="G1409" t="inlineStr">
         <is>
-          <t>대판 2023.7.13. 2022다265093</t>
+          <t>대판 2024.10.31. 2024다241152</t>
         </is>
       </c>
       <c r="H1409" t="inlineStr">
         <is>
-          <t>제367조</t>
+          <t>제168조</t>
         </is>
       </c>
     </row>
     <row r="1410">
       <c r="A1410" t="n">
-        <v>1555</v>
+        <v>1556</v>
       </c>
       <c r="B1410" t="inlineStr">
         <is>
@@ -56835,7 +56835,7 @@
       </c>
       <c r="C1410" t="inlineStr">
         <is>
-          <t>유치권자가 피담보채권에 대한 별도의 시효중단 조치 없이 유치권확인의 소만을 제기하였더라도, 그 소송에서 피담보채권의 존재에 관한 주장에 대하여 실질적인 심리가 이루어졌다면 재판상 청구에 준하는 소멸시효 중단의 효력이 인정된다.</t>
+          <t>착오송금을 이유로 부당이득반환을 청구하는 소송에서 송금에 착오가 있었는지에 대한 증명책임은 반환을 구하는 송금인에게 있다.</t>
         </is>
       </c>
       <c r="D1410" t="inlineStr">
@@ -56845,28 +56845,28 @@
       </c>
       <c r="E1410" t="inlineStr">
         <is>
-          <t>문25·유치권확인시효</t>
+          <t>문26·착오송금입증</t>
         </is>
       </c>
       <c r="F1410" t="inlineStr">
         <is>
-          <t>판례는 유치권확인소송에서 피담보채권에 관한 실질적 심리가 이루어지면 재판상 청구에 준하여 시효중단 효력을 인정한다.</t>
+          <t>부당이득반환을 구하는 자가 법률상 원인 없음(착오)을 증명하여야 한다.</t>
         </is>
       </c>
       <c r="G1410" t="inlineStr">
         <is>
-          <t>대판 2019.3.14. 2018다255648</t>
+          <t>민법 제741조 · 판례</t>
         </is>
       </c>
       <c r="H1410" t="inlineStr">
         <is>
-          <t>제168조</t>
+          <t>제741조</t>
         </is>
       </c>
     </row>
     <row r="1411">
       <c r="A1411" t="n">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="B1411" t="inlineStr">
         <is>
@@ -56875,7 +56875,7 @@
       </c>
       <c r="C1411" t="inlineStr">
         <is>
-          <t>착오송금을 이유로 부당이득반환을 청구하는 소송에서 송금에 착오가 있었는지에 대한 증명책임은 반환을 구하는 송금인에게 있다.</t>
+          <t>토지소유자가 불법점유자를 상대로 차임 상당 부당이득반환을 청구하는 소송에서 점유자가 '불법점유가 없었더라도 소유자에게 차임 상당 이익이 발생할 여지가 없었다'고 주장하는 경우, 그 특별한 사정에 대한 증명책임은 점유자가 진다.</t>
         </is>
       </c>
       <c r="D1411" t="inlineStr">
@@ -56885,17 +56885,17 @@
       </c>
       <c r="E1411" t="inlineStr">
         <is>
-          <t>문26·착오송금입증</t>
+          <t>문26·손실부존재입증</t>
         </is>
       </c>
       <c r="F1411" t="inlineStr">
         <is>
-          <t>부당이득반환을 구하는 자가 법률상 원인 없음(착오)을 증명하여야 한다.</t>
+          <t>판례는 손실이 없었다는 특별한 사정은 이를 주장하는 점유자(이득자)가 증명하여야 한다고 한다.</t>
         </is>
       </c>
       <c r="G1411" t="inlineStr">
         <is>
-          <t>민법 제741조 · 판례</t>
+          <t>대판 2008.1.17. 2006다586</t>
         </is>
       </c>
       <c r="H1411" t="inlineStr">
@@ -56906,7 +56906,7 @@
     </row>
     <row r="1412">
       <c r="A1412" t="n">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="B1412" t="inlineStr">
         <is>
@@ -56915,38 +56915,38 @@
       </c>
       <c r="C1412" t="inlineStr">
         <is>
-          <t>토지소유자가 불법점유자를 상대로 차임 상당 부당이득반환을 청구하는 소송에서 점유자가 '불법점유가 없었더라도 소유자에게 차임 상당 이익이 발생할 여지가 없었다'고 주장하는 경우, 그 특별한 사정에 대한 증명책임은 점유자가 진다.</t>
+          <t>기존 금전채무의 변제에 갈음하여 부동산 소유권을 이전하기로 하는 대물변제예약을 체결한 경우, 소유권이전등기를 완료하기 전에 기존 금전채무가 소멸하였더라도 당사자 사이에서는 예약된 대물변제 계약에 기하여 소유권이전등기를 청구할 수 있다.</t>
         </is>
       </c>
       <c r="D1412" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1412" t="inlineStr">
         <is>
-          <t>문26·손실부존재입증</t>
+          <t>문27·대물변제예약</t>
         </is>
       </c>
       <c r="F1412" t="inlineStr">
         <is>
-          <t>판례는 손실이 없었다는 특별한 사정은 이를 주장하는 점유자(이득자)가 증명하여야 한다고 한다.</t>
+          <t>대물변제예약은 기존 채무의 변제를 위한 것이므로 기존 채무가 소멸하면 대물변제할 이유가 없어 소유권이전등기를 청구할 수 없다.</t>
         </is>
       </c>
       <c r="G1412" t="inlineStr">
         <is>
-          <t>대판 2008.1.17. 2006다586</t>
+          <t>민법 제466조 · 판례</t>
         </is>
       </c>
       <c r="H1412" t="inlineStr">
         <is>
-          <t>제741조</t>
+          <t>제466조</t>
         </is>
       </c>
     </row>
     <row r="1413">
       <c r="A1413" t="n">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="B1413" t="inlineStr">
         <is>
@@ -56955,38 +56955,38 @@
       </c>
       <c r="C1413" t="inlineStr">
         <is>
-          <t>기존 금전채무의 변제에 갈음하여 부동산 소유권을 이전하기로 하는 대물변제예약을 체결한 경우, 소유권이전등기를 완료하기 전에 기존 금전채무가 소멸하였더라도 당사자 사이에서는 예약된 대물변제 계약에 기하여 소유권이전등기를 청구할 수 있다.</t>
+          <t>변제기 전 변제에 관한 약정이 없는 이자부 금전소비대차의 채무자가 변제기 전에 변제하는 경우, 변제기까지의 약정이자 등 채권자의 손해를 함께 제공하지 않으면 채권자는 그 수령을 거절할 수 있다.</t>
         </is>
       </c>
       <c r="D1413" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E1413" t="inlineStr">
         <is>
-          <t>문27·대물변제예약</t>
+          <t>문27·기한전변제</t>
         </is>
       </c>
       <c r="F1413" t="inlineStr">
         <is>
-          <t>대물변제예약은 기존 채무의 변제를 위한 것이므로 기존 채무가 소멸하면 대물변제할 이유가 없어 소유권이전등기를 청구할 수 없다.</t>
+          <t>판례는 이자부 소비대차에서 기한 전 변제 시 채권자의 기한이익(약정이자)을 배상하지 않으면 수령을 거절할 수 있다고 한다.</t>
         </is>
       </c>
       <c r="G1413" t="inlineStr">
         <is>
-          <t>민법 제466조 · 판례</t>
+          <t>민법 제468조 · 판례</t>
         </is>
       </c>
       <c r="H1413" t="inlineStr">
         <is>
-          <t>제466조</t>
+          <t>제468조</t>
         </is>
       </c>
     </row>
     <row r="1414">
       <c r="A1414" t="n">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="B1414" t="inlineStr">
         <is>
@@ -56995,7 +56995,7 @@
       </c>
       <c r="C1414" t="inlineStr">
         <is>
-          <t>변제기 전 변제에 관한 약정이 없는 이자부 금전소비대차의 채무자가 변제기 전에 변제하는 경우, 변제기까지의 약정이자 등 채권자의 손해를 함께 제공하지 않으면 채권자는 그 수령을 거절할 수 있다.</t>
+          <t>공작물책임에서 공작물이 본래 갖추어야 할 안전성은 그 용도에 한정된 안전성만이 아니라, 공작물이 현실적으로 설치되어 사용되고 있는 상황에서 요구되는 안전성을 의미한다.</t>
         </is>
       </c>
       <c r="D1414" t="inlineStr">
@@ -57005,28 +57005,28 @@
       </c>
       <c r="E1414" t="inlineStr">
         <is>
-          <t>문27·기한전변제</t>
+          <t>문28·공작물안전성</t>
         </is>
       </c>
       <c r="F1414" t="inlineStr">
         <is>
-          <t>판례는 이자부 소비대차에서 기한 전 변제 시 채권자의 기한이익(약정이자)을 배상하지 않으면 수령을 거절할 수 있다고 한다.</t>
+          <t>판례는 공작물의 안전성을 현실적 설치·사용 상황에서 요구되는 정도로 본다.</t>
         </is>
       </c>
       <c r="G1414" t="inlineStr">
         <is>
-          <t>민법 제468조 · 판례</t>
+          <t>대판 2018.7.12. 2015다68348 · 판례</t>
         </is>
       </c>
       <c r="H1414" t="inlineStr">
         <is>
-          <t>제468조</t>
+          <t>제758조</t>
         </is>
       </c>
     </row>
     <row r="1415">
       <c r="A1415" t="n">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="B1415" t="inlineStr">
         <is>
@@ -57035,27 +57035,27 @@
       </c>
       <c r="C1415" t="inlineStr">
         <is>
-          <t>공작물책임에서 공작물이 본래 갖추어야 할 안전성은 그 용도에 한정된 안전성만이 아니라, 공작물이 현실적으로 설치되어 사용되고 있는 상황에서 요구되는 안전성을 의미한다.</t>
+          <t>공작물책임에서 공작물의 점유자는 자신의 과실 유무와 관계없이 책임을 지고, 소유자는 자신의 과실이 있는 경우에만 책임을 진다.</t>
         </is>
       </c>
       <c r="D1415" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1415" t="inlineStr">
         <is>
-          <t>문28·공작물안전성</t>
+          <t>문28·점유자소유자책임</t>
         </is>
       </c>
       <c r="F1415" t="inlineStr">
         <is>
-          <t>판례는 공작물의 안전성을 현실적 설치·사용 상황에서 요구되는 정도로 본다.</t>
+          <t>점유자는 손해 방지에 필요한 주의를 다하였음을 증명하면 면책되는 중간책임을 지고, 소유자는 면책이 인정되지 않는 무과실책임을 진다.</t>
         </is>
       </c>
       <c r="G1415" t="inlineStr">
         <is>
-          <t>대판 2018.7.12. 2015다68348 · 판례</t>
+          <t>민법 제758조 제1항</t>
         </is>
       </c>
       <c r="H1415" t="inlineStr">
@@ -57066,7 +57066,7 @@
     </row>
     <row r="1416">
       <c r="A1416" t="n">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="B1416" t="inlineStr">
         <is>
@@ -57075,38 +57075,38 @@
       </c>
       <c r="C1416" t="inlineStr">
         <is>
-          <t>공작물책임에서 공작물의 점유자는 자신의 과실 유무와 관계없이 책임을 지고, 소유자는 자신의 과실이 있는 경우에만 책임을 진다.</t>
+          <t>부동산 매매에서 매수인이 선이행하여야 할 중도금을 지급하지 않은 채 잔대금 지급일을 경과한 경우, 특별한 사정이 없는 한 매수인의 중도금 및 그에 대한 지연손해금과 잔대금 지급의무는 매도인의 소유권이전등기의무와 동시이행관계에 있다.</t>
         </is>
       </c>
       <c r="D1416" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E1416" t="inlineStr">
         <is>
-          <t>문28·점유자소유자책임</t>
+          <t>문29·중도금동시이행</t>
         </is>
       </c>
       <c r="F1416" t="inlineStr">
         <is>
-          <t>점유자는 손해 방지에 필요한 주의를 다하였음을 증명하면 면책되는 중간책임을 지고, 소유자는 면책이 인정되지 않는 무과실책임을 진다.</t>
+          <t>판례는 중도금 미지급 후 잔대금일이 지나면 중도금·지연손해금·잔대금 지급의무와 이전등기의무가 동시이행관계에 있다고 한다.</t>
         </is>
       </c>
       <c r="G1416" t="inlineStr">
         <is>
-          <t>민법 제758조 제1항</t>
+          <t>대판 1991.3.27. 90다19930</t>
         </is>
       </c>
       <c r="H1416" t="inlineStr">
         <is>
-          <t>제758조</t>
+          <t>제536조</t>
         </is>
       </c>
     </row>
     <row r="1417">
       <c r="A1417" t="n">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="B1417" t="inlineStr">
         <is>
@@ -57115,7 +57115,7 @@
       </c>
       <c r="C1417" t="inlineStr">
         <is>
-          <t>부동산 매매에서 매수인이 선이행하여야 할 중도금을 지급하지 않은 채 잔대금 지급일을 경과한 경우, 특별한 사정이 없는 한 매수인의 중도금 및 그에 대한 지연손해금과 잔대금 지급의무는 매도인의 소유권이전등기의무와 동시이행관계에 있다.</t>
+          <t>동시이행관계에 있는 쌍방 채무 중 어느 한 채무가 이행불능이 되어 손해배상채무로 변한 경우, 그 손해배상채무도 다른 채무와 여전히 동시이행관계에 있다.</t>
         </is>
       </c>
       <c r="D1417" t="inlineStr">
@@ -57125,17 +57125,17 @@
       </c>
       <c r="E1417" t="inlineStr">
         <is>
-          <t>문29·중도금동시이행</t>
+          <t>문29·손배동시이행</t>
         </is>
       </c>
       <c r="F1417" t="inlineStr">
         <is>
-          <t>판례는 중도금 미지급 후 잔대금일이 지나면 중도금·지연손해금·잔대금 지급의무와 이전등기의무가 동시이행관계에 있다고 한다.</t>
+          <t>판례는 동시이행관계의 채무가 손해배상채무로 변경되어도 동일성이 유지되어 동시이행관계가 존속한다고 한다.</t>
         </is>
       </c>
       <c r="G1417" t="inlineStr">
         <is>
-          <t>대판 1991.3.27. 90다19930</t>
+          <t>대판 2000.2.25. 97다30066</t>
         </is>
       </c>
       <c r="H1417" t="inlineStr">
@@ -57146,7 +57146,7 @@
     </row>
     <row r="1418">
       <c r="A1418" t="n">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="B1418" t="inlineStr">
         <is>
@@ -57155,7 +57155,7 @@
       </c>
       <c r="C1418" t="inlineStr">
         <is>
-          <t>동시이행관계에 있는 쌍방 채무 중 어느 한 채무가 이행불능이 되어 손해배상채무로 변한 경우, 그 손해배상채무도 다른 채무와 여전히 동시이행관계에 있다.</t>
+          <t>매수인이 매매대금을 완납하였다면 목적물을 아직 인도받지 못하였더라도 그 이후 목적물에서 생기는 과실의 수취권은 매수인에게 귀속된다.</t>
         </is>
       </c>
       <c r="D1418" t="inlineStr">
@@ -57165,28 +57165,28 @@
       </c>
       <c r="E1418" t="inlineStr">
         <is>
-          <t>문29·손배동시이행</t>
+          <t>문30·과실수취권</t>
         </is>
       </c>
       <c r="F1418" t="inlineStr">
         <is>
-          <t>판례는 동시이행관계의 채무가 손해배상채무로 변경되어도 동일성이 유지되어 동시이행관계가 존속한다고 한다.</t>
+          <t>민법 제587조에 따라 매수인이 대금을 완납하면 그 후의 과실수취권은 매수인에게 귀속된다.</t>
         </is>
       </c>
       <c r="G1418" t="inlineStr">
         <is>
-          <t>대판 2000.2.25. 97다30066</t>
+          <t>민법 제587조</t>
         </is>
       </c>
       <c r="H1418" t="inlineStr">
         <is>
-          <t>제536조</t>
+          <t>제587조</t>
         </is>
       </c>
     </row>
     <row r="1419">
       <c r="A1419" t="n">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="B1419" t="inlineStr">
         <is>
@@ -57195,38 +57195,38 @@
       </c>
       <c r="C1419" t="inlineStr">
         <is>
-          <t>매수인이 매매대금을 완납하였다면 목적물을 아직 인도받지 못하였더라도 그 이후 목적물에서 생기는 과실의 수취권은 매수인에게 귀속된다.</t>
+          <t>매매목적물을 인도받지 못하고 매수인 자신도 대금을 지급하지 않은 경우, 매수인은 매도인에게 인도의무의 지체로 인한 손해배상금의 지급을 구할 수 있다.</t>
         </is>
       </c>
       <c r="D1419" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1419" t="inlineStr">
         <is>
-          <t>문30·과실수취권</t>
+          <t>문30·동시이행지체</t>
         </is>
       </c>
       <c r="F1419" t="inlineStr">
         <is>
-          <t>민법 제587조에 따라 매수인이 대금을 완납하면 그 후의 과실수취권은 매수인에게 귀속된다.</t>
+          <t>매수인이 대금을 지급하지 않은 이상 매도인의 인도의무는 동시이행 항변으로 지체에 빠지지 않으므로 지체로 인한 손해배상을 구할 수 없다.</t>
         </is>
       </c>
       <c r="G1419" t="inlineStr">
         <is>
-          <t>민법 제587조</t>
+          <t>민법 제536조 · 제587조</t>
         </is>
       </c>
       <c r="H1419" t="inlineStr">
         <is>
-          <t>제587조</t>
+          <t>제536조</t>
         </is>
       </c>
     </row>
     <row r="1420">
       <c r="A1420" t="n">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="B1420" t="inlineStr">
         <is>
@@ -57235,38 +57235,38 @@
       </c>
       <c r="C1420" t="inlineStr">
         <is>
-          <t>매매목적물을 인도받지 못하고 매수인 자신도 대금을 지급하지 않은 경우, 매수인은 매도인에게 인도의무의 지체로 인한 손해배상금의 지급을 구할 수 있다.</t>
+          <t>상가건물 임대차에서 임차인이 임대차기간 중 3기의 차임액에 이르도록 차임을 연체한 사실이 있다면, 계약갱신 요구 당시 연체액이 3기에 이르지 않게 되었더라도 임대인은 그 갱신 요구를 거절할 수 있다.</t>
         </is>
       </c>
       <c r="D1420" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E1420" t="inlineStr">
         <is>
-          <t>문30·동시이행지체</t>
+          <t>문31·3기연체갱신</t>
         </is>
       </c>
       <c r="F1420" t="inlineStr">
         <is>
-          <t>매수인이 대금을 지급하지 않은 이상 매도인의 인도의무는 동시이행 항변으로 지체에 빠지지 않으므로 지체로 인한 손해배상을 구할 수 없다.</t>
+          <t>판례는 과거에 3기 연체 사실이 있으면 갱신 요구 당시 연체가 해소되었어도 갱신거절 사유가 된다고 한다.</t>
         </is>
       </c>
       <c r="G1420" t="inlineStr">
         <is>
-          <t>민법 제536조 · 제587조</t>
+          <t>대판 2021.5.13. 2020다255429</t>
         </is>
       </c>
       <c r="H1420" t="inlineStr">
         <is>
-          <t>제536조</t>
+          <t>제640조</t>
         </is>
       </c>
     </row>
     <row r="1421">
       <c r="A1421" t="n">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="B1421" t="inlineStr">
         <is>
@@ -57275,7 +57275,7 @@
       </c>
       <c r="C1421" t="inlineStr">
         <is>
-          <t>상가건물 임대차에서 임차인이 임대차기간 중 3기의 차임액에 이르도록 차임을 연체한 사실이 있다면, 계약갱신 요구 당시 연체액이 3기에 이르지 않게 되었더라도 임대인은 그 갱신 요구를 거절할 수 있다.</t>
+          <t>임대차보증금이 수수된 임대차에서 차임채권에 압류 및 추심명령이 있었더라도, 임대차가 종료되어 목적물이 반환될 때까지 추심되지 않은 차임채권액은 임대차보증금에서 당연히 공제된다.</t>
         </is>
       </c>
       <c r="D1421" t="inlineStr">
@@ -57285,28 +57285,28 @@
       </c>
       <c r="E1421" t="inlineStr">
         <is>
-          <t>문31·3기연체갱신</t>
+          <t>문31·차임공제</t>
         </is>
       </c>
       <c r="F1421" t="inlineStr">
         <is>
-          <t>판례는 과거에 3기 연체 사실이 있으면 갱신 요구 당시 연체가 해소되었어도 갱신거절 사유가 된다고 한다.</t>
+          <t>판례는 차임채권에 압류·추심명령이 있어도 종료 시까지 미추심 차임은 보증금에서 당연 공제된다고 한다.</t>
         </is>
       </c>
       <c r="G1421" t="inlineStr">
         <is>
-          <t>대판 2021.5.13. 2020다255429</t>
+          <t>대판 2004.12.23. 2004다56554</t>
         </is>
       </c>
       <c r="H1421" t="inlineStr">
         <is>
-          <t>제640조</t>
+          <t>제618조</t>
         </is>
       </c>
     </row>
     <row r="1422">
       <c r="A1422" t="n">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="B1422" t="inlineStr">
         <is>
@@ -57315,38 +57315,38 @@
       </c>
       <c r="C1422" t="inlineStr">
         <is>
-          <t>임대차보증금이 수수된 임대차에서 차임채권에 압류 및 추심명령이 있었더라도, 임대차가 종료되어 목적물이 반환될 때까지 추심되지 않은 차임채권액은 임대차보증금에서 당연히 공제된다.</t>
+          <t>자필증서에 의한 유언에서 유언자가 주소를 자서하지 않았더라도 유언자의 특정에 지장이 없다면 그 유언은 유효하다.</t>
         </is>
       </c>
       <c r="D1422" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1422" t="inlineStr">
         <is>
-          <t>문31·차임공제</t>
+          <t>문32·자필증서주소</t>
         </is>
       </c>
       <c r="F1422" t="inlineStr">
         <is>
-          <t>판례는 차임채권에 압류·추심명령이 있어도 종료 시까지 미추심 차임은 보증금에서 당연 공제된다고 한다.</t>
+          <t>민법 제1066조는 자필증서 유언의 요건으로 주소의 자서를 요구하므로, 주소를 자서하지 않은 자필증서 유언은 무효이다.</t>
         </is>
       </c>
       <c r="G1422" t="inlineStr">
         <is>
-          <t>대판 2004.12.23. 2004다56554</t>
+          <t>민법 제1066조</t>
         </is>
       </c>
       <c r="H1422" t="inlineStr">
         <is>
-          <t>제618조</t>
+          <t>제1066조</t>
         </is>
       </c>
     </row>
     <row r="1423">
       <c r="A1423" t="n">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="B1423" t="inlineStr">
         <is>
@@ -57355,38 +57355,38 @@
       </c>
       <c r="C1423" t="inlineStr">
         <is>
-          <t>자필증서에 의한 유언에서 유언자가 주소를 자서하지 않았더라도 유언자의 특정에 지장이 없다면 그 유언은 유효하다.</t>
+          <t>유언증서가 성립한 후에 멸실되거나 분실되었더라도 유언자가 유언을 철회한 것으로 볼 수 없는 이상 그 사유만으로 유언이 실효되는 것은 아니고, 이해관계인은 유언증서의 내용을 증명하여 유언의 효력을 주장할 수 있다.</t>
         </is>
       </c>
       <c r="D1423" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E1423" t="inlineStr">
         <is>
-          <t>문32·자필증서주소</t>
+          <t>문32·유언증서멸실</t>
         </is>
       </c>
       <c r="F1423" t="inlineStr">
         <is>
-          <t>민법 제1066조는 자필증서 유언의 요건으로 주소의 자서를 요구하므로, 주소를 자서하지 않은 자필증서 유언은 무효이다.</t>
+          <t>판례는 유언증서의 멸실·분실만으로 유언이 실효되지 않고 내용을 증명하여 효력을 주장할 수 있다고 한다.</t>
         </is>
       </c>
       <c r="G1423" t="inlineStr">
         <is>
-          <t>민법 제1066조</t>
+          <t>대판 1996.9.20. 96다21119</t>
         </is>
       </c>
       <c r="H1423" t="inlineStr">
         <is>
-          <t>제1066조</t>
+          <t>제1060조</t>
         </is>
       </c>
     </row>
     <row r="1424">
       <c r="A1424" t="n">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="B1424" t="inlineStr">
         <is>
@@ -57395,38 +57395,38 @@
       </c>
       <c r="C1424" t="inlineStr">
         <is>
-          <t>유언증서가 성립한 후에 멸실되거나 분실되었더라도 유언자가 유언을 철회한 것으로 볼 수 없는 이상 그 사유만으로 유언이 실효되는 것은 아니고, 이해관계인은 유언증서의 내용을 증명하여 유언의 효력을 주장할 수 있다.</t>
+          <t>가정법원은 부 또는 모가 친권을 남용하여 자녀의 복리를 현저히 해치거나 해칠 우려가 있는 경우, 일정한 기간을 정하여 그 친권을 상실시킬 수 있다.</t>
         </is>
       </c>
       <c r="D1424" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1424" t="inlineStr">
         <is>
-          <t>문32·유언증서멸실</t>
+          <t>문33·친권상실기간</t>
         </is>
       </c>
       <c r="F1424" t="inlineStr">
         <is>
-          <t>판례는 유언증서의 멸실·분실만으로 유언이 실효되지 않고 내용을 증명하여 효력을 주장할 수 있다고 한다.</t>
+          <t>친권상실 선고에는 기간을 정하지 않으며, 기간을 정하여 제한하는 것은 친권의 일시 정지에 해당한다.</t>
         </is>
       </c>
       <c r="G1424" t="inlineStr">
         <is>
-          <t>대판 1996.9.20. 96다21119</t>
+          <t>민법 제924조</t>
         </is>
       </c>
       <c r="H1424" t="inlineStr">
         <is>
-          <t>제1060조</t>
+          <t>제924조</t>
         </is>
       </c>
     </row>
     <row r="1425">
       <c r="A1425" t="n">
-        <v>1570</v>
+        <v>1571</v>
       </c>
       <c r="B1425" t="inlineStr">
         <is>
@@ -57435,7 +57435,7 @@
       </c>
       <c r="C1425" t="inlineStr">
         <is>
-          <t>가정법원은 부 또는 모가 친권을 남용하여 자녀의 복리를 현저히 해치거나 해칠 우려가 있는 경우, 일정한 기간을 정하여 그 친권을 상실시킬 수 있다.</t>
+          <t>상속재산분할에 관하여 공동상속인 사이에 협의가 성립되지 않거나 협의할 수 없는 경우, 각 공동상속인은 상속재산에 속하는 개별 재산에 관하여 공유물분할청구의 소를 제기할 수 있다.</t>
         </is>
       </c>
       <c r="D1425" t="inlineStr">
@@ -57445,28 +57445,28 @@
       </c>
       <c r="E1425" t="inlineStr">
         <is>
-          <t>문33·친권상실기간</t>
+          <t>문34·상속공유물분할</t>
         </is>
       </c>
       <c r="F1425" t="inlineStr">
         <is>
-          <t>친권상실 선고에는 기간을 정하지 않으며, 기간을 정하여 제한하는 것은 친권의 일시 정지에 해당한다.</t>
+          <t>상속재산분할은 가사비송인 상속재산분할심판에 의하여야 하고, 개별 재산에 관한 공유물분할청구의 소로 할 수 없다.</t>
         </is>
       </c>
       <c r="G1425" t="inlineStr">
         <is>
-          <t>민법 제924조</t>
+          <t>대판 2015.8.13. 2015다18367</t>
         </is>
       </c>
       <c r="H1425" t="inlineStr">
         <is>
-          <t>제924조</t>
+          <t>제1013조</t>
         </is>
       </c>
     </row>
     <row r="1426">
       <c r="A1426" t="n">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="B1426" t="inlineStr">
         <is>
@@ -57475,38 +57475,38 @@
       </c>
       <c r="C1426" t="inlineStr">
         <is>
-          <t>상속재산분할에 관하여 공동상속인 사이에 협의가 성립되지 않거나 협의할 수 없는 경우, 각 공동상속인은 상속재산에 속하는 개별 재산에 관하여 공유물분할청구의 소를 제기할 수 있다.</t>
+          <t>협의분할로 공동상속인 중 일부가 자기 고유의 상속분을 초과하여 상속재산을 취득한 경우, 이는 상속개시 당시에 소급하여 피상속인으로부터 승계받은 것으로 보아야 하고 다른 공동상속인으로부터 증여받은 것으로 볼 수 없다.</t>
         </is>
       </c>
       <c r="D1426" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E1426" t="inlineStr">
         <is>
-          <t>문34·상속공유물분할</t>
+          <t>문34·협의분할소급</t>
         </is>
       </c>
       <c r="F1426" t="inlineStr">
         <is>
-          <t>상속재산분할은 가사비송인 상속재산분할심판에 의하여야 하고, 개별 재산에 관한 공유물분할청구의 소로 할 수 없다.</t>
+          <t>민법 제1015조에 따라 상속재산분할은 상속개시 시로 소급하여 효력이 있으므로 증여로 보지 않는다.</t>
         </is>
       </c>
       <c r="G1426" t="inlineStr">
         <is>
-          <t>대판 2015.8.13. 2015다18367</t>
+          <t>민법 제1015조</t>
         </is>
       </c>
       <c r="H1426" t="inlineStr">
         <is>
-          <t>제1013조</t>
+          <t>제1015조</t>
         </is>
       </c>
     </row>
     <row r="1427">
       <c r="A1427" t="n">
-        <v>1572</v>
+        <v>1573</v>
       </c>
       <c r="B1427" t="inlineStr">
         <is>
@@ -57515,7 +57515,7 @@
       </c>
       <c r="C1427" t="inlineStr">
         <is>
-          <t>협의분할로 공동상속인 중 일부가 자기 고유의 상속분을 초과하여 상속재산을 취득한 경우, 이는 상속개시 당시에 소급하여 피상속인으로부터 승계받은 것으로 보아야 하고 다른 공동상속인으로부터 증여받은 것으로 볼 수 없다.</t>
+          <t>이혼에 따른 재산분할에서 일방이 제3자와 합유하는 재산은 임의로 처분할 수 없어 직접 분할을 명할 수는 없으나, 그 지분의 가액을 산정하여 분할 대상으로 삼거나 다른 재산의 분할에 참작하는 방법으로 분할 대상에 포함하여야 한다.</t>
         </is>
       </c>
       <c r="D1427" t="inlineStr">
@@ -57525,28 +57525,28 @@
       </c>
       <c r="E1427" t="inlineStr">
         <is>
-          <t>문34·협의분할소급</t>
+          <t>문35·합유재산분할</t>
         </is>
       </c>
       <c r="F1427" t="inlineStr">
         <is>
-          <t>민법 제1015조에 따라 상속재산분할은 상속개시 시로 소급하여 효력이 있으므로 증여로 보지 않는다.</t>
+          <t>판례는 합유재산은 직접 분할을 명할 수 없으나 지분 가액을 산정하여 재산분할에 참작하여야 한다고 한다.</t>
         </is>
       </c>
       <c r="G1427" t="inlineStr">
         <is>
-          <t>민법 제1015조</t>
+          <t>대판 2009.11.12. 2009므2840</t>
         </is>
       </c>
       <c r="H1427" t="inlineStr">
         <is>
-          <t>제1015조</t>
+          <t>제839조의2</t>
         </is>
       </c>
     </row>
     <row r="1428">
       <c r="A1428" t="n">
-        <v>1573</v>
+        <v>1574</v>
       </c>
       <c r="B1428" t="inlineStr">
         <is>
@@ -57555,7 +57555,7 @@
       </c>
       <c r="C1428" t="inlineStr">
         <is>
-          <t>이혼에 따른 재산분할에서 일방이 제3자와 합유하는 재산은 임의로 처분할 수 없어 직접 분할을 명할 수는 없으나, 그 지분의 가액을 산정하여 분할 대상으로 삼거나 다른 재산의 분할에 참작하는 방법으로 분할 대상에 포함하여야 한다.</t>
+          <t>이혼에 따른 재산분할 사건에서 법원은 당사자가 특정한 분할 방법에 구애받지 않고 재산분할의 대상과 가액을 직권으로 조사·판단할 수 있다.</t>
         </is>
       </c>
       <c r="D1428" t="inlineStr">
@@ -57565,17 +57565,17 @@
       </c>
       <c r="E1428" t="inlineStr">
         <is>
-          <t>문35·합유재산분할</t>
+          <t>문35·직권조사</t>
         </is>
       </c>
       <c r="F1428" t="inlineStr">
         <is>
-          <t>판례는 합유재산은 직접 분할을 명할 수 없으나 지분 가액을 산정하여 재산분할에 참작하여야 한다고 한다.</t>
+          <t>재산분할은 가사비송사건으로 법원이 후견적 입장에서 직권으로 대상과 가액을 조사·판단한다.</t>
         </is>
       </c>
       <c r="G1428" t="inlineStr">
         <is>
-          <t>대판 2009.11.12. 2009므2840</t>
+          <t>대판 2022.1.27. 2018므11273 · 판례</t>
         </is>
       </c>
       <c r="H1428" t="inlineStr">
@@ -57586,7 +57586,7 @@
     </row>
     <row r="1429">
       <c r="A1429" t="n">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="B1429" t="inlineStr">
         <is>
@@ -57595,27 +57595,27 @@
       </c>
       <c r="C1429" t="inlineStr">
         <is>
-          <t>이혼에 따른 재산분할 사건에서 법원은 당사자가 특정한 분할 방법에 구애받지 않고 재산분할의 대상과 가액을 직권으로 조사·판단할 수 있다.</t>
+          <t>재산분할청구권은 이혼이 성립한 때 법적 효과로서 발생하므로, 협의나 심판에 의하여 그 구체적 내용이 형성되기 전이라도 이혼 성립 후에는 곧바로 채권양도의 대상이 된다.</t>
         </is>
       </c>
       <c r="D1429" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E1429" t="inlineStr">
         <is>
-          <t>문35·직권조사</t>
+          <t>문35·분할청구권양도</t>
         </is>
       </c>
       <c r="F1429" t="inlineStr">
         <is>
-          <t>재산분할은 가사비송사건으로 법원이 후견적 입장에서 직권으로 대상과 가액을 조사·판단한다.</t>
+          <t>협의나 심판으로 구체적 내용이 형성되기 전의 재산분할청구권은 범위와 내용이 불명확하여 양도의 대상이 될 수 없다.</t>
         </is>
       </c>
       <c r="G1429" t="inlineStr">
         <is>
-          <t>대판 2022.1.27. 2018므11273 · 판례</t>
+          <t>대판 1999.4.9. 98다58016</t>
         </is>
       </c>
       <c r="H1429" t="inlineStr">
@@ -57626,7 +57626,7 @@
     </row>
     <row r="1430">
       <c r="A1430" t="n">
-        <v>1575</v>
+        <v>1576</v>
       </c>
       <c r="B1430" t="inlineStr">
         <is>
@@ -57635,32 +57635,232 @@
       </c>
       <c r="C1430" t="inlineStr">
         <is>
-          <t>재산분할청구권은 이혼이 성립한 때 법적 효과로서 발생하므로, 협의나 심판에 의하여 그 구체적 내용이 형성되기 전이라도 이혼 성립 후에는 곧바로 채권양도의 대상이 된다.</t>
+          <t>손해배상 예정액이 부당히 과다한지 여부는 계약 당시가 아니라 사실심 변론종결 당시를 기준으로 판단하여야 한다.</t>
         </is>
       </c>
       <c r="D1430" t="inlineStr">
         <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1430" t="inlineStr">
+        <is>
+          <t>문21·감액기준시</t>
+        </is>
+      </c>
+      <c r="F1430" t="inlineStr">
+        <is>
+          <t>판례는 손해배상 예정액의 과다 여부를 사실심 변론종결 시를 기준으로 판단한다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1430" t="inlineStr">
+        <is>
+          <t>대판 2017.8.18. 2017다228762 · 판례</t>
+        </is>
+      </c>
+      <c r="H1430" t="inlineStr">
+        <is>
+          <t>제398조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="n">
+        <v>1577</v>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr">
+        <is>
+          <t>위약벌의 약정은 손해배상액의 예정과 그 내용이 다르므로, 민법 제398조 제2항을 유추적용하여 그 액을 감액할 수 없다.</t>
+        </is>
+      </c>
+      <c r="D1431" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1431" t="inlineStr">
+        <is>
+          <t>문21·위약벌감액</t>
+        </is>
+      </c>
+      <c r="F1431" t="inlineStr">
+        <is>
+          <t>판례는 위약벌은 손해배상액의 예정과 달라 제398조 제2항에 의한 직권 감액의 대상이 아니라고 한다(공서양속 위반 시 일부 무효만 가능).</t>
+        </is>
+      </c>
+      <c r="G1431" t="inlineStr">
+        <is>
+          <t>대판 2016.1.28. 2015다239324</t>
+        </is>
+      </c>
+      <c r="H1431" t="inlineStr">
+        <is>
+          <t>제398조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="n">
+        <v>1578</v>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr">
+        <is>
+          <t>손해배상액이 예정된 경우, 채무불이행으로 인한 손해의 발생·확대에 채권자의 과실이 있더라도 제398조 제2항에 따른 감액과는 별도로 과실상계를 적용하여 직권으로 감경하여야 한다.</t>
+        </is>
+      </c>
+      <c r="D1432" t="inlineStr">
+        <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E1430" t="inlineStr">
-        <is>
-          <t>문35·분할청구권양도</t>
-        </is>
-      </c>
-      <c r="F1430" t="inlineStr">
-        <is>
-          <t>협의나 심판으로 구체적 내용이 형성되기 전의 재산분할청구권은 범위와 내용이 불명확하여 양도의 대상이 될 수 없다.</t>
-        </is>
-      </c>
-      <c r="G1430" t="inlineStr">
-        <is>
-          <t>대판 1999.4.9. 98다58016</t>
-        </is>
-      </c>
-      <c r="H1430" t="inlineStr">
-        <is>
-          <t>제839조의2</t>
+      <c r="E1432" t="inlineStr">
+        <is>
+          <t>문21·예정액과실상계</t>
+        </is>
+      </c>
+      <c r="F1432" t="inlineStr">
+        <is>
+          <t>손해배상액이 예정된 경우에는 과실상계를 따로 적용할 수 없고, 예정액이 부당히 과다하면 제398조 제2항에 의한 직권 감액만 할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1432" t="inlineStr">
+        <is>
+          <t>대판 2016.6.10. 2014다200763</t>
+        </is>
+      </c>
+      <c r="H1432" t="inlineStr">
+        <is>
+          <t>제398조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="n">
+        <v>1579</v>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr">
+        <is>
+          <t>전세권이 존속하는 동안은 전세권을 존속시키기로 하면서 전세금반환채권만을 전세권과 분리하여 확정적으로 양도하는 것은 허용되지 않으며, 이는 임대차보증금반환채권을 담보하기 위하여 설정된 전세권에 관하여도 동일하게 적용된다.</t>
+        </is>
+      </c>
+      <c r="D1433" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1433" t="inlineStr">
+        <is>
+          <t>문22·전세금채권분리양도</t>
+        </is>
+      </c>
+      <c r="F1433" t="inlineStr">
+        <is>
+          <t>판례는 전세권 존속 중 전세금반환채권만의 확정적 분리양도를 허용하지 않으며 담보 목적 전세권에도 동일하게 본다.</t>
+        </is>
+      </c>
+      <c r="G1433" t="inlineStr">
+        <is>
+          <t>대판 2002.8.23. 2001다69122 · 판례</t>
+        </is>
+      </c>
+      <c r="H1433" t="inlineStr">
+        <is>
+          <t>제303조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="n">
+        <v>1580</v>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr">
+        <is>
+          <t>전세권설정자가 전세권 소멸 후 전세권자로부터 목적물을 인도받았더라도, 전세권설정등기의 말소에 필요한 서류를 교부받기 전까지는 전세금 반환을 거부하더라도 특별한 사정이 없는 한 전세금에 대한 이자 상당액을 부당이득으로 반환할 의무가 없다.</t>
+        </is>
+      </c>
+      <c r="D1434" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1434" t="inlineStr">
+        <is>
+          <t>문22·전세금동시이행</t>
+        </is>
+      </c>
+      <c r="F1434" t="inlineStr">
+        <is>
+          <t>전세금 반환의무와 전세권설정등기 말소서류 교부의무는 동시이행관계이므로, 목적물을 인도받았더라도 말소서류를 받기 전에는 이자 상당 부당이득 반환의무가 없다.</t>
+        </is>
+      </c>
+      <c r="G1434" t="inlineStr">
+        <is>
+          <t>대판 2002.2.5. 2001다62091</t>
+        </is>
+      </c>
+      <c r="H1434" t="inlineStr">
+        <is>
+          <t>제317조</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="n">
+        <v>1581</v>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>변시15</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr">
+        <is>
+          <t>전세권이 존속기간의 만료로 소멸한 경우, 전세금반환채권 양도계약 당사자 간의 특약에 따라 채권양수인은 담보물권이 없는 무담보의 전세금반환채권을 유효하게 취득할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D1435" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E1435" t="inlineStr">
+        <is>
+          <t>문22·무담보채권양수</t>
+        </is>
+      </c>
+      <c r="F1435" t="inlineStr">
+        <is>
+          <t>판례는 존속기간 만료로 전세권이 소멸한 경우 특약에 의하여 전세권과 분리된 무담보의 전세금반환채권을 양수할 수 있다고 한다.</t>
+        </is>
+      </c>
+      <c r="G1435" t="inlineStr">
+        <is>
+          <t>대판 1997.11.25. 97다29790 · 판례</t>
+        </is>
+      </c>
+      <c r="H1435" t="inlineStr">
+        <is>
+          <t>제303조</t>
         </is>
       </c>
     </row>

</xml_diff>